<commit_message>
Force numeric conversion inside custom constraint functions
</commit_message>
<xml_diff>
--- a/outputs/template.xlsx
+++ b/outputs/template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="282">
   <si>
     <t>Logic Attainement</t>
   </si>
@@ -511,13 +511,13 @@
     <t>SK12_6, SK12_13, SK12_15, SK12_18, SK12_22, SK12_27, SK12_41, SK12_43, SK12_45, SK12_46, SK12_49, SK12_65, SK12_68, SK12_77, SK12_78, SK12_84, SK12_102, SK12_108, SK12_116, SK12_119, SK12_120, SK12_122, SK12_131, SK12_146, SK12_148, SK12_155, SK12_161, SK12_201, SK12_205, SK12_206, SK12_210, SK12_213, SK12_217, SK12_226, SK12_237, SK12_239, SK12_245, SK12_265, SK12_298, SK12_306, SK12_315, SK12_321, SK12_323, SK12_333, SK12_335, SK12_353, SK12_371, SK12_378, SK12_381, SK12_431, SK17_6, SK17_13, SK17_15, SK17_18, SK17_22, SK17_27, SK17_41, SK17_43, SK17_45, SK17_46, SK17_49, SK17_65, SK17_68, SK17_77, SK17_78, SK17_84, SK17_102, SK17_108, SK17_116, SK17_119, SK17_120, SK17_122, SK17_131, SK17_146, SK17_148, SK17_155, SK17_161, SK17_201, SK17_205, SK17_206, SK17_210, SK17_213, SK17_217, SK17_226, SK17_237, SK17_239, SK17_245, SK17_265, SK17_298, SK17_306, SK17_315, SK17_321, SK17_323, SK17_333, SK17_335, SK17_353, SK17_371, SK17_378, SK17_381, SK17_431</t>
   </si>
   <si>
-    <t>234.51</t>
-  </si>
-  <si>
-    <t>12131</t>
-  </si>
-  <si>
-    <t>13, 15, 20, 28, 32, 33, 45, 48, 70, 76, 94, 104, 105, 117, 121, 131, 136, 139, 153, 155, 163, 164, 173, 175, 186, 188, 203, 205, 216, 232, 235, 236, 240, 248, 250, 252, 256, 260, 263, 272, 277, 285, 286, 289, 291, 304, 316, 326, 328, 330, 332, 336, 340, 351, 361, 371, 375, 380, 382, 384, 388, 399, 402, 405, 409, 419, 420, 425, 431, 436, 439, 440, 441, 445, 453, 458, 483, 485, 500, 512, 514, 530, 535, 541, 542, 558, 561, 577, 583, 584, 594, 597, 599, 605, 607, 618, 629, 636, 647, 649, 650, 656, 660, 668, 675, 676, 684, 686, 690, 701, 703, 712, 715, 721, 724, 725, 729, 732, 743, 754, 760, 762, 763, 774, 776, 784, 787, 788, 790, 804, 830, 839, 840, 841, 863, 866, 877, 881, 889, 905, 911, 919, 920, 941, 942, 954, 964, 965, 976, 977, 1004, 1007, 1011, 1016, 1030, 1031, 1050, 1053, 1054, 1056, 1066, 1080, 1082, 1083, 1087, 1096, 1105, 1110, 1112, 1116, 1119, 1145, 1154, 1159, 1164, 1165, 1170, 1180, 1186, 1191, 1194, 1197, 1207, 1220, 1222, 1223, 1235, 1240, 1246, 1248, 1249, 1262, 1263, 1264, 1267, 1269, 1276, 1288, 1298, 1301, 1302, 1315, 1326, 1332, 1351, 1354, 1368, 1371, 1389, 1397, 1401, 1413, 1417, 1420, 1431, 1439, 1443, 1446, 1447, 1455, 1459, 1461, 1463, 1464, 1467, 1472, 1491, 1494, 1495, 1496, 1499, 1522, 1534, 1552, 1569, 1581, 1583, 1588, 1595, 1613, 1625, 1628, 1630, 1634, 1636, 1643, 1647, 1654, 1657, 1675, 1677, 1680, 1697, 1705, 1708, 1716, 1717, 1719, 1726, 1737, 1747, 1748, 1759, 1767, 1770, 1772, 1781, 1783, 1787, 1798, 1807, 1808, 1810, 1814, 1815, 1822, 1832, 1838, 1839, 1844, 1848, 1852, 1854, 1859, 1868, 1877, 1878, 1883, 1884, 1888, 1889, 1891, 1892, 1896, 1903, 1904, 1905, 1906, 1911, 1912, 1915, 1916, 1918, 1919, 1922, 1928, 1933, 1938, 1943, 1955, 1968, 1980, 1981, 1986, 1993, 1995, 1996, 2003, 2007, 2008, 2026, 2027, 2029, 2030, 2032, 2048, 2050, 2063, 2068, 2070, 2073, 2079, 2097, 2106, 2107, 2112, 2116, 2121, 2124, 2125, 2126, 2131, 2133, 2137, 2139, 2163, 2165, 2166, 2168, 2175, 2178, 2181, 2185, 2187, 2191, 2192, 2223, 2229, 2241, 2256, 2261, 2262, 2265, 2266, 2269, 2273, 2276, 2279, 2282, 2284, 2291, 2292, 2297, 2298, 2313, 2315, 2316, 2319, 2320, 2322, 2323, 2324, 2328, 2332, 2334, 2337, 2338, 2340, 2341, 2347, 2354, 2355, 2356, 2368, 2372, 2374, 2375, 2376, 2383, 2385, 2397, 2404, 2406, 2411, 2412, 2416, 2433, 2463, 2471, 2476, 2478, 2483, 2485, 2499, 2500, 2502, 2503, 2504, 2505, 2507, 2545, 2551, 2552, 2556, 2560, 2562, 2567, 2568, 2572, 2589, 2593, 2597, 2601, 2615, 2617, 2624, 2627, 2642, 2659, 2660, 2672, 2678, 2683, 2686, 2690, 2693, 2696, 2701, 2706, 2710, 2748, 2753, 2771, 2772, 2780, 2801, 2804, 2813, 2814, 2815, 2819, 2821, 2825, 2828, 2833, 2837, 2843, 2847, 2857, 2863, 2868, 2874, 2878, 2882, 2888, 2902, 2911, 2917, 2931, 2935, 2948, 2953, 2955, 2956, 2964, 2979, 2983, 2985, 2986, 2987, 2988, 2993, 3025, 3032, 3040, 3043, 3051, 3054, 3071, 3072, 3079, 3085, 3095, 3102, 3105, 3109, 3113, 3121, 3126, 3127, 3130, 3135, 3136, 3155, 3167, 3172, 3174, 3175, 3177, 3178, 3181, 3185, 3194, 3195, 3197, 3200, 3208, 3216, 3219, 3220, 3223, 3228, 3232, 3233, 3236, 3246, 3249, 3253, 3263, 3280, 3293, 3302, 3307, 3314, 3326, 3332, 3333, 3335, 3346, 3350, 3352, 3353, 3359, 3360, 3366, 3367, 3371, 3377, 3378, 3382, 3399, 3404, 3410, 3414, 3416, 3425, 3428, 3435, 3438, 3442, 3452, 3458, 3461, 3463, 3465, 3487, 3502, 3519, 3521, 3530, 3540, 3542, 3561, 3569, 3582, 3586, 3590, 3595, 3597, 3603, 3608, 3618, 3621, 3622, 3629, 3632, 3633, 3641, 3649, 3659, 3661, 3663, 3665, 3666, 3677, 3679, 3686, 3687, 3689, 3694, 3701, 3710, 3720, 3721, 3725, 3728, 3733, 3734, 3743, 3760, 3769, 3783, 3785, 3786, 3801, 3803, 3819, 3827, 3829, 3834, 3851, 3858, 3859, 3860, 3864, 3867, 3876, 3877, 3885, 3894, 3895, 3909, 3912, 3914, 3915, 3917, 3921, 3925, 3927, 3933, 3936, 3945, 3952, 3955, 3980, 3987, 4003, 4018, 4021, 4024, 4026, 4038, 4051, 4057, 4058, 4064, 4066, 4067, 4076, 4084, 4088, 4092, 4096, 4114, 4117, 4120, 4123, 4139, 4142, 4145, 4151, 4152, 4159, 4162, 4169, 4180, 4184, 4185, 4186, 4193, 4198, 4209, 4216, 4219, 4237, 4243, 4250, 4251, 4263, 4265, 4272, 4273, 4282, 4289, 4329, 4331, 4333, 4338, 4339, 4345, 4346, 4347, 4352, 4354, 4355, 4356, 4373, 4388, 4389, 4393, 4396, 4408, 4410, 4415, 4430, 4433, 4436, 4439, 4449, 4451, 4455, 4458, 4468, 4491, 4501, 4505, 4514, 4515, 4527, 4534, 4538, 4540, 4542, 4544, 4555, 4558, 4560, 4564, 4565, 4569, 4573, 4579, 4583, 4593, 4597, 4602, 4613, 4618, 4624, 4626, 4628, 4632, 4633, 4636, 4637, 4638, 4645, 4656, 4667, 4672, 4679, 4681, 4682, 4693, 4699, 4721, 4729, 4732, 4734, 4736, 4758, 4759, 4765, 4778, 4779, 4780, 4782, 4785, 4787, 4792, 4797, 4799, 4803, 4828, 4832, 4841, 4856, 4884, 4892, 4925, 4936, 4947, 4953, 4956, 4957, 4964, 4965, 4971, 4974, 4979, 4980, 4989, 5007, 5008, 5014, 5018, 5020, 5033, 5037, 5042, 5055, 5063, 5075, 5076, 5079, 5081, 5084, 5085, 5087, 5089, 5097, 5102, 5107, 5111, 5113, 5115, 5126, 5129, 5149, 5150, 5158, 5160, 5163, 5167, 15, 26, 28, 38, 56, 62, 79, 104, 106, 121, 123, 125, 171, 174, 175, 260, 278, 320, 394, 432, 433, 487, 512, 536, 538, 543, 562, 581, 590, 605, 633, 644, 666, 688, 725, 735, 748, 763, 793, 804, 815, 866, 905, 913, 925, 926, 933, 987, 990, 1053, 1106, 1123, 1138, 1145, 1196, 1218, 1225, 1255, 1256, 1265, 1293, 1307, 1337, 1356, 1364, 1378, 1419, 1422, 1450, 1494, 1529, 1549, 1628, 1633, 1649, 1659, 1683, 1686, 1744, 1747, 1765, 1774, 1778, 1788, 1809, 1822, 1826, 1843, 1849, 1859, 1880, 1894, 1907, 1910, 1996, 2049, 2058, 2062, 2115, 2155, 2198, 2236, 2282, 2296, 2305, 2336, 2346, 2350, 2385, 2426, 2516, 2557, 2610, 2644, 2660, 2709, 2725, 2748, 2821, 2873, 2902, 2912, 2938, 2946, 2964, 2984, 2997, 3020, 3034, 3035, 3051, 3065, 3068, 3083, 3089, 3154, 3168, 3200, 3207, 3223, 3236, 3273, 3292, 3325, 3335, 3370, 3371, 3387, 3404, 3414, 3423, 3451, 3513, 3521, 3587, 3595, 3598, 3608, 3619, 3637, 3646, 3653, 3667, 3675, 3739, 3752, 3758, 3774, 3775, 3829, 3862, 3904, 3914, 3915, 3921, 3928, 3934, 3948, 3967, 3990, 4005, 4038, 4049, 4061, 4094, 4107, 4114, 4157, 4179, 4202, 4220, 4222, 4259, 4264, 4270, 4274, 4288, 4312, 4337, 4351, 4393, 4424, 4426, 4449, 4479, 4506, 4540, 4550, 4555, 4564, 4569, 4590, 4619, 4630, 4635, 4640, 4654, 4656, 4672, 4710, 4711, 4723, 4740, 4745, 4927, 4929, 4952, 4989, 5037, 5042, 5065, 5082, 5112, 5143, 5144, 5148, 1, 8, 13, 15, 24, 25, 31, 32, 37, 38, 43, 68, 75, 76, 79, 85, 86, 87, 94, 103, 111, 113, 126, 128, 130, 131, 133, 135, 139, 143, 145, 154, 155, 166, 171, 172, 173, 174, 178, 185, 188, 198, 203, 206, 212, 221, 250, 252, 256, 265, 271, 272, 277, 279, 285, 286, 296, 301, 311, 326, 327, 336, 337, 340, 349, 350, 352, 361, 365, 380, 386, 405, 406, 410, 424, 425, 432, 436, 439, 441, 445, 451, 454, 460, 469, 473, 476, 477, 480, 484, 485, 490, 504, 506, 512, 514, 515, 520, 521, 524, 526, 528, 539, 541, 542, 545, 547, 555, 558, 563, 566, 570, 574, 577, 581, 588, 594, 598, 604, 615, 623, 627, 629, 640, 660, 672, 675, 679, 681, 686, 700, 707, 717, 724, 728, 731, 732, 736, 741, 754, 759, 760, 767, 768, 771, 774, 776, 784, 787, 790, 796, 823, 826, 827, 829, 831, 837, 840, 841, 842, 844, 851, 856, 860, 862, 863, 868, 873, 877, 881, 885, 890, 897, 899, 900, 914, 915, 925, 930, 941, 950, 956, 960, 964, 965, 971, 974, 977, 979, 983, 987, 988, 998, 1003, 1004, 1039, 1044, 1045, 1054, 1062, 1081, 1082, 1087, 1090, 1111, 1112, 1116, 1135, 1138, 1142, 1148, 1156, 1164, 1168, 1172, 1182, 1185, 1186, 1207, 1208, 1214, 1215, 1219, 1223, 1224, 1230, 1239, 1241, 1243, 1246, 1248, 1252, 1255, 1256, 1259, 1262, 1263, 1276, 1301, 1312, 1320, 1324, 1337, 1342, 1351, 1353, 1363, 1366, 1367, 1375, 1386, 1388, 1389, 1394, 1397, 1401, 1403, 1410, 1413, 1417, 1426, 1428, 1439, 1444, 1446, 1447, 1449, 1455, 1459, 1463, 1464, 1475, 1483, 1493, 1494, 1495, 1498, 1499, 1504, 1510, 1519, 1520, 1528, 1534, 1540, 1541, 1544, 1552, 1558, 1569, 1572, 1574, 1581, 1583, 1596, 1601, 1603, 1608, 1618, 1623, 1625, 1630, 1636, 1639, 1644, 1646, 1649, 1655, 1656, 1660, 1665, 1666, 1670, 1675, 1676, 1677, 1680, 1681, 1682, 1683, 1693, 1698, 1708, 1711, 1717, 1722, 1727, 1730, 1737, 1742, 1749, 1752, 1757, 1759, 1762, 1767, 1772, 1776, 1779, 1782, 1787, 1792, 1797, 1805, 1806, 1808, 1816, 1844, 1849, 1854, 1857, 1864, 1867, 1868, 1871, 1873, 1877, 1884, 1889, 1890, 1892, 1896, 1904, 1906, 1912, 1917, 1921, 1922, 1924, 1930, 1934, 1937, 1944, 1954, 1958, 1962, 1975, 1976, 1980, 1981, 1990, 1993, 1996, 2008, 2012, 2013, 2016, 2023, 2030, 2037, 2038, 2040, 2043, 2051, 2054, 2056, 2066, 2067, 2074, 2079, 2083, 2090, 2103, 2104, 2105, 2106, 2107, 2112, 2113, 2114, 2115, 2124, 2126, 2133, 2141, 2145, 2148, 2156, 2163, 2167, 2170, 2171, 2185, 2192, 2198, 2204, 2218, 2227, 2234, 2241, 2243, 2246, 2266, 2271, 2273, 2276, 2280, 2284, 2288, 2292, 2298, 2301, 2303, 2308, 2316, 2320, 2322, 2323, 2332, 2334, 2335, 2338, 2341, 2346, 2347, 2348, 2352, 2365, 2368, 2372, 2376, 2385, 2391, 2417, 2419, 2435, 2436, 2439, 2447, 2450, 2452, 2454, 2456, 2458, 2468, 2469, 2471, 2477, 2478, 2482, 2485, 2486, 2488, 2491, 2492, 2494, 2495, 2499, 2515, 2521, 2522, 2531, 2535, 2545, 2550, 2553, 2554, 2559, 2560, 2562, 2563, 2567, 2568, 2570, 2588, 2604, 2608, 2609, 2610, 2613, 2617, 2624, 2625, 2627, 2630, 2633, 2634, 2636, 2641, 2648, 2650, 2654, 2658, 2659, 2660, 2662, 2665, 2674, 2678, 2679, 2683, 2685, 2686, 2687, 2689, 2696, 2701, 2706, 2709, 2711, 2722, 2723, 2724, 2734, 2739, 2744, 2745, 2747, 2749, 2753, 2764, 2766, 2768, 2772, 2775, 2777, 2780, 2781, 2785, 2787, 2795, 2815, 2818, 2819, 2820, 2829, 2837, 2846, 2848, 2850, 2856, 2863, 2865, 2866, 2875, 2878, 2881, 2905, 2911, 2913, 2921, 2935, 2936, 2940, 2948, 2973, 2975, 2978, 2983, 2985, 2998, 2999, 3008, 3010, 3026, 3030, 3035, 3038, 3044, 3045, 3057, 3069, 3071, 3076, 3079, 3090, 3092, 3097, 3098, 3102, 3108, 3109, 3110, 3113, 3119, 3127, 3130, 3131, 3134, 3136, 3138, 3155, 3161, 3168, 3174, 3180, 3181, 3182, 3187, 3197, 3198, 3200, 3208, 3213, 3219, 3222, 3235, 3236, 3246, 3251, 3261, 3263, 3264, 3265, 3279, 3280, 3286, 3302, 3305, 3308, 3309, 3314, 3321, 3326, 3329, 3332, 3333, 3340, 3343, 3350, 3353, 3356, 3371, 3381, 3391, 3399, 3403, 3414, 3423, 3424, 3425, 3431, 3432, 3435, 3438, 3442, 3449, 3453, 3456, 3465, 3466, 3471, 3474, 3476, 3482, 3483, 3484, 3497, 3506, 3508, 3521, 3541, 3551, 3567, 3569, 3575, 3577, 3582, 3585, 3587, 3595, 3596, 3597, 3601, 3605, 3608, 3618, 3619, 3626, 3628, 3631, 3632, 3648, 3649, 3656, 3657, 3660, 3666, 3673, 3677, 3682, 3685, 3686, 3687, 3693, 3708, 3710, 3718, 3720, 3722, 3724, 3732, 3758, 3759, 3764, 3771, 3777, 3790, 3815, 3827, 3834, 3838, 3840, 3851, 3852, 3853, 3859, 3865, 3880, 3884, 3887, 3889, 3892, 3894, 3895, 3896, 3899, 3904, 3907, 3912, 3915, 3917, 3925, 3926, 3932, 3937, 3949, 3953, 3958, 3962, 3970, 3971, 3972, 3975, 3980, 3984, 3985, 3987, 3988, 3990, 3998, 4011, 4012, 4018, 4022, 4026, 4030, 4037, 4051, 4055, 4056, 4061, 4064, 4066, 4073, 4077, 4082, 4084, 4096, 4097, 4098, 4105, 4113, 4114, 4116, 4119, 4120, 4122, 4123, 4124, 4136, 4138, 4139, 4140, 4162, 4163, 4166, 4171, 4173, 4179, 4180, 4185, 4192, 4199, 4209, 4216, 4223, 4238, 4246, 4259, 4262, 4270, 4277, 4289, 4290, 4297, 4301, 4306, 4310, 4316, 4321, 4329, 4331, 4337, 4338, 4339, 4343, 4345, 4348, 4351, 4354, 4356, 4357, 4360, 4378, 4393, 4395, 4396, 4401, 4409, 4412, 4428, 4429, 4433, 4438, 4442, 4446, 4468, 4475, 4484, 4488, 4501, 4502, 4504, 4505, 4507, 4508, 4515, 4520, 4525, 4526, 4532, 4540, 4541, 4542, 4544, 4546, 4552, 4561, 4564, 4573, 4577, 4582, 4602, 4612, 4616, 4624, 4626, 4627, 4628, 4629, 4632, 4638, 4649, 4652, 4667, 4679, 4688, 4691, 4692, 4712, 4728, 4731, 4734, 4744, 4759, 4763, 4770, 4778, 4782, 4783, 4785, 4787, 4790, 4792, 4796, 4797, 4798, 4805, 4812, 4815, 4816, 4839, 4841, 4847, 4850, 4861, 4862, 4864, 4866, 4868, 4872, 4874, 4880, 4883, 4892, 4913, 4919, 4922, 4927, 4928, 4929, 4942, 4951, 4954, 4957, 4962, 4964, 4966, 4981, 4984, 4986, 4988, 5018, 5020, 5030, 5031, 5033, 5036, 5037, 5041, 5044, 5047, 5060, 5062, 5063, 5072, 5075, 5077, 5084, 5113, 5118, 5121, 5133, 5144, 5155, 5160, 5161, 5169, 5172, 15, 18, 26, 37, 48, 57, 80, 86, 92, 102, 104, 116, 131, 135, 139, 146, 148, 154, 157, 173, 188, 216, 218, 231, 237, 252, 265, 269, 295, 333, 335, 340, 358, 365, 368, 374, 375, 380, 385, 387, 406, 413, 425, 436, 441, 444, 445, 455, 461, 468, 477, 480, 482, 491, 498, 511, 527, 547, 583, 588, 591, 603, 612, 618, 627, 629, 636, 657, 661, 662, 669, 682, 695, 717, 748, 754, 762, 764, 776, 795, 825, 846, 848, 856, 857, 862, 863, 865, 866, 874, 884, 901, 913, 915, 1008, 1020, 1025, 1033, 1049, 1054, 1068, 1093, 1100, 1124, 1133, 1146, 1168, 1185, 1186, 1190, 1191, 1194, 1196, 1204, 1207, 1208, 1221, 1233, 1248, 1249, 1278, 1300, 1312, 1315, 1346, 1350, 1371, 1374, 1377, 1412, 1443, 1464, 1466, 1513, 1535, 1544, 1574, 1584, 1602, 1625, 1628, 1631, 1640, 1653, 1692, 1696, 1697, 1699, 1702, 1718, 1738, 1746, 1753, 1757, 1813, 1838, 1851, 1864, 1865, 1881, 1885, 1890, 1897, 1900, 1902, 1904, 1909, 1917, 1918, 1939, 1944, 1958, 1971, 1978, 1984, 1986, 2000, 2011, 2016, 2018, 2068, 2083, 2087, 2116, 2133, 2144, 2162, 2165, 2171, 2172, 2176, 2185, 2195, 2207, 2221, 2223, 2256, 2260, 2268, 2271, 2302, 2303, 2313, 2331, 2359, 2362, 2366, 2384, 2435, 2445, 2447, 2449, 2458, 2483, 2499, 2508, 2525, 2531, 2558, 2560, 2583, 2586, 2587, 2614, 2624, 2634, 2636, 2654, 2662, 2684, 2696, 2701, 2707, 2719, 2727, 2745, 2749, 2772, 2787, 2789, 2795, 2804, 2812, 2818, 2820, 2839, 2840, 2852, 2855, 2856, 2857, 2863, 2866, 2876, 2921, 2947, 2961, 2974, 2975, 2980, 2993, 3012, 3016, 3026, 3050, 3061, 3062, 3078, 3081, 3083, 3117, 3121, 3129, 3134, 3158, 3183, 3187, 3192, 3200, 3216, 3221, 3232, 3241, 3245, 3246, 3264, 3294, 3301, 3313, 3322, 3327, 3336, 3355, 3356, 3360, 3364, 3378, 3379, 3399, 3404, 3405, 3409, 3426, 3449, 3458, 3468, 3484, 3496, 3503, 3506, 3508, 3511, 3520, 3521, 3525, 3534, 3554, 3572, 3580, 3582, 3598, 3617, 3633, 3679, 3748, 3752, 3769, 3789, 3796, 3809, 3832, 3833, 3844, 3865, 3868, 3875, 3884, 3893, 3905, 3926, 3929, 3936, 3952, 3959, 3974, 3987, 3991, 4003, 4008, 4023, 4064, 4075, 4076, 4082, 4095, 4097, 4102, 4108, 4110, 4122, 4131, 4139, 4143, 4155, 4162, 4169, 4172, 4173, 4234, 4238, 4241, 4262, 4265, 4274, 4296, 4301, 4309, 4311, 4323, 4362, 4389, 4393, 4394, 4400, 4406, 4461, 4485, 4492, 4501, 4502, 4505, 4526, 4542, 4547, 4552, 4560, 4580, 4594, 4599, 4607, 4611, 4616, 4624, 4642, 4648, 4660, 4685, 4697, 4712, 4723, 4773, 4774, 4775, 4784, 4787, 4812, 4822, 4841, 4869, 4872, 4925, 4935, 4948, 4964, 4970, 4977, 4983, 4988, 5005, 5006, 5018, 5034, 5045, 5051, 5075, 5079, 5085, 5088, 5090, 5115, 5122, 5126, 5164, 5169, 5170, 111, 187, 281, 294, 300, 349, 384, 515, 584, 608, 851, 899, 1010, 1152, 1153, 1552, 1897, 2245, 2250, 2359, 2721, 2786, 2935, 3127, 3136, 3164, 3201, 3208, 3232, 3293, 3302, 3418, 3441, 3612, 4048, 4061, 4065, 4066, 4096, 4245, 4252, 4486, 4526, 4672, 4956, 5020, 5126, 5136, 29, 49, 66, 93, 98, 120, 124, 184, 187, 205, 220, 238, 245, 257, 263, 287, 345, 349, 360, 442, 457, 564, 584, 627, 657, 672, 775, 799, 818, 852, 898, 979, 1008, 1011, 1024, 1041, 1057, 1061, 1126, 1140, 1153, 1159, 1194, 1196, 1200, 1228, 1263, 1277, 1296, 1375, 1397, 1404, 1457, 1483, 1495, 1528, 1531, 1533, 1570, 1584, 1592, 1666, 1689, 1699, 1747, 1762, 1857, 1868, 1887, 1905, 1926, 1936, 1951, 1954, 1956, 1962, 1972, 1973, 2032, 2054, 2101, 2127, 2140, 2145, 2148, 2155, 2192, 2237, 2265, 2315, 2346, 2350, 2367, 2454, 2468, 2477, 2568, 2601, 2699, 2768, 2825, 2828, 2835, 2839, 2862, 2880, 2881, 2930, 3044, 3082, 3123, 3127, 3164, 3165, 3178, 3305, 3333, 3345, 3361, 3404, 3418, 3452, 3544, 3584, 3605, 3610, 3663, 3666, 3672, 3703, 3723, 3728, 3785, 3837, 3862, 3863, 3929, 3949, 3964, 4034, 4127, 4144, 4154, 4186, 4200, 4243, 4252, 4339, 4348, 4387, 4424, 4429, 4446, 4473, 4486, 4535, 4577, 4588, 4637, 4640, 4647, 4661, 4672, 4690, 4728, 4734, 4796, 4804, 4816, 4825, 4890, 4901, 4918, 4924, 4948, 4959, 5037, 5046, 5094, 5117, 5124, 5157, 38, 41, 56, 84, 89, 99, 112, 133, 136, 141, 152, 228, 257, 281, 294, 295, 321, 346, 347, 363, 424, 433, 468, 541, 544, 548, 582, 611, 631, 657, 711, 721, 760, 826, 848, 906, 988, 1028, 1034, 1052, 1061, 1071, 1107, 1113, 1131, 1138, 1145, 1150, 1153, 1186, 1188, 1191, 1210, 1250, 1281, 1292, 1300, 1324, 1353, 1384, 1393, 1414, 1417, 1438, 1443, 1482, 1510, 1530, 1589, 1632, 1652, 1707, 1747, 1749, 1774, 1782, 1810, 1835, 1861, 1877, 1903, 1912, 1928, 1940, 1954, 1975, 1991, 2044, 2094, 2118, 2147, 2166, 2226, 2231, 2261, 2266, 2303, 2342, 2364, 2369, 2390, 2429, 2436, 2437, 2449, 2483, 2539, 2556, 2560, 2608, 2614, 2634, 2651, 2652, 2685, 2699, 2715, 2722, 2742, 2759, 2764, 2771, 2784, 2816, 2838, 2840, 2889, 2916, 2919, 2938, 2941, 2944, 2957, 2960, 2972, 3025, 3057, 3077, 3089, 3124, 3126, 3159, 3161, 3167, 3175, 3183, 3248, 3327, 3341, 3345, 3390, 3396, 3409, 3431, 3451, 3452, 3456, 3515, 3517, 3551, 3559, 3561, 3569, 3610, 3617, 3627, 3669, 3685, 3693, 3694, 3698, 3739, 3741, 3827, 3859, 3863, 3873, 3874, 3919, 4003, 4083, 4118, 4128, 4150, 4177, 4220, 4316, 4343, 4410, 4412, 4426, 4446, 4483, 4486, 4492, 4500, 4520, 4527, 4535, 4569, 4579, 4589, 4602, 4616, 4645, 4667, 4689, 4690, 4697, 4717, 4732, 4734, 4790, 4803, 4849, 4853, 4872, 4873, 4878, 4887, 4890, 4919, 4964, 4992, 5018, 5027, 5031, 5035, 5047, 5051, 5059, 5163, 101, 125, 146, 225, 258, 419, 447, 528, 533, 582, 583, 712, 799, 919, 927, 940, 1066, 1201, 1223, 1531, 1569, 1586, 1692, 1875, 1919, 1976, 2002, 2032, 2092, 2133, 2191, 2193, 2244, 2325, 2342, 2440, 2518, 2533, 2549, 2613, 2652, 2668, 2692, 2702, 2704, 2828, 2873, 2887, 2999, 3017, 3044, 3062, 3231, 3302, 3388, 3452, 3821, 3877, 3901, 3910, 3964, 3965, 4004, 4049, 4112, 4175, 4283, 4384, 4586, 4709, 4810, 4817, 4888, 4997, 5016, 5098, 101, 121, 455, 538, 1073, 1183, 1555, 1659, 2078, 2121, 2402, 2539, 2582, 2620, 3079, 3095, 3167, 3390, 3452, 3529, 3541, 3597, 3919, 3935, 4085, 4135, 4378, 4624, 4677, 4887, 4908, 810, 1889, 1954, 2005, 1, 59, 70, 249, 350, 448, 537, 643, 666, 718, 761, 775, 798, 866, 873, 927, 963, 1028, 1069, 1200, 1231, 1307, 1358, 1360, 1618, 1651, 1664, 1711, 1722, 1749, 1766, 1780, 1795, 1827, 1831, 1895, 1904, 1914, 1973, 2077, 2083, 2211, 2254, 2272, 2337, 2348, 2391, 2422, 2433, 2515, 2545, 2569, 2627, 2664, 2677, 2679, 2693, 2873, 2886, 2916, 3059, 3062, 3081, 3212, 3236, 3246, 3395, 3405, 3450, 3490, 3725, 3808, 3921, 3962, 3996, 4015, 4037, 4106, 4143, 4274, 4327, 4404, 4484, 4619, 4678, 4712, 4736, 4814, 4881, 4900, 4940, 5013, 5091, 5108, 5111, 5126, 25, 101, 144, 171, 180, 186, 189, 206, 228, 276, 280, 281, 300, 327, 329, 380, 560, 582, 600, 606, 699, 763, 764, 777, 792, 815, 885, 898, 983, 997, 1041, 1189, 1231, 1256, 1274, 1280, 1305, 1362, 1393, 1415, 1438, 1458, 1475, 1493, 1495, 1621, 1680, 1698, 1733, 1774, 1775, 1802, 1812, 1827, 1835, 1861, 1883, 1954, 2111, 2127, 2150, 2158, 2162, 2166, 2234, 2343, 2364, 2422, 2439, 2474, 2504, 2513, 2539, 2587, 2662, 2664, 2693, 2771, 2777, 2782, 2785, 2806, 2816, 2835, 2860, 2953, 3006, 3015, 3020, 3135, 3159, 3249, 3280, 3302, 3315, 3345, 3355, 3420, 3448, 3531, 3551, 3610, 3625, 3638, 3640, 3663, 3689, 3694, 3724, 3728, 3744, 3837, 3877, 3891, 3900, 3934, 3944, 3966, 4034, 4048, 4093, 4149, 4164, 4169, 4333, 4378, 4392, 4429, 4442, 4451, 4579, 4602, 4607, 4624, 4717, 4742, 4749, 4763, 4786, 4798, 4830, 4872, 4906, 5001, 5013, 5023, 5126, 5156, 5159, 13, 71, 93, 94, 304, 312, 373, 413, 422, 534, 544, 595, 642, 681, 693, 721, 806, 809, 841, 1148, 1208, 1232, 1241, 1361, 1476, 1586, 1616, 1642, 1654, 1695, 1777, 1854, 1917, 1967, 1969, 1971, 1976, 1997, 2256, 2275, 2345, 2381, 2492, 2561, 2563, 2594, 2618, 2625, 2683, 2702, 2768, 2792, 2860, 2865, 2889, 3039, 3104, 3185, 3193, 3215, 3245, 3266, 3274, 3294, 3303, 3322, 3326, 3333, 3339, 3352, 3474, 3520, 3539, 3648, 3663, 3672, 3673, 3754, 3904, 3953, 3963, 4023, 4035, 4131, 4165, 4195, 4209, 4332, 4338, 4409, 4467, 4585, 4684, 4761, 4783, 4832, 4856, 4970, 4995, 5063, 5140, 58, 109, 121, 125, 146, 172, 182, 210, 258, 311, 319, 325, 375, 381, 409, 419, 422, 447, 455, 462, 485, 563, 583, 693, 810, 927, 940, 954, 1061, 1066, 1073, 1093, 1291, 1338, 1435, 1467, 1535, 1555, 1569, 1600, 1614, 1666, 1898, 1917, 1919, 1923, 1954, 2002, 2007, 2028, 2053, 2058, 2089, 2092, 2099, 2121, 2133, 2221, 2270, 2289, 2291, 2325, 2374, 2421, 2440, 2533, 2613, 2614, 2619, 2668, 2699, 2731, 2828, 2838, 2846, 2886, 2896, 2967, 3095, 3105, 3124, 3185, 3194, 3197, 3198, 3228, 3260, 3380, 3388, 3404, 3451, 3460, 3521, 3529, 3642, 3651, 3684, 3740, 3801, 3823, 3935, 3952, 3970, 3990, 4077, 4135, 4304, 4333, 4369, 4400, 4540, 4586, 4627, 4711, 4721, 4778, 4810, 4817, 4879, 4888, 5005, 349, 422, 627, 661, 927, 932, 952, 1124, 1311, 1351, 1366, 1440, 1512, 1532, 1702, 1886, 1895, 1923, 1997, 2072, 2133, 2404, 2450, 2531, 2990, 3006, 3030, 3197, 3354, 3448, 3838, 3948, 4213, 4585, 84, 116, 205, 2634, 10, 18, 37, 41, 45, 48, 49, 75, 84, 85, 105, 109, 111, 131, 140, 146, 161, 167, 172, 173, 175, 176, 179, 180, 184, 207, 211, 215, 220, 269, 279, 290, 292, 299, 311, 312, 314, 315, 320, 329, 340, 354, 358, 368, 369, 370, 372, 384, 385, 396, 400, 419, 422, 425, 433, 434, 435, 438, 440, 458, 476, 479, 514, 517, 537, 555, 563, 583, 589, 627, 631, 642, 660, 665, 669, 671, 672, 673, 686, 699, 700, 714, 716, 718, 720, 724, 737, 761, 766, 809, 831, 833, 841, 844, 846, 850, 852, 873, 874, 903, 905, 906, 918, 929, 937, 941, 955, 963, 988, 997, 1008, 1017, 1029, 1034, 1057, 1060, 1061, 1064, 1070, 1079, 1117, 1119, 1123, 1133, 1142, 1162, 1163, 1177, 1189, 1190, 1191, 1215, 1225, 1229, 1263, 1281, 1307, 1315, 1346, 1352, 1353, 1355, 1374, 1383, 1395, 1435, 1436, 1443, 1445, 1453, 1455, 1458, 1474, 1480, 1492, 1500, 1525, 1535, 1542, 1549, 1555, 1568, 1578, 1579, 1605, 1608, 1627, 1634, 1636, 1637, 1642, 1653, 1658, 1663, 1677, 1721, 1725, 1741, 1744, 1753, 1761, 1764, 1778, 1787, 1801, 1809, 1814, 1816, 1826, 1831, 1850, 1852, 1863, 1868, 1878, 1886, 1940, 1954, 1969, 1972, 1996, 2005, 2011, 2019, 2023, 2050, 2086, 2088, 2090, 2104, 2116, 2121, 2133, 2151, 2175, 2176, 2180, 2206, 2218, 2222, 2230, 2241, 2268, 2273, 2275, 2279, 2291, 2292, 2297, 2309, 2315, 2324, 2326, 2348, 2351, 2356, 2358, 2366, 2373, 2406, 2413, 2415, 2417, 2418, 2421, 2445, 2449, 2461, 2470, 2483, 2485, 2491, 2492, 2518, 2538, 2540, 2547, 2551, 2553, 2557, 2576, 2596, 2641, 2675, 2680, 2688, 2696, 2703, 2706, 2711, 2733, 2741, 2745, 2747, 2757, 2784, 2785, 2787, 2793, 2806, 2822, 2831, 2833, 2837, 2839, 2845, 2896, 2897, 2903, 2907, 2910, 2911, 2916, 2930, 2932, 2936, 2937, 2942, 2953, 2960, 2973, 2975, 2980, 2985, 2987, 2998, 3010, 3021, 3023, 3029, 3043, 3051, 3061, 3069, 3095, 3124, 3126, 3127, 3150, 3176, 3180, 3184, 3186, 3193, 3202, 3210, 3223, 3232, 3263, 3273, 3274, 3276, 3298, 3317, 3322, 3331, 3343, 3374, 3382, 3388, 3400, 3414, 3425, 3448, 3453, 3460, 3466, 3468, 3469, 3471, 3479, 3484, 3488, 3507, 3517, 3521, 3529, 3533, 3538, 3569, 3571, 3588, 3602, 3605, 3611, 3617, 3633, 3645, 3663, 3667, 3669, 3683, 3693, 3698, 3708, 3715, 3717, 3730, 3732, 3737, 3738, 3740, 3766, 3790, 3793, 3805, 3828, 3837, 3841, 3845, 3849, 3852, 3862, 3870, 3890, 3914, 3922, 3935, 3947, 3952, 3953, 3965, 3969, 3981, 3985, 3996, 4000, 4028, 4029, 4032, 4034, 4037, 4056, 4069, 4070, 4071, 4081, 4084, 4088, 4096, 4119, 4120, 4129, 4140, 4149, 4157, 4162, 4168, 4169, 4184, 4202, 4209, 4246, 4253, 4262, 4263, 4276, 4279, 4293, 4301, 4310, 4312, 4317, 4320, 4323, 4331, 4338, 4340, 4356, 4360, 4372, 4375, 4393, 4405, 4412, 4421, 4423, 4424, 4426, 4434, 4441, 4446, 4452, 4485, 4486, 4507, 4572, 4589, 4619, 4626, 4636, 4644, 4645, 4651, 4671, 4681, 4693, 4717, 4731, 4732, 4735, 4745, 4750, 4751, 4752, 4755, 4756, 4759, 4775, 4778, 4787, 4790, 4800, 4801, 4802, 4803, 4811, 4828, 4851, 4853, 4881, 4897, 4900, 4908, 4919, 4924, 4926, 4937, 4938, 4942, 4944, 4950, 4955, 4957, 4964, 4970, 4976, 4977, 4986, 4989, 5005, 5030, 5040, 5045, 5060, 5071, 5089, 5090, 5097, 5104, 5115, 5118, 5131, 5147, 5150, 5162, 5164, 5165, 5172, 7, 24, 30, 43, 45, 49, 65, 77, 90, 93, 98, 100, 118, 123, 134, 143, 147, 149, 151, 162, 163, 172, 173, 179, 180, 191, 202, 205, 208, 212, 230, 231, 241, 245, 261, 265, 267, 276, 277, 283, 286, 289, 300, 319, 330, 335, 357, 389, 390, 415, 420, 426, 432, 441, 450, 462, 474, 485, 494, 504, 514, 542, 544, 548, 563, 567, 574, 585, 588, 590, 606, 607, 627, 631, 636, 654, 662, 665, 666, 682, 707, 710, 717, 732, 736, 737, 741, 766, 771, 791, 804, 805, 808, 810, 814, 817, 824, 834, 839, 840, 842, 846, 848, 852, 864, 866, 873, 884, 891, 895, 905, 915, 919, 926, 930, 932, 933, 944, 960, 961, 965, 970, 977, 982, 989, 990, 992, 997, 1001, 1007, 1009, 1040, 1052, 1055, 1065, 1066, 1075, 1080, 1090, 1105, 1112, 1113, 1115, 1120, 1130, 1137, 1138, 1166, 1176, 1179, 1184, 1185, 1190, 1195, 1209, 1212, 1213, 1218, 1220, 1223, 1224, 1231, 1236, 1240, 1251, 1259, 1260, 1265, 1272, 1280, 1304, 1306, 1312, 1320, 1328, 1337, 1354, 1362, 1383, 1386, 1388, 1397, 1410, 1412, 1435, 1438, 1439, 1442, 1448, 1466, 1467, 1475, 1490, 1492, 1499, 1510, 1530, 1534, 1541, 1542, 1549, 1551, 1552, 1554, 1560, 1569, 1581, 1590, 1618, 1625, 1627, 1628, 1635, 1639, 1640, 1659, 1661, 1670, 1673, 1689, 1692, 1697, 1699, 1707, 1715, 1724, 1732, 1737, 1757, 1768, 1769, 1782, 1785, 1798, 1802, 1805, 1810, 1815, 1859, 1869, 1870, 1886, 1888, 1889, 1890, 1911, 1922, 1924, 1929, 1934, 1940, 1941, 1944, 1955, 1971, 1975, 1976, 1977, 1980, 1984, 1995, 2007, 2010, 2018, 2028, 2030, 2047, 2048, 2049, 2051, 2054, 2063, 2064, 2079, 2093, 2112, 2131, 2133, 2162, 2175, 2178, 2198, 2213, 2221, 2230, 2231, 2232, 2233, 2234, 2236, 2237, 2243, 2256, 2271, 2272, 2287, 2288, 2295, 2309, 2313, 2344, 2345, 2346, 2348, 2364, 2371, 2402, 2414, 2417, 2426, 2433, 2437, 2443, 2444, 2447, 2458, 2464, 2479, 2486, 2487, 2492, 2494, 2501, 2515, 2518, 2533, 2539, 2545, 2555, 2560, 2564, 2568, 2570, 2573, 2576, 2580, 2581, 2597, 2599, 2602, 2608, 2611, 2613, 2616, 2621, 2634, 2665, 2668, 2678, 2690, 2692, 2699, 2703, 2706, 2707, 2710, 2725, 2730, 2736, 2748, 2756, 2772, 2782, 2785, 2786, 2790, 2809, 2835, 2836, 2842, 2850, 2858, 2861, 2866, 2868, 2872, 2873, 2875, 2878, 2882, 2893, 2896, 2903, 2909, 2915, 2931, 2947, 2951, 2957, 2960, 2961, 2964, 2968, 2972, 2985, 2986, 2997, 3000, 3017, 3022, 3030, 3039, 3050, 3055, 3068, 3071, 3087, 3093, 3095, 3107, 3109, 3112, 3126, 3127, 3132, 3138, 3159, 3168, 3207, 3208, 3212, 3228, 3236, 3238, 3241, 3247, 3255, 3258, 3287, 3298, 3300, 3302, 3321, 3326, 3339, 3352, 3359, 3375, 3380, 3397, 3401, 3404, 3417, 3427, 3433, 3462, 3469, 3471, 3485, 3487, 3496, 3516, 3518, 3519, 3521, 3529, 3530, 3557, 3559, 3562, 3609, 3610, 3613, 3619, 3633, 3642, 3662, 3664, 3665, 3682, 3698, 3702, 3703, 3721, 3731, 3735, 3740, 3743, 3754, 3769, 3812, 3833, 3834, 3840, 3842, 3846, 3849, 3857, 3882, 3885, 3887, 3896, 3914, 3915, 3918, 3920, 3925, 3934, 3953, 3961, 3962, 3966, 3967, 3968, 3973, 3979, 4021, 4023, 4036, 4041, 4048, 4050, 4058, 4061, 4065, 4092, 4094, 4115, 4118, 4126, 4133, 4138, 4139, 4141, 4142, 4149, 4152, 4156, 4170, 4180, 4210, 4216, 4222, 4225, 4234, 4240, 4278, 4291, 4292, 4293, 4301, 4308, 4320, 4327, 4328, 4334, 4342, 4345, 4355, 4361, 4370, 4382, 4385, 4393, 4394, 4400, 4402, 4408, 4411, 4450, 4456, 4458, 4476, 4505, 4506, 4507, 4524, 4531, 4541, 4550, 4551, 4561, 4569, 4580, 4582, 4586, 4592, 4597, 4599, 4602, 4617, 4634, 4646, 4650, 4653, 4656, 4665, 4668, 4677, 4697, 4714, 4717, 4722, 4727, 4734, 4749, 4761, 4763, 4768, 4779, 4787, 4802, 4805, 4809, 4825, 4844, 4849, 4888, 4907, 4929, 4931, 4932, 4937, 4942, 4952, 4959, 4971, 5007, 5030, 5032, 5035, 5039, 5046, 5050, 5066, 5072, 5075, 5079, 5134, 5148, 5149, 5165, 809, 1954, 2270, 2898, 3190, 3604, 4137, 4329, 4520, 5151, 205, 534, 539, 611, 1519, 314, 457, 566, 912, 1030, 1181, 1409, 1459, 1467, 1630, 1797, 1967, 2084, 2099, 2164, 2207, 2239, 2364, 2433, 2483, 2495, 2665, 2765, 2941, 2945, 3061, 3088, 3132, 3192, 3199, 3352, 3807, 3824, 3867, 4034, 4193, 4201, 4498, 4741, 4773, 4805, 5126, 281, 554, 610, 764, 979, 1012, 1185, 1194, 1383, 1517, 1528, 1541, 1620, 1774, 1980, 2178, 2221, 2226, 2369, 2538, 2583, 2614, 2737, 2768, 2770, 2847, 3063, 3088, 3354, 3498, 3564, 3625, 3638, 3867, 3952, 3972, 4536, 4803, 4852, 5008, 1, 58, 210, 0, 14, 17, 18, 24, 29, 54, 56, 58, 64, 70, 83, 136, 161, 180, 186, 188, 200, 216, 237, 251, 256, 257, 277, 278, 280, 281, 321, 334, 346, 352, 354, 379, 439, 478, 485, 520, 524, 529, 530, 566, 606, 611, 621, 624, 638, 650, 668, 670, 704, 712, 723, 771, 834, 848, 890, 919, 938, 966, 1007, 1010, 1029, 1060, 1063, 1065, 1070, 1078, 1081, 1085, 1093, 1109, 1160, 1185, 1208, 1214, 1223, 1242, 1261, 1262, 1263, 1269, 1272, 1274, 1312, 1333, 1350, 1351, 1352, 1366, 1374, 1378, 1383, 1390, 1398, 1439, 1441, 1449, 1463, 1467, 1480, 1482, 1492, 1517, 1527, 1572, 1601, 1652, 1660, 1682, 1687, 1702, 1720, 1728, 1768, 1777, 1790, 1791, 1801, 1826, 1827, 1828, 1834, 1847, 1850, 1858, 1861, 1863, 1870, 1877, 1885, 1889, 1897, 1910, 1915, 1922, 1929, 1951, 1971, 2048, 2059, 2062, 2108, 2123, 2190, 2227, 2235, 2244, 2250, 2255, 2274, 2281, 2350, 2352, 2368, 2373, 2376, 2387, 2391, 2394, 2404, 2413, 2458, 2459, 2477, 2483, 2487, 2488, 2545, 2547, 2568, 2570, 2589, 2616, 2627, 2631, 2654, 2669, 2672, 2700, 2702, 2703, 2704, 2718, 2731, 2747, 2775, 2789, 2818, 2845, 2855, 2865, 2874, 2881, 2930, 2949, 2952, 2967, 2988, 3006, 3014, 3029, 3030, 3055, 3063, 3064, 3089, 3098, 3120, 3126, 3127, 3130, 3154, 3166, 3176, 3178, 3197, 3257, 3292, 3299, 3309, 3345, 3354, 3387, 3389, 3390, 3392, 3401, 3431, 3435, 3439, 3472, 3487, 3531, 3534, 3555, 3559, 3568, 3598, 3603, 3611, 3645, 3674, 3683, 3687, 3695, 3699, 3705, 3708, 3727, 3730, 3762, 3786, 3787, 3812, 3824, 3831, 3832, 3875, 3876, 3885, 3909, 3918, 3932, 3933, 3946, 3959, 3972, 3985, 4029, 4034, 4061, 4068, 4076, 4080, 4081, 4113, 4117, 4128, 4144, 4156, 4176, 4202, 4228, 4229, 4274, 4279, 4290, 4293, 4303, 4306, 4315, 4332, 4360, 4365, 4371, 4375, 4392, 4420, 4424, 4440, 4442, 4476, 4506, 4535, 4566, 4569, 4586, 4589, 4593, 4606, 4607, 4610, 4613, 4619, 4623, 4626, 4629, 4633, 4645, 4650, 4688, 4704, 4717, 4721, 4737, 4745, 4755, 4776, 4777, 4779, 4782, 4785, 4790, 4810, 4814, 4816, 4825, 4842, 4853, 4863, 4874, 4878, 4903, 4904, 4929, 4935, 4940, 4947, 4955, 4964, 4984, 5006, 5017, 5027, 5034, 5038, 5039, 5058, 5063, 5081, 5098, 5132, 5140, 5157, 5164, 5166, 5169, 42, 60, 122, 180, 189, 320, 329, 357, 410, 455, 506, 514, 517, 557, 582, 615, 637, 752, 753, 800, 808, 898, 944, 983, 1139, 1189, 1204, 1213, 1274, 1370, 1375, 1387, 1393, 1438, 1505, 1601, 1695, 1699, 1745, 1759, 1773, 1814, 1886, 1971, 2082, 2088, 2092, 2150, 2203, 2221, 2272, 2296, 2359, 2415, 2487, 2500, 2543, 2587, 2693, 2716, 2777, 2806, 2844, 2857, 2885, 2890, 2994, 3004, 3010, 3012, 3025, 3026, 3038, 3059, 3113, 3125, 3280, 3302, 3340, 3377, 3386, 3423, 3441, 3474, 3517, 3572, 3596, 3610, 3663, 3726, 3750, 3761, 3780, 3795, 3796, 3809, 3832, 3843, 3864, 3891, 3915, 3969, 3989, 4048, 4129, 4138, 4151, 4215, 4251, 4302, 4327, 4349, 4404, 4424, 4460, 4497, 4570, 4576, 4579, 4589, 4607, 4667, 4723, 4763, 4768, 4779, 4786, 4862, 5023, 5047, 5079, 5083, 5167, 0, 19, 37, 56, 59, 86, 90, 92, 98, 117, 118, 119, 131, 136, 141, 164, 167, 173, 187, 189, 190, 202, 214, 217, 227, 236, 249, 256, 263, 286, 287, 289, 291, 307, 308, 324, 326, 332, 334, 336, 347, 363, 371, 382, 389, 402, 409, 411, 425, 434, 440, 482, 507, 512, 517, 535, 561, 566, 567, 572, 577, 580, 581, 582, 597, 599, 608, 637, 642, 650, 656, 691, 692, 694, 698, 700, 703, 721, 729, 732, 743, 751, 754, 762, 777, 781, 787, 790, 831, 840, 873, 874, 877, 888, 889, 904, 905, 906, 908, 911, 923, 932, 938, 942, 944, 946, 954, 968, 976, 989, 1001, 1003, 1007, 1011, 1016, 1018, 1030, 1050, 1053, 1057, 1083, 1101, 1110, 1157, 1161, 1162, 1163, 1168, 1187, 1202, 1212, 1220, 1240, 1246, 1249, 1262, 1276, 1298, 1301, 1302, 1331, 1354, 1384, 1389, 1428, 1442, 1444, 1447, 1452, 1455, 1459, 1460, 1463, 1465, 1476, 1499, 1512, 1514, 1518, 1522, 1529, 1534, 1560, 1595, 1597, 1604, 1605, 1628, 1636, 1641, 1643, 1651, 1677, 1681, 1697, 1700, 1719, 1726, 1748, 1764, 1787, 1808, 1810, 1819, 1822, 1848, 1854, 1896, 1897, 1902, 1903, 1905, 1906, 1911, 1919, 1922, 1923, 1938, 1947, 1968, 1973, 1975, 1980, 1981, 1984, 1987, 1990, 1993, 2003, 2020, 2029, 2030, 2031, 2039, 2077, 2089, 2095, 2097, 2106, 2112, 2113, 2117, 2121, 2133, 2139, 2148, 2159, 2165, 2167, 2178, 2192, 2196, 2213, 2231, 2241, 2243, 2251, 2255, 2260, 2261, 2283, 2298, 2315, 2319, 2321, 2328, 2332, 2337, 2341, 2353, 2365, 2374, 2397, 2403, 2404, 2412, 2424, 2433, 2450, 2460, 2471, 2476, 2483, 2491, 2502, 2503, 2505, 2515, 2520, 2532, 2563, 2568, 2572, 2591, 2597, 2602, 2614, 2616, 2617, 2627, 2628, 2636, 2640, 2649, 2685, 2690, 2693, 2753, 2759, 2766, 2771, 2789, 2814, 2820, 2841, 2861, 2863, 2871, 2881, 2888, 2897, 2902, 2903, 2911, 2928, 2935, 2956, 2</t>
+    <t>234.6</t>
+  </si>
+  <si>
+    <t>12136</t>
+  </si>
+  <si>
+    <t>13, 15, 20, 28, 32, 33, 45, 48, 70, 76, 94, 104, 105, 117, 121, 131, 136, 139, 153, 155, 163, 164, 173, 175, 186, 188, 203, 205, 216, 232, 235, 236, 240, 248, 250, 252, 256, 260, 263, 272, 277, 285, 286, 289, 291, 304, 316, 326, 328, 330, 332, 336, 340, 351, 361, 371, 375, 380, 382, 384, 388, 399, 402, 405, 409, 419, 420, 425, 431, 436, 439, 440, 441, 445, 453, 458, 483, 485, 500, 512, 514, 530, 535, 541, 542, 558, 561, 577, 583, 584, 594, 597, 599, 605, 607, 618, 629, 636, 647, 649, 650, 656, 660, 668, 675, 676, 684, 686, 690, 701, 703, 712, 715, 721, 724, 725, 729, 732, 743, 754, 760, 762, 763, 774, 776, 784, 787, 788, 790, 804, 830, 839, 840, 841, 863, 866, 877, 881, 889, 905, 911, 919, 920, 941, 942, 954, 964, 965, 976, 977, 1004, 1007, 1011, 1016, 1030, 1031, 1050, 1053, 1054, 1056, 1066, 1080, 1082, 1083, 1087, 1096, 1105, 1110, 1112, 1116, 1119, 1145, 1154, 1159, 1164, 1165, 1170, 1180, 1186, 1191, 1194, 1197, 1207, 1220, 1222, 1223, 1235, 1240, 1246, 1248, 1249, 1262, 1263, 1264, 1267, 1269, 1276, 1288, 1298, 1301, 1302, 1315, 1326, 1332, 1351, 1354, 1368, 1371, 1389, 1397, 1401, 1413, 1417, 1420, 1431, 1439, 1443, 1446, 1447, 1455, 1459, 1461, 1463, 1464, 1467, 1472, 1491, 1494, 1495, 1496, 1499, 1522, 1534, 1552, 1569, 1581, 1583, 1588, 1595, 1613, 1625, 1628, 1630, 1634, 1636, 1643, 1647, 1654, 1657, 1675, 1677, 1680, 1697, 1705, 1708, 1716, 1717, 1719, 1726, 1737, 1747, 1748, 1759, 1767, 1770, 1772, 1781, 1783, 1787, 1798, 1807, 1808, 1810, 1814, 1815, 1822, 1832, 1838, 1839, 1844, 1848, 1852, 1854, 1859, 1868, 1877, 1878, 1883, 1884, 1888, 1889, 1891, 1892, 1896, 1903, 1904, 1905, 1906, 1911, 1912, 1915, 1916, 1918, 1919, 1922, 1928, 1933, 1938, 1943, 1955, 1968, 1980, 1981, 1986, 1993, 1995, 1996, 2003, 2007, 2008, 2026, 2027, 2029, 2030, 2032, 2048, 2050, 2063, 2068, 2070, 2073, 2079, 2097, 2106, 2107, 2112, 2116, 2121, 2124, 2125, 2126, 2131, 2133, 2137, 2139, 2163, 2165, 2166, 2168, 2175, 2178, 2181, 2185, 2187, 2191, 2192, 2223, 2229, 2241, 2256, 2261, 2262, 2265, 2266, 2269, 2273, 2276, 2279, 2282, 2284, 2291, 2292, 2297, 2298, 2313, 2315, 2316, 2319, 2320, 2322, 2323, 2324, 2328, 2332, 2334, 2337, 2338, 2340, 2341, 2347, 2354, 2355, 2356, 2368, 2372, 2374, 2375, 2376, 2383, 2385, 2397, 2404, 2406, 2411, 2412, 2416, 2433, 2463, 2471, 2476, 2478, 2483, 2485, 2499, 2500, 2502, 2503, 2504, 2505, 2507, 2545, 2551, 2552, 2556, 2560, 2562, 2567, 2568, 2572, 2589, 2593, 2597, 2601, 2615, 2617, 2624, 2627, 2642, 2659, 2660, 2672, 2678, 2683, 2686, 2690, 2693, 2696, 2701, 2706, 2710, 2748, 2753, 2771, 2772, 2780, 2801, 2804, 2813, 2814, 2815, 2819, 2821, 2825, 2828, 2833, 2837, 2843, 2847, 2857, 2863, 2868, 2874, 2878, 2882, 2888, 2902, 2911, 2917, 2931, 2935, 2948, 2953, 2955, 2956, 2964, 2979, 2983, 2985, 2986, 2987, 2988, 2993, 3025, 3032, 3040, 3043, 3051, 3054, 3071, 3072, 3079, 3085, 3095, 3102, 3105, 3109, 3113, 3121, 3126, 3127, 3130, 3135, 3136, 3155, 3167, 3172, 3174, 3175, 3177, 3178, 3181, 3185, 3194, 3195, 3197, 3200, 3208, 3216, 3219, 3220, 3223, 3228, 3232, 3233, 3236, 3246, 3249, 3253, 3263, 3280, 3293, 3302, 3307, 3314, 3326, 3332, 3333, 3335, 3346, 3350, 3352, 3353, 3359, 3360, 3366, 3367, 3371, 3377, 3378, 3382, 3399, 3404, 3410, 3414, 3416, 3425, 3428, 3435, 3438, 3442, 3452, 3458, 3461, 3463, 3465, 3487, 3502, 3519, 3521, 3530, 3540, 3542, 3561, 3569, 3582, 3586, 3590, 3595, 3597, 3603, 3608, 3618, 3621, 3622, 3629, 3632, 3633, 3641, 3649, 3659, 3661, 3663, 3665, 3666, 3677, 3679, 3686, 3687, 3689, 3694, 3701, 3710, 3720, 3721, 3725, 3728, 3733, 3734, 3743, 3760, 3769, 3783, 3785, 3786, 3801, 3803, 3819, 3827, 3829, 3834, 3851, 3858, 3859, 3860, 3864, 3867, 3876, 3877, 3885, 3894, 3895, 3909, 3912, 3914, 3915, 3917, 3921, 3925, 3927, 3933, 3936, 3945, 3952, 3955, 3980, 3987, 4003, 4018, 4021, 4024, 4026, 4038, 4051, 4057, 4058, 4064, 4066, 4067, 4076, 4084, 4088, 4092, 4096, 4114, 4117, 4120, 4123, 4139, 4142, 4145, 4151, 4152, 4159, 4162, 4169, 4180, 4184, 4185, 4186, 4193, 4198, 4209, 4216, 4219, 4237, 4243, 4250, 4251, 4263, 4265, 4272, 4273, 4282, 4289, 4329, 4331, 4333, 4338, 4339, 4345, 4346, 4347, 4352, 4354, 4355, 4356, 4373, 4388, 4389, 4393, 4396, 4408, 4410, 4415, 4430, 4433, 4436, 4439, 4449, 4451, 4455, 4458, 4468, 4491, 4501, 4505, 4514, 4515, 4527, 4534, 4538, 4540, 4542, 4544, 4555, 4558, 4560, 4564, 4565, 4569, 4573, 4579, 4583, 4593, 4597, 4602, 4613, 4618, 4624, 4626, 4628, 4632, 4633, 4636, 4637, 4638, 4645, 4656, 4667, 4672, 4679, 4681, 4682, 4693, 4699, 4721, 4729, 4732, 4734, 4736, 4758, 4759, 4765, 4778, 4779, 4780, 4782, 4785, 4787, 4792, 4797, 4799, 4803, 4828, 4832, 4841, 4856, 4884, 4892, 4925, 4936, 4947, 4953, 4956, 4957, 4964, 4965, 4971, 4974, 4979, 4980, 4989, 5007, 5008, 5014, 5018, 5020, 5033, 5037, 5042, 5055, 5063, 5075, 5076, 5079, 5081, 5084, 5085, 5087, 5089, 5097, 5102, 5107, 5111, 5113, 5115, 5126, 5129, 5149, 5150, 5158, 5160, 5163, 5167, 15, 26, 28, 38, 56, 62, 79, 104, 106, 121, 123, 125, 171, 174, 175, 260, 278, 320, 394, 432, 433, 487, 512, 536, 538, 543, 562, 581, 590, 605, 633, 644, 666, 688, 725, 735, 748, 763, 793, 804, 815, 866, 905, 913, 925, 926, 933, 987, 990, 1053, 1106, 1123, 1138, 1145, 1196, 1218, 1225, 1255, 1256, 1265, 1293, 1307, 1337, 1356, 1364, 1378, 1419, 1422, 1450, 1494, 1529, 1549, 1628, 1633, 1649, 1659, 1683, 1686, 1744, 1747, 1765, 1774, 1778, 1788, 1809, 1822, 1826, 1843, 1849, 1859, 1880, 1894, 1907, 1910, 1996, 2049, 2058, 2062, 2115, 2155, 2198, 2236, 2282, 2296, 2305, 2336, 2346, 2350, 2385, 2426, 2516, 2557, 2610, 2644, 2660, 2709, 2725, 2748, 2821, 2873, 2902, 2912, 2938, 2946, 2964, 2984, 2997, 3020, 3034, 3035, 3051, 3065, 3068, 3083, 3089, 3154, 3168, 3200, 3207, 3223, 3236, 3273, 3292, 3325, 3335, 3370, 3371, 3387, 3404, 3414, 3423, 3451, 3513, 3521, 3587, 3595, 3598, 3608, 3619, 3637, 3646, 3653, 3667, 3675, 3739, 3752, 3758, 3774, 3775, 3829, 3862, 3904, 3914, 3915, 3921, 3928, 3934, 3948, 3967, 3990, 4005, 4038, 4049, 4061, 4094, 4107, 4114, 4157, 4179, 4202, 4220, 4222, 4259, 4264, 4270, 4274, 4288, 4312, 4337, 4351, 4393, 4424, 4426, 4449, 4479, 4506, 4540, 4550, 4555, 4564, 4569, 4590, 4619, 4630, 4635, 4640, 4654, 4656, 4672, 4710, 4711, 4723, 4740, 4745, 4927, 4929, 4952, 4989, 5037, 5042, 5065, 5082, 5112, 5143, 5144, 5148, 1, 8, 13, 15, 24, 25, 31, 32, 37, 38, 43, 68, 75, 76, 79, 85, 86, 87, 94, 103, 111, 113, 126, 128, 130, 131, 133, 135, 139, 143, 145, 154, 155, 166, 171, 172, 173, 174, 178, 185, 188, 198, 203, 206, 212, 221, 250, 252, 256, 265, 271, 272, 277, 279, 285, 286, 296, 301, 311, 326, 327, 336, 337, 340, 349, 350, 352, 361, 365, 380, 386, 405, 406, 410, 424, 425, 432, 436, 439, 441, 445, 451, 454, 460, 469, 473, 476, 477, 480, 484, 485, 490, 504, 506, 512, 514, 515, 520, 521, 524, 526, 528, 539, 541, 542, 545, 547, 555, 558, 563, 566, 570, 574, 577, 581, 588, 594, 598, 604, 615, 623, 627, 629, 640, 660, 672, 675, 679, 681, 686, 700, 707, 717, 724, 728, 731, 732, 736, 741, 754, 759, 760, 767, 768, 771, 774, 776, 784, 787, 790, 796, 823, 826, 827, 829, 831, 837, 840, 841, 842, 844, 851, 856, 860, 862, 863, 868, 873, 877, 881, 885, 890, 897, 899, 900, 914, 915, 925, 930, 941, 950, 956, 960, 964, 965, 971, 974, 977, 979, 983, 987, 988, 998, 1003, 1004, 1039, 1044, 1045, 1054, 1062, 1081, 1082, 1087, 1090, 1111, 1112, 1116, 1135, 1138, 1142, 1148, 1156, 1164, 1168, 1172, 1182, 1185, 1186, 1207, 1208, 1214, 1215, 1219, 1223, 1224, 1230, 1239, 1241, 1243, 1246, 1248, 1252, 1255, 1256, 1259, 1262, 1263, 1276, 1301, 1312, 1320, 1324, 1337, 1342, 1351, 1353, 1363, 1366, 1367, 1375, 1386, 1388, 1389, 1394, 1397, 1401, 1403, 1410, 1413, 1417, 1426, 1428, 1439, 1444, 1446, 1447, 1449, 1455, 1459, 1463, 1464, 1475, 1483, 1493, 1494, 1495, 1498, 1499, 1504, 1510, 1519, 1520, 1528, 1534, 1540, 1541, 1544, 1552, 1558, 1569, 1572, 1574, 1581, 1583, 1596, 1601, 1603, 1608, 1618, 1623, 1625, 1630, 1636, 1639, 1644, 1646, 1649, 1655, 1656, 1660, 1665, 1666, 1670, 1675, 1676, 1677, 1680, 1681, 1682, 1683, 1693, 1698, 1708, 1711, 1717, 1722, 1727, 1730, 1737, 1742, 1749, 1752, 1757, 1759, 1762, 1767, 1772, 1776, 1779, 1782, 1787, 1792, 1797, 1805, 1806, 1808, 1816, 1844, 1849, 1854, 1857, 1864, 1867, 1868, 1871, 1873, 1877, 1884, 1889, 1890, 1892, 1896, 1904, 1906, 1912, 1917, 1921, 1922, 1924, 1930, 1934, 1937, 1944, 1954, 1958, 1962, 1975, 1976, 1980, 1981, 1990, 1993, 1996, 2008, 2012, 2013, 2016, 2023, 2030, 2037, 2038, 2040, 2043, 2051, 2054, 2056, 2066, 2067, 2074, 2079, 2083, 2090, 2103, 2104, 2105, 2106, 2107, 2112, 2113, 2114, 2115, 2124, 2126, 2133, 2141, 2145, 2148, 2156, 2163, 2167, 2170, 2171, 2185, 2192, 2198, 2204, 2218, 2227, 2234, 2241, 2243, 2246, 2266, 2271, 2273, 2276, 2280, 2284, 2288, 2292, 2298, 2301, 2303, 2308, 2316, 2320, 2322, 2323, 2332, 2334, 2335, 2338, 2341, 2346, 2347, 2348, 2352, 2365, 2368, 2372, 2376, 2385, 2391, 2417, 2419, 2435, 2436, 2439, 2447, 2450, 2452, 2454, 2456, 2458, 2468, 2469, 2471, 2477, 2478, 2482, 2485, 2486, 2488, 2491, 2492, 2494, 2495, 2499, 2515, 2521, 2522, 2531, 2535, 2545, 2550, 2553, 2554, 2559, 2560, 2562, 2563, 2567, 2568, 2570, 2588, 2604, 2608, 2609, 2610, 2613, 2617, 2624, 2625, 2627, 2630, 2633, 2634, 2636, 2641, 2648, 2650, 2654, 2658, 2659, 2660, 2662, 2665, 2674, 2678, 2679, 2683, 2685, 2686, 2687, 2689, 2696, 2701, 2706, 2709, 2711, 2722, 2723, 2724, 2734, 2739, 2744, 2745, 2747, 2749, 2753, 2764, 2766, 2768, 2772, 2775, 2777, 2780, 2781, 2785, 2787, 2795, 2815, 2818, 2819, 2820, 2829, 2837, 2846, 2848, 2850, 2856, 2863, 2865, 2866, 2875, 2878, 2881, 2905, 2911, 2913, 2921, 2935, 2936, 2940, 2948, 2973, 2975, 2978, 2983, 2985, 2998, 2999, 3008, 3010, 3026, 3030, 3035, 3038, 3044, 3045, 3057, 3069, 3071, 3076, 3079, 3090, 3092, 3097, 3098, 3102, 3108, 3109, 3110, 3113, 3119, 3127, 3130, 3131, 3134, 3136, 3138, 3155, 3161, 3168, 3174, 3180, 3181, 3182, 3187, 3197, 3198, 3200, 3208, 3213, 3219, 3222, 3235, 3236, 3246, 3251, 3261, 3263, 3264, 3265, 3279, 3280, 3286, 3302, 3305, 3308, 3309, 3314, 3321, 3326, 3329, 3332, 3333, 3340, 3343, 3350, 3353, 3356, 3371, 3381, 3391, 3399, 3403, 3414, 3423, 3424, 3425, 3431, 3432, 3435, 3438, 3442, 3449, 3453, 3456, 3465, 3466, 3471, 3474, 3476, 3482, 3483, 3484, 3497, 3506, 3508, 3521, 3541, 3551, 3567, 3569, 3575, 3577, 3582, 3585, 3587, 3595, 3596, 3597, 3601, 3605, 3608, 3618, 3619, 3626, 3628, 3631, 3632, 3648, 3649, 3656, 3657, 3660, 3666, 3673, 3677, 3682, 3685, 3686, 3687, 3693, 3708, 3710, 3718, 3720, 3722, 3724, 3732, 3758, 3759, 3764, 3771, 3777, 3790, 3815, 3827, 3834, 3838, 3840, 3851, 3852, 3853, 3859, 3865, 3880, 3884, 3887, 3889, 3892, 3894, 3895, 3896, 3899, 3904, 3907, 3912, 3915, 3917, 3925, 3926, 3932, 3937, 3949, 3953, 3958, 3962, 3970, 3971, 3972, 3975, 3980, 3984, 3985, 3987, 3988, 3990, 3998, 4011, 4012, 4018, 4022, 4026, 4030, 4037, 4051, 4055, 4056, 4061, 4064, 4066, 4073, 4077, 4082, 4084, 4096, 4097, 4098, 4105, 4113, 4114, 4116, 4119, 4120, 4122, 4123, 4124, 4136, 4138, 4139, 4140, 4162, 4163, 4166, 4171, 4173, 4179, 4180, 4185, 4192, 4199, 4209, 4216, 4223, 4238, 4246, 4259, 4262, 4270, 4277, 4289, 4290, 4297, 4301, 4306, 4310, 4316, 4321, 4329, 4331, 4337, 4338, 4339, 4343, 4345, 4348, 4351, 4354, 4356, 4357, 4360, 4378, 4393, 4395, 4396, 4401, 4409, 4412, 4428, 4429, 4433, 4438, 4442, 4446, 4468, 4475, 4484, 4488, 4501, 4502, 4504, 4505, 4507, 4508, 4515, 4520, 4525, 4526, 4532, 4540, 4541, 4542, 4544, 4546, 4552, 4561, 4564, 4573, 4577, 4582, 4602, 4612, 4616, 4624, 4626, 4627, 4628, 4629, 4632, 4638, 4649, 4652, 4667, 4679, 4688, 4691, 4692, 4712, 4728, 4731, 4734, 4744, 4759, 4763, 4770, 4778, 4782, 4783, 4785, 4787, 4790, 4792, 4796, 4797, 4798, 4805, 4812, 4815, 4816, 4839, 4841, 4847, 4850, 4861, 4862, 4864, 4866, 4868, 4872, 4874, 4880, 4883, 4892, 4913, 4919, 4922, 4927, 4928, 4929, 4942, 4951, 4954, 4957, 4962, 4964, 4966, 4981, 4984, 4986, 4988, 5018, 5020, 5030, 5031, 5033, 5036, 5037, 5041, 5044, 5047, 5060, 5062, 5063, 5072, 5075, 5077, 5084, 5113, 5118, 5121, 5133, 5144, 5155, 5160, 5161, 5169, 5172, 15, 18, 26, 37, 48, 57, 80, 86, 92, 102, 104, 116, 131, 135, 139, 146, 148, 154, 157, 173, 188, 216, 218, 231, 237, 252, 265, 269, 295, 333, 335, 340, 358, 365, 368, 374, 375, 380, 385, 387, 406, 413, 425, 436, 441, 444, 445, 455, 461, 468, 477, 480, 482, 491, 498, 511, 527, 547, 583, 588, 591, 603, 612, 618, 627, 629, 636, 657, 661, 662, 669, 682, 695, 717, 748, 754, 762, 764, 776, 795, 825, 846, 848, 856, 857, 862, 863, 865, 866, 874, 884, 901, 913, 915, 1008, 1020, 1025, 1033, 1049, 1054, 1068, 1093, 1100, 1124, 1133, 1146, 1168, 1185, 1186, 1190, 1191, 1194, 1196, 1204, 1207, 1208, 1221, 1233, 1248, 1249, 1278, 1300, 1312, 1315, 1346, 1350, 1371, 1374, 1377, 1412, 1443, 1464, 1466, 1513, 1535, 1544, 1574, 1584, 1602, 1625, 1628, 1631, 1640, 1653, 1692, 1696, 1697, 1699, 1702, 1718, 1738, 1746, 1753, 1757, 1813, 1838, 1851, 1864, 1865, 1881, 1885, 1890, 1897, 1900, 1902, 1904, 1909, 1917, 1918, 1939, 1944, 1958, 1971, 1978, 1984, 1986, 2000, 2011, 2016, 2018, 2068, 2083, 2087, 2116, 2133, 2144, 2162, 2165, 2171, 2172, 2176, 2185, 2195, 2207, 2221, 2223, 2256, 2260, 2268, 2271, 2302, 2303, 2313, 2331, 2359, 2362, 2366, 2384, 2435, 2445, 2447, 2449, 2458, 2483, 2499, 2508, 2525, 2531, 2558, 2560, 2583, 2586, 2587, 2614, 2624, 2634, 2636, 2654, 2662, 2684, 2696, 2701, 2707, 2719, 2727, 2745, 2749, 2772, 2787, 2789, 2795, 2804, 2812, 2818, 2820, 2839, 2840, 2852, 2855, 2856, 2857, 2863, 2866, 2876, 2921, 2947, 2961, 2974, 2975, 2980, 2993, 3012, 3016, 3026, 3050, 3061, 3062, 3078, 3081, 3083, 3117, 3121, 3129, 3134, 3158, 3183, 3187, 3192, 3200, 3216, 3221, 3232, 3241, 3245, 3246, 3264, 3294, 3301, 3313, 3322, 3327, 3336, 3355, 3356, 3360, 3364, 3378, 3379, 3399, 3404, 3405, 3409, 3426, 3449, 3458, 3468, 3484, 3496, 3503, 3506, 3508, 3511, 3520, 3521, 3525, 3534, 3554, 3572, 3580, 3582, 3598, 3617, 3633, 3679, 3748, 3752, 3769, 3789, 3796, 3809, 3832, 3833, 3844, 3865, 3868, 3875, 3884, 3893, 3905, 3926, 3929, 3936, 3952, 3959, 3974, 3987, 3991, 4003, 4008, 4023, 4064, 4075, 4076, 4082, 4095, 4097, 4102, 4108, 4110, 4122, 4131, 4139, 4143, 4155, 4162, 4169, 4172, 4173, 4234, 4238, 4241, 4262, 4265, 4274, 4296, 4301, 4309, 4311, 4323, 4362, 4389, 4393, 4394, 4400, 4406, 4461, 4485, 4492, 4501, 4502, 4505, 4526, 4542, 4547, 4552, 4560, 4580, 4594, 4599, 4607, 4611, 4616, 4624, 4642, 4648, 4660, 4685, 4697, 4712, 4723, 4773, 4774, 4775, 4784, 4787, 4812, 4822, 4841, 4869, 4872, 4925, 4935, 4948, 4964, 4970, 4977, 4983, 4988, 5005, 5006, 5018, 5034, 5045, 5051, 5075, 5079, 5085, 5088, 5090, 5115, 5122, 5126, 5164, 5169, 5170, 111, 187, 281, 294, 300, 349, 384, 515, 584, 608, 851, 899, 1010, 1152, 1153, 1552, 1897, 2245, 2250, 2359, 2721, 2786, 2935, 3127, 3136, 3164, 3201, 3208, 3232, 3293, 3302, 3418, 3441, 3612, 4048, 4061, 4065, 4066, 4096, 4245, 4252, 4486, 4526, 4672, 4956, 5020, 5126, 5136, 29, 49, 66, 93, 98, 120, 124, 184, 187, 205, 220, 238, 245, 257, 263, 287, 345, 349, 360, 442, 457, 564, 584, 627, 657, 672, 775, 799, 818, 852, 898, 979, 1008, 1011, 1024, 1041, 1057, 1061, 1126, 1140, 1153, 1159, 1194, 1196, 1200, 1228, 1263, 1277, 1296, 1375, 1397, 1404, 1457, 1483, 1495, 1528, 1531, 1533, 1570, 1584, 1592, 1666, 1689, 1699, 1747, 1762, 1857, 1868, 1887, 1905, 1926, 1936, 1951, 1954, 1956, 1962, 1972, 1973, 2032, 2054, 2101, 2127, 2140, 2145, 2148, 2155, 2192, 2237, 2265, 2315, 2346, 2350, 2367, 2454, 2468, 2477, 2568, 2601, 2699, 2768, 2825, 2828, 2835, 2839, 2862, 2880, 2881, 2930, 3044, 3082, 3123, 3127, 3164, 3165, 3178, 3305, 3333, 3345, 3361, 3404, 3418, 3452, 3544, 3584, 3605, 3610, 3663, 3666, 3672, 3703, 3723, 3728, 3785, 3837, 3862, 3863, 3929, 3949, 3964, 4034, 4127, 4144, 4154, 4186, 4200, 4243, 4252, 4339, 4348, 4387, 4424, 4429, 4446, 4473, 4486, 4535, 4577, 4588, 4637, 4640, 4647, 4661, 4672, 4690, 4728, 4734, 4796, 4804, 4816, 4825, 4890, 4901, 4918, 4924, 4948, 4959, 5037, 5046, 5094, 5117, 5124, 5157, 38, 41, 56, 84, 89, 99, 112, 133, 136, 141, 152, 228, 257, 281, 294, 295, 321, 346, 347, 363, 424, 433, 468, 541, 544, 548, 582, 611, 631, 657, 711, 721, 760, 826, 848, 906, 988, 1028, 1034, 1052, 1061, 1071, 1107, 1113, 1131, 1138, 1145, 1150, 1153, 1186, 1188, 1191, 1210, 1250, 1281, 1292, 1300, 1324, 1353, 1384, 1393, 1414, 1417, 1438, 1443, 1482, 1510, 1530, 1589, 1632, 1652, 1707, 1747, 1749, 1774, 1782, 1810, 1835, 1861, 1877, 1903, 1912, 1928, 1940, 1954, 1975, 1991, 2044, 2094, 2118, 2147, 2166, 2226, 2231, 2261, 2266, 2303, 2342, 2364, 2369, 2390, 2429, 2436, 2437, 2449, 2483, 2539, 2556, 2560, 2608, 2614, 2634, 2651, 2652, 2685, 2699, 2715, 2722, 2742, 2759, 2764, 2771, 2784, 2816, 2838, 2840, 2889, 2916, 2919, 2938, 2941, 2944, 2957, 2960, 2972, 3025, 3057, 3077, 3089, 3124, 3126, 3159, 3161, 3167, 3175, 3183, 3248, 3327, 3341, 3345, 3390, 3396, 3409, 3431, 3451, 3452, 3456, 3515, 3517, 3551, 3559, 3561, 3569, 3610, 3617, 3627, 3669, 3685, 3693, 3694, 3698, 3739, 3741, 3827, 3859, 3863, 3873, 3874, 3919, 4003, 4083, 4118, 4128, 4150, 4177, 4220, 4316, 4343, 4410, 4412, 4426, 4446, 4483, 4486, 4492, 4500, 4520, 4527, 4535, 4569, 4579, 4589, 4602, 4616, 4645, 4667, 4689, 4690, 4697, 4717, 4732, 4734, 4790, 4803, 4849, 4853, 4872, 4873, 4878, 4887, 4890, 4919, 4964, 4992, 5018, 5027, 5031, 5035, 5047, 5051, 5059, 5163, 101, 125, 146, 225, 258, 419, 447, 528, 533, 582, 583, 712, 799, 919, 927, 940, 1066, 1201, 1223, 1531, 1569, 1586, 1692, 1875, 1919, 1976, 2002, 2032, 2092, 2133, 2191, 2193, 2244, 2325, 2342, 2440, 2518, 2533, 2549, 2613, 2652, 2668, 2692, 2702, 2704, 2828, 2873, 2887, 2999, 3017, 3044, 3062, 3231, 3302, 3388, 3452, 3821, 3877, 3901, 3910, 3964, 3965, 4004, 4049, 4112, 4175, 4283, 4384, 4586, 4709, 4810, 4817, 4888, 4997, 5016, 5098, 101, 121, 455, 538, 810, 1073, 1183, 1555, 1659, 1889, 1954, 2005, 2078, 2121, 2402, 2539, 2582, 2620, 3079, 3095, 3167, 3390, 3452, 3529, 3541, 3597, 3919, 3935, 4085, 4135, 4378, 4624, 4677, 4887, 4908, 1, 59, 70, 249, 350, 448, 537, 643, 666, 718, 761, 775, 798, 866, 873, 927, 963, 1028, 1069, 1200, 1231, 1307, 1358, 1360, 1618, 1651, 1664, 1711, 1722, 1749, 1766, 1780, 1795, 1827, 1831, 1895, 1904, 1914, 1973, 2077, 2083, 2211, 2254, 2272, 2337, 2348, 2391, 2422, 2433, 2515, 2545, 2569, 2627, 2664, 2677, 2679, 2693, 2873, 2886, 2916, 3059, 3062, 3081, 3212, 3236, 3246, 3395, 3405, 3450, 3490, 3725, 3808, 3921, 3962, 3996, 4015, 4037, 4106, 4143, 4274, 4327, 4404, 4484, 4619, 4678, 4712, 4736, 4814, 4881, 4900, 4940, 5013, 5091, 5108, 5111, 5126, 25, 101, 144, 171, 180, 186, 189, 206, 228, 276, 280, 281, 300, 327, 329, 380, 560, 582, 600, 606, 699, 763, 764, 777, 792, 815, 885, 898, 983, 997, 1041, 1189, 1231, 1256, 1274, 1280, 1305, 1362, 1393, 1415, 1438, 1458, 1475, 1493, 1495, 1621, 1680, 1698, 1733, 1774, 1775, 1802, 1812, 1827, 1835, 1861, 1883, 1954, 2111, 2127, 2150, 2158, 2162, 2166, 2234, 2343, 2364, 2422, 2439, 2474, 2504, 2513, 2539, 2587, 2662, 2664, 2693, 2771, 2777, 2782, 2785, 2806, 2816, 2835, 2860, 2953, 3006, 3015, 3020, 3135, 3159, 3249, 3280, 3302, 3315, 3345, 3355, 3420, 3448, 3531, 3551, 3610, 3625, 3638, 3640, 3663, 3689, 3694, 3724, 3728, 3744, 3837, 3877, 3891, 3900, 3934, 3944, 3966, 4034, 4048, 4093, 4149, 4164, 4169, 4333, 4378, 4392, 4429, 4442, 4451, 4579, 4602, 4607, 4624, 4717, 4742, 4749, 4763, 4786, 4798, 4830, 4872, 4906, 5001, 5013, 5023, 5126, 5156, 5159, 13, 71, 93, 94, 304, 312, 373, 413, 422, 534, 544, 595, 642, 681, 693, 721, 806, 809, 841, 1148, 1208, 1232, 1241, 1361, 1476, 1586, 1616, 1642, 1654, 1695, 1777, 1854, 1917, 1967, 1969, 1971, 1976, 1997, 2256, 2275, 2345, 2381, 2492, 2561, 2563, 2594, 2618, 2625, 2683, 2702, 2768, 2792, 2860, 2865, 2889, 3039, 3104, 3185, 3193, 3215, 3245, 3266, 3274, 3294, 3303, 3322, 3326, 3333, 3339, 3352, 3474, 3520, 3539, 3648, 3663, 3672, 3673, 3754, 3904, 3953, 3963, 4023, 4035, 4131, 4165, 4195, 4209, 4332, 4338, 4409, 4467, 4585, 4684, 4761, 4783, 4832, 4856, 4970, 4995, 5063, 5140, 58, 109, 121, 125, 146, 172, 182, 210, 258, 311, 319, 325, 375, 381, 409, 419, 422, 447, 455, 462, 485, 563, 583, 693, 810, 927, 940, 954, 1061, 1066, 1073, 1093, 1291, 1338, 1435, 1467, 1535, 1555, 1569, 1600, 1614, 1666, 1898, 1917, 1919, 1923, 1954, 2002, 2007, 2028, 2053, 2058, 2089, 2092, 2099, 2121, 2133, 2221, 2270, 2289, 2291, 2325, 2374, 2421, 2440, 2533, 2613, 2614, 2619, 2668, 2699, 2731, 2828, 2838, 2846, 2886, 2896, 2967, 3095, 3105, 3124, 3185, 3194, 3197, 3198, 3228, 3260, 3380, 3388, 3404, 3451, 3460, 3521, 3529, 3642, 3651, 3684, 3740, 3801, 3823, 3935, 3952, 3970, 3990, 4077, 4135, 4304, 4333, 4369, 4400, 4540, 4586, 4627, 4711, 4721, 4778, 4810, 4817, 4879, 4888, 5005, 84, 116, 205, 349, 422, 627, 661, 927, 932, 952, 1124, 1311, 1351, 1366, 1440, 1512, 1532, 1702, 1886, 1895, 1923, 1997, 2072, 2133, 2404, 2450, 2531, 2634, 2990, 3006, 3030, 3197, 3354, 3448, 3838, 3948, 4213, 4585, 10, 18, 37, 41, 45, 48, 49, 75, 84, 85, 105, 109, 111, 131, 140, 146, 161, 167, 172, 173, 175, 176, 179, 180, 184, 207, 211, 215, 220, 269, 279, 290, 292, 299, 311, 312, 314, 315, 320, 329, 340, 354, 358, 368, 369, 370, 372, 384, 385, 396, 400, 419, 422, 425, 433, 434, 435, 438, 440, 458, 476, 479, 514, 517, 537, 555, 563, 583, 589, 627, 631, 642, 660, 665, 669, 671, 672, 673, 686, 699, 700, 714, 716, 718, 720, 724, 737, 761, 766, 809, 831, 833, 841, 844, 846, 850, 852, 873, 874, 903, 905, 906, 918, 929, 937, 941, 955, 963, 988, 997, 1008, 1017, 1029, 1034, 1057, 1060, 1061, 1064, 1070, 1079, 1117, 1119, 1123, 1133, 1142, 1162, 1163, 1177, 1189, 1190, 1191, 1215, 1225, 1229, 1263, 1281, 1307, 1315, 1346, 1352, 1353, 1355, 1374, 1383, 1395, 1435, 1436, 1443, 1445, 1453, 1455, 1458, 1474, 1480, 1492, 1500, 1525, 1535, 1542, 1549, 1555, 1568, 1578, 1579, 1605, 1608, 1627, 1634, 1636, 1637, 1642, 1653, 1658, 1663, 1677, 1721, 1725, 1741, 1744, 1753, 1761, 1764, 1778, 1787, 1801, 1809, 1814, 1816, 1826, 1831, 1850, 1852, 1863, 1868, 1878, 1886, 1940, 1954, 1969, 1972, 1996, 2005, 2011, 2019, 2023, 2050, 2086, 2088, 2090, 2104, 2116, 2121, 2133, 2151, 2175, 2176, 2180, 2206, 2218, 2222, 2230, 2241, 2268, 2273, 2275, 2279, 2291, 2292, 2297, 2309, 2315, 2324, 2326, 2348, 2351, 2356, 2358, 2366, 2373, 2406, 2413, 2415, 2417, 2418, 2421, 2445, 2449, 2461, 2470, 2483, 2485, 2491, 2492, 2518, 2538, 2540, 2547, 2551, 2553, 2557, 2576, 2596, 2641, 2675, 2680, 2688, 2696, 2703, 2706, 2711, 2733, 2741, 2745, 2747, 2757, 2784, 2785, 2787, 2793, 2806, 2822, 2831, 2833, 2837, 2839, 2845, 2896, 2897, 2903, 2907, 2910, 2911, 2916, 2930, 2932, 2936, 2937, 2942, 2953, 2960, 2973, 2975, 2980, 2985, 2987, 2998, 3010, 3021, 3023, 3029, 3043, 3051, 3061, 3069, 3095, 3124, 3126, 3127, 3150, 3176, 3180, 3184, 3186, 3193, 3202, 3210, 3223, 3232, 3263, 3273, 3274, 3276, 3298, 3317, 3322, 3331, 3343, 3374, 3382, 3388, 3400, 3414, 3425, 3448, 3453, 3460, 3466, 3468, 3469, 3471, 3479, 3484, 3488, 3507, 3517, 3521, 3529, 3533, 3538, 3569, 3571, 3588, 3602, 3605, 3611, 3617, 3633, 3645, 3663, 3667, 3669, 3683, 3693, 3698, 3708, 3715, 3717, 3730, 3732, 3737, 3738, 3740, 3766, 3790, 3793, 3805, 3828, 3837, 3841, 3845, 3849, 3852, 3862, 3870, 3890, 3914, 3922, 3935, 3947, 3952, 3953, 3965, 3969, 3981, 3985, 3996, 4000, 4028, 4029, 4032, 4034, 4037, 4056, 4069, 4070, 4071, 4081, 4084, 4088, 4096, 4119, 4120, 4129, 4140, 4149, 4157, 4162, 4168, 4169, 4184, 4202, 4209, 4246, 4253, 4262, 4263, 4276, 4279, 4293, 4301, 4310, 4312, 4317, 4320, 4323, 4331, 4338, 4340, 4356, 4360, 4372, 4375, 4393, 4405, 4412, 4421, 4423, 4424, 4426, 4434, 4441, 4446, 4452, 4485, 4486, 4507, 4572, 4589, 4619, 4626, 4636, 4644, 4645, 4651, 4671, 4681, 4693, 4717, 4731, 4732, 4735, 4745, 4750, 4751, 4752, 4755, 4756, 4759, 4775, 4778, 4787, 4790, 4800, 4801, 4802, 4803, 4811, 4828, 4851, 4853, 4881, 4897, 4900, 4908, 4919, 4924, 4926, 4937, 4938, 4942, 4944, 4950, 4955, 4957, 4964, 4970, 4976, 4977, 4986, 4989, 5005, 5030, 5040, 5045, 5060, 5071, 5089, 5090, 5097, 5104, 5115, 5118, 5131, 5147, 5150, 5162, 5164, 5165, 5172, 7, 24, 30, 43, 45, 49, 65, 77, 90, 93, 98, 100, 118, 123, 134, 143, 147, 149, 151, 162, 163, 172, 173, 179, 180, 191, 202, 205, 208, 212, 230, 231, 241, 245, 261, 265, 267, 276, 277, 283, 286, 289, 300, 319, 330, 335, 357, 389, 390, 415, 420, 426, 432, 441, 450, 462, 474, 485, 494, 504, 514, 542, 544, 548, 563, 567, 574, 585, 588, 590, 606, 607, 627, 631, 636, 654, 662, 665, 666, 682, 707, 710, 717, 732, 736, 737, 741, 766, 771, 791, 804, 805, 808, 810, 814, 817, 824, 834, 839, 840, 842, 846, 848, 852, 864, 866, 873, 884, 891, 895, 905, 915, 919, 926, 930, 932, 933, 944, 960, 961, 965, 970, 977, 982, 989, 990, 992, 997, 1001, 1007, 1009, 1040, 1052, 1055, 1065, 1066, 1075, 1080, 1090, 1105, 1112, 1113, 1115, 1120, 1130, 1137, 1138, 1166, 1176, 1179, 1184, 1185, 1190, 1195, 1209, 1212, 1213, 1218, 1220, 1223, 1224, 1231, 1236, 1240, 1251, 1259, 1260, 1265, 1272, 1280, 1304, 1306, 1312, 1320, 1328, 1337, 1354, 1362, 1383, 1386, 1388, 1397, 1410, 1412, 1435, 1438, 1439, 1442, 1448, 1466, 1467, 1475, 1490, 1492, 1499, 1510, 1530, 1534, 1541, 1542, 1549, 1551, 1552, 1554, 1560, 1569, 1581, 1590, 1618, 1625, 1627, 1628, 1635, 1639, 1640, 1659, 1661, 1670, 1673, 1689, 1692, 1697, 1699, 1707, 1715, 1724, 1732, 1737, 1757, 1768, 1769, 1782, 1785, 1798, 1802, 1805, 1810, 1815, 1859, 1869, 1870, 1886, 1888, 1889, 1890, 1911, 1922, 1924, 1929, 1934, 1940, 1941, 1944, 1955, 1971, 1975, 1976, 1977, 1980, 1984, 1995, 2007, 2010, 2018, 2028, 2030, 2047, 2048, 2049, 2051, 2054, 2063, 2064, 2079, 2093, 2112, 2131, 2133, 2162, 2175, 2178, 2198, 2213, 2221, 2230, 2231, 2232, 2233, 2234, 2236, 2237, 2243, 2256, 2271, 2272, 2287, 2288, 2295, 2309, 2313, 2344, 2345, 2346, 2348, 2364, 2371, 2402, 2414, 2417, 2426, 2433, 2437, 2443, 2444, 2447, 2458, 2464, 2479, 2486, 2487, 2492, 2494, 2501, 2515, 2518, 2533, 2539, 2545, 2555, 2560, 2564, 2568, 2570, 2573, 2576, 2580, 2581, 2597, 2599, 2602, 2608, 2611, 2613, 2616, 2621, 2634, 2665, 2668, 2678, 2690, 2692, 2699, 2703, 2706, 2707, 2710, 2725, 2730, 2736, 2748, 2756, 2772, 2782, 2785, 2786, 2790, 2809, 2835, 2836, 2842, 2850, 2858, 2861, 2866, 2868, 2872, 2873, 2875, 2878, 2882, 2893, 2896, 2903, 2909, 2915, 2931, 2947, 2951, 2957, 2960, 2961, 2964, 2968, 2972, 2985, 2986, 2997, 3000, 3017, 3022, 3030, 3039, 3050, 3055, 3068, 3071, 3087, 3093, 3095, 3107, 3109, 3112, 3126, 3127, 3132, 3138, 3159, 3168, 3207, 3208, 3212, 3228, 3236, 3238, 3241, 3247, 3255, 3258, 3287, 3298, 3300, 3302, 3321, 3326, 3339, 3352, 3359, 3375, 3380, 3397, 3401, 3404, 3417, 3427, 3433, 3462, 3469, 3471, 3485, 3487, 3496, 3516, 3518, 3519, 3521, 3529, 3530, 3557, 3559, 3562, 3609, 3610, 3613, 3619, 3633, 3642, 3662, 3664, 3665, 3682, 3698, 3702, 3703, 3721, 3731, 3735, 3740, 3743, 3754, 3769, 3812, 3833, 3834, 3840, 3842, 3846, 3849, 3857, 3882, 3885, 3887, 3896, 3914, 3915, 3918, 3920, 3925, 3934, 3953, 3961, 3962, 3966, 3967, 3968, 3973, 3979, 4021, 4023, 4036, 4041, 4048, 4050, 4058, 4061, 4065, 4092, 4094, 4115, 4118, 4126, 4133, 4138, 4139, 4141, 4142, 4149, 4152, 4156, 4170, 4180, 4210, 4216, 4222, 4225, 4234, 4240, 4278, 4291, 4292, 4293, 4301, 4308, 4320, 4327, 4328, 4334, 4342, 4345, 4355, 4361, 4370, 4382, 4385, 4393, 4394, 4400, 4402, 4408, 4411, 4450, 4456, 4458, 4476, 4505, 4506, 4507, 4524, 4531, 4541, 4550, 4551, 4561, 4569, 4580, 4582, 4586, 4592, 4597, 4599, 4602, 4617, 4634, 4646, 4650, 4653, 4656, 4665, 4668, 4677, 4697, 4714, 4717, 4722, 4727, 4734, 4749, 4761, 4763, 4768, 4779, 4787, 4802, 4805, 4809, 4825, 4844, 4849, 4888, 4907, 4929, 4931, 4932, 4937, 4942, 4952, 4959, 4971, 5007, 5030, 5032, 5035, 5039, 5046, 5050, 5066, 5072, 5075, 5079, 5134, 5148, 5149, 5165, 205, 534, 539, 611, 809, 1519, 1954, 2270, 2898, 3190, 3604, 4137, 4329, 4520, 5151, 314, 457, 566, 912, 1030, 1181, 1409, 1459, 1467, 1630, 1797, 1967, 2084, 2099, 2164, 2207, 2239, 2364, 2433, 2483, 2495, 2665, 2765, 2941, 2945, 3061, 3088, 3132, 3192, 3199, 3352, 3807, 3824, 3867, 4034, 4193, 4201, 4498, 4741, 4773, 4805, 5126, 1, 58, 210, 281, 554, 610, 764, 979, 1012, 1185, 1194, 1383, 1517, 1528, 1541, 1620, 1774, 1980, 2178, 2221, 2226, 2369, 2538, 2583, 2614, 2737, 2768, 2770, 2847, 3063, 3088, 3354, 3498, 3564, 3625, 3638, 3867, 3952, 3972, 4536, 4803, 4852, 5008, 0, 14, 17, 18, 24, 29, 54, 56, 58, 64, 70, 83, 136, 161, 180, 186, 188, 200, 216, 237, 251, 256, 257, 277, 278, 280, 281, 321, 334, 346, 352, 354, 379, 439, 478, 485, 520, 524, 529, 530, 566, 606, 611, 621, 624, 638, 650, 668, 670, 704, 712, 723, 771, 834, 848, 890, 919, 938, 966, 1007, 1010, 1029, 1060, 1063, 1065, 1070, 1078, 1081, 1085, 1093, 1109, 1160, 1185, 1208, 1214, 1223, 1242, 1261, 1262, 1263, 1269, 1272, 1274, 1312, 1333, 1350, 1351, 1352, 1366, 1374, 1378, 1383, 1390, 1398, 1439, 1441, 1449, 1463, 1467, 1480, 1482, 1492, 1517, 1527, 1572, 1601, 1652, 1660, 1682, 1687, 1702, 1720, 1728, 1768, 1777, 1790, 1791, 1801, 1826, 1827, 1828, 1834, 1847, 1850, 1858, 1861, 1863, 1870, 1877, 1885, 1889, 1897, 1910, 1915, 1922, 1929, 1951, 1971, 2048, 2059, 2062, 2108, 2123, 2190, 2227, 2235, 2244, 2250, 2255, 2274, 2281, 2350, 2352, 2368, 2373, 2376, 2387, 2391, 2394, 2404, 2413, 2458, 2459, 2477, 2483, 2487, 2488, 2545, 2547, 2568, 2570, 2589, 2616, 2627, 2631, 2654, 2669, 2672, 2700, 2702, 2703, 2704, 2718, 2731, 2747, 2775, 2789, 2818, 2845, 2855, 2865, 2874, 2881, 2930, 2949, 2952, 2967, 2988, 3006, 3014, 3029, 3030, 3055, 3063, 3064, 3089, 3098, 3120, 3126, 3127, 3130, 3154, 3166, 3176, 3178, 3197, 3257, 3292, 3299, 3309, 3345, 3354, 3387, 3389, 3390, 3392, 3401, 3431, 3435, 3439, 3472, 3487, 3531, 3534, 3555, 3559, 3568, 3598, 3603, 3611, 3645, 3674, 3683, 3687, 3695, 3699, 3705, 3708, 3727, 3730, 3762, 3786, 3787, 3812, 3824, 3831, 3832, 3875, 3876, 3885, 3909, 3918, 3932, 3933, 3946, 3959, 3972, 3985, 4029, 4034, 4061, 4068, 4076, 4080, 4081, 4113, 4117, 4128, 4144, 4156, 4176, 4202, 4228, 4229, 4274, 4279, 4290, 4293, 4303, 4306, 4315, 4332, 4360, 4365, 4371, 4375, 4392, 4420, 4424, 4440, 4442, 4476, 4506, 4535, 4566, 4569, 4586, 4589, 4593, 4606, 4607, 4610, 4613, 4619, 4623, 4626, 4629, 4633, 4645, 4650, 4688, 4704, 4717, 4721, 4737, 4745, 4755, 4776, 4777, 4779, 4782, 4785, 4790, 4810, 4814, 4816, 4825, 4842, 4853, 4863, 4874, 4878, 4903, 4904, 4929, 4935, 4940, 4947, 4955, 4964, 4984, 5006, 5017, 5027, 5034, 5038, 5039, 5058, 5063, 5081, 5098, 5132, 5140, 5157, 5164, 5166, 5169, 42, 60, 122, 180, 189, 320, 329, 357, 410, 455, 506, 514, 517, 557, 582, 615, 637, 752, 753, 800, 808, 898, 944, 983, 1139, 1189, 1204, 1213, 1274, 1370, 1375, 1387, 1393, 1438, 1505, 1601, 1695, 1699, 1745, 1759, 1773, 1814, 1886, 1971, 2082, 2088, 2092, 2150, 2203, 2221, 2272, 2296, 2359, 2415, 2487, 2500, 2543, 2587, 2693, 2716, 2777, 2806, 2844, 2857, 2885, 2890, 2994, 3004, 3010, 3012, 3025, 3026, 3038, 3059, 3113, 3125, 3280, 3302, 3340, 3377, 3386, 3423, 3441, 3474, 3517, 3572, 3596, 3610, 3663, 3726, 3750, 3761, 3780, 3795, 3796, 3809, 3832, 3843, 3864, 3891, 3915, 3969, 3989, 4048, 4129, 4138, 4151, 4215, 4251, 4302, 4327, 4349, 4404, 4424, 4460, 4497, 4570, 4576, 4579, 4589, 4607, 4667, 4723, 4763, 4768, 4779, 4786, 4862, 5023, 5047, 5079, 5083, 5167, 0, 19, 37, 56, 59, 86, 90, 92, 98, 117, 118, 119, 131, 136, 141, 164, 167, 173, 187, 189, 190, 202, 214, 217, 227, 236, 249, 256, 263, 286, 287, 289, 291, 307, 308, 324, 326, 332, 334, 336, 347, 363, 371, 382, 389, 402, 409, 411, 425, 434, 440, 482, 507, 512, 517, 535, 561, 566, 567, 572, 577, 580, 581, 582, 597, 599, 608, 637, 642, 650, 656, 691, 692, 694, 698, 700, 703, 721, 729, 732, 743, 751, 754, 762, 777, 781, 787, 790, 831, 840, 873, 874, 877, 888, 889, 904, 905, 906, 908, 911, 923, 932, 938, 942, 944, 946, 954, 968, 976, 989, 1001, 1003, 1007, 1011, 1016, 1018, 1030, 1050, 1053, 1057, 1083, 1101, 1110, 1157, 1161, 1162, 1163, 1168, 1187, 1202, 1212, 1220, 1240, 1246, 1249, 1262, 1276, 1298, 1301, 1302, 1331, 1354, 1384, 1389, 1428, 1442, 1444, 1447, 1452, 1455, 1459, 1460, 1463, 1465, 1476, 1499, 1512, 1514, 1518, 1522, 1529, 1534, 1560, 1595, 1597, 1604, 1605, 1628, 1636, 1641, 1643, 1651, 1677, 1681, 1697, 1700, 1719, 1726, 1748, 1764, 1787, 1808, 1810, 1819, 1822, 1848, 1854, 1896, 1897, 1902, 1903, 1905, 1906, 1911, 1919, 1922, 1923, 1938, 1947, 1968, 1973, 1975, 1980, 1981, 1984, 1987, 1990, 1993, 2003, 2020, 2029, 2030, 2031, 2039, 2077, 2089, 2095, 2097, 2106, 2112, 2113, 2117, 2121, 2133, 2139, 2148, 2159, 2165, 2167, 2178, 2192, 2196, 2213, 2231, 2241, 2243, 2251, 2255, 2260, 2261, 2283, 2298, 2315, 2319, 2321, 2328, 2332, 2337, 2341, 2353, 2365, 2374, 2397, 2403, 2404, 2412, 2424, 2433, 2450, 2460, 2471, 2476, 2483, 2491, 2502, 2503, 2505, 2515, 2520, 2532, 2563, 2568, 2572, 2591, 2597, 2602, 2614, 2616, 2617, 2627, 2628, 2636, 2640, 2649, 2685, 2690, 2693, 2753, 2759, 2766, 2771, 2789, 2814, 2820, 2841, 2861, 2863, 2871, 2881, 2888, 2897, 2902, 2903, 2911, 2928, 2935, 2956, 2</t>
   </si>
   <si>
     <t>259.78999999999996</t>
@@ -535,13 +535,13 @@
     <t>MU12_6, MU12_10, MU12_13, MU12_16, MU12_20, MU12_21, MU12_29, MU12_38, MU12_43, MU12_45, MU12_46, MU12_49, MU12_68, MU12_74, MU12_75, MU12_76, MU12_77, MU12_88, MU12_94, MU12_99, MU12_102, MU12_114, MU12_119, MU12_120, MU12_122, MU12_131, MU12_136, MU12_140, MU12_144, MU12_145, MU12_152, MU12_166, MU12_176, MU12_195, MU12_197, MU12_213, MU12_230, MU12_231, MU12_237, MU12_244, MU12_245, MU12_320, MU12_323, MU12_357, MU12_404, MU12_431, MU17_6, MU17_10, MU17_13, MU17_16, MU17_20, MU17_21, MU17_29, MU17_38, MU17_43, MU17_45, MU17_46, MU17_49, MU17_68, MU17_74, MU17_75, MU17_76, MU17_77, MU17_88, MU17_94, MU17_99, MU17_102, MU17_114, MU17_119, MU17_120, MU17_122, MU17_131, MU17_136, MU17_140, MU17_144, MU17_145, MU17_152, MU17_166, MU17_176, MU17_195, MU17_197, MU17_213, MU17_230, MU17_231, MU17_237, MU17_244, MU17_245, MU17_320, MU17_323, MU17_357, MU17_404, MU17_431</t>
   </si>
   <si>
-    <t>33.769999999999996</t>
-  </si>
-  <si>
-    <t>1747</t>
-  </si>
-  <si>
-    <t>172, 238, 264, 272, 314, 457, 579, 657, 746, 847, 1121, 1319, 1432, 1650, 1972, 2237, 2337, 2340, 2590, 2599, 2987, 3251, 3530, 3703, 3818, 4033, 4097, 4136, 4234, 4394, 4396, 4484, 4651, 4655, 4724, 4755, 12, 22, 50, 51, 57, 106, 112, 125, 149, 178, 188, 200, 206, 223, 226, 247, 275, 290, 300, 305, 316, 320, 370, 432, 436, 442, 461, 472, 489, 498, 520, 534, 544, 562, 599, 611, 656, 664, 678, 698, 731, 740, 747, 783, 803, 869, 876, 877, 879, 888, 935, 945, 954, 964, 969, 987, 1003, 1029, 1034, 1035, 1038, 1057, 1068, 1080, 1089, 1094, 1116, 1125, 1128, 1136, 1165, 1190, 1191, 1207, 1249, 1254, 1341, 1363, 1367, 1373, 1432, 1443, 1450, 1460, 1474, 1488, 1518, 1538, 1543, 1562, 1563, 1574, 1585, 1589, 1592, 1598, 1600, 1677, 1679, 1682, 1695, 1705, 1719, 1725, 1743, 1793, 1818, 1819, 1822, 1833, 1869, 1877, 1903, 1931, 1937, 1939, 2016, 2085, 2137, 2195, 2244, 2271, 2306, 2311, 2335, 2346, 2350, 2361, 2368, 2395, 2446, 2449, 2453, 2458, 2485, 2491, 2523, 2558, 2599, 2609, 2626, 2629, 2660, 2665, 2694, 2715, 2744, 2772, 2776, 2779, 2787, 2806, 2827, 2833, 2842, 2845, 2862, 2899, 2978, 3026, 3063, 3091, 3102, 3117, 3133, 3155, 3226, 3299, 3306, 3310, 3324, 3328, 3333, 3334, 3359, 3390, 3394, 3395, 3403, 3432, 3439, 3467, 3508, 3530, 3539, 3542, 3543, 3555, 3561, 3578, 3588, 3615, 3620, 3627, 3628, 3641, 3659, 3667, 3698, 3703, 3705, 3721, 3738, 3883, 3901, 3925, 3953, 3979, 3980, 4004, 4021, 4087, 4104, 4105, 4175, 4179, 4207, 4216, 4266, 4272, 4297, 4313, 4350, 4384, 4389, 4396, 4438, 4486, 4507, 4511, 4519, 4534, 4551, 4565, 4649, 4675, 4681, 4717, 4718, 4732, 4747, 4778, 4842, 4861, 4872, 4937, 4947, 4987, 4997, 5022, 5029, 5054, 5058, 5061, 5103, 5150, 5157, 717, 3440, 3486, 3653, 57, 70, 200, 581, 1338, 1526, 1761, 1772, 1903, 2175, 2291, 2410, 2842, 3155, 3286, 3361, 3670, 3677, 3691, 3890, 4111, 4318, 4443, 4542, 4624, 4833, 5093, 1272, 357, 471, 675, 690, 828, 1288, 1295, 1327, 1350, 1673, 1930, 2205, 2244, 2282, 2442, 2617, 2960, 3106, 3361, 3606, 3812, 3844, 4080, 4174, 4529, 4606, 4664, 4718, 5043, 4718, 230, 446, 690, 747, 942, 1135, 1185, 2124, 2309, 2310, 2447, 2895, 3439, 4304, 4389, 4526, 130, 234, 397, 514, 1066, 1106, 1168, 1361, 1402, 1577, 1590, 1938, 1992, 2011, 2244, 2282, 2777, 2960, 2995, 3480, 3503, 3746, 4017, 4029, 4174, 4216, 4306, 4526, 4554, 4945, 5162, 219, 489, 597, 709, 1256, 1407, 1557, 1694, 2632, 2710, 2899, 3501, 4087, 4314, 4784, 4902, 150, 1518, 1536, 1952, 2470, 3689, 3851, 3869, 4247, 417, 446, 893, 915, 1066, 1402, 1614, 1687, 1930, 1938, 2011, 2125, 2198, 2442, 2662, 2680, 3181, 3338, 3818, 4029, 4306, 4308, 4439, 4551, 4554, 4596, 5111, 513, 717, 747, 923, 1011, 1098, 1145, 1265, 2065, 2710, 2987, 2992, 3063, 3323, 3845, 4389, 4562, 4570, 1288, 1465, 1518, 3414, 3503, 3583, 4171, 4316, 204, 332, 661, 700, 911, 953, 1224, 1459, 1527, 1889, 2035, 2099, 2260, 2298, 2405, 2553, 3153, 3316, 3539, 3581, 3788, 4080, 4207, 5150, 23, 353, 579, 711, 775, 935, 981, 985, 1140, 1257, 1510, 1536, 1592, 1610, 1683, 1931, 1965, 2035, 2164, 2244, 2378, 2405, 2667, 2883, 3324, 3395, 3401, 3415, 3464, 3469, 3567, 3621, 3629, 3647, 3653, 3693, 3716, 3922, 4146, 4351, 4423, 4603, 4712, 4717, 4727, 5066, 5078, 5112, 78, 411, 446, 528, 854, 1066, 1225, 2011, 2034, 2656, 2977, 3177, 3181, 3206, 4423, 4852, 125, 403, 500, 557, 597, 605, 667, 720, 864, 893, 993, 1014, 1165, 1178, 1340, 1370, 1614, 1664, 1929, 1948, 2009, 2238, 2255, 2257, 2311, 2407, 2576, 2645, 2735, 2772, 2875, 2943, 3046, 3063, 3090, 3134, 3224, 3252, 3431, 3502, 3517, 3654, 3661, 3791, 4130, 4374, 4454, 4487, 4495, 4598, 4675, 4960, 4994, 5028, 5056, 5123, 5169, 78, 209, 294, 392, 603, 686, 746, 1033, 1161, 1174, 1195, 1282, 1291, 1338, 1444, 1460, 1654, 1963, 1992, 2029, 2084, 2436, 2600, 2628, 2763, 2963, 3071, 3266, 3352, 3503, 3564, 3703, 3716, 3917, 4004, 4132, 4147, 4155, 4350, 4434, 4598, 4770, 4782, 4828, 4853, 4893, 4960, 4963, 307, 746, 758, 853, 965, 1482, 1510, 1577, 1722, 1901, 1965, 2006, 2442, 2703, 2947, 3049, 3314, 3338, 3363, 3464, 3567, 3779, 4068, 4445, 4463, 4591, 4795, 4861, 56, 969, 1538, 1639, 2346, 2442, 3063, 3177, 3286, 3885, 5111, 294, 706, 2583, 3693, 5151, 534, 1113, 1282, 2338, 2346, 2517, 2987, 3342, 3722, 3885, 3890, 4234, 1647, 3082, 3310, 51, 77, 314, 606, 926, 1817, 1822, 1827, 1960, 2198, 2865, 3156, 3517, 3634, 4029, 4306, 4918, 4967, 506, 880, 913, 950, 1159, 1502, 2161, 2512, 3147, 3406, 3644, 4097, 4494, 4839, 4923, 5013, 5042, 23, 3146, 3296, 3693, 3883, 4779, 4923, 5099, 19, 32, 56, 283, 328, 363, 446, 520, 606, 632, 699, 717, 720, 761, 778, 802, 813, 885, 918, 921, 931, 973, 1002, 1049, 1117, 1128, 1192, 1287, 1315, 1338, 1344, 1468, 1478, 1542, 1572, 1573, 1604, 1611, 1614, 1622, 1632, 1682, 1695, 1939, 1972, 2018, 2069, 2183, 2199, 2283, 2449, 2455, 2479, 2558, 2621, 2636, 2664, 2703, 2776, 2793, 2845, 2995, 3028, 3031, 3214, 3243, 3338, 3384, 3415, 3440, 3472, 3526, 3562, 3620, 3662, 3677, 3716, 3770, 3890, 3902, 3903, 3937, 4049, 4139, 4248, 4263, 4314, 4400, 4533, 4555, 4651, 4678, 4757, 4759, 4781, 4811, 4823, 5097, 5162, 307, 807, 1002, 1181, 1364, 1482, 1667, 1802, 2442, 2458, 2903, 3338, 3779, 3869, 4093, 4591, 4643, 4937, 4981, 77, 108, 267, 667, 743, 753, 812, 893, 945, 1048, 1080, 1431, 1828, 1851, 1884, 1952, 2144, 2201, 2350, 2462, 2555, 2706, 2720, 2767, 3090, 3096, 3159, 3344, 3457, 3631, 3703, 3705, 4024, 4097, 4454, 4578, 4611, 4741, 4853, 429, 2282, 2579, 2671, 2699, 2995, 3336, 3626, 4077, 4287, 4299, 4324, 4598, 4764, 143, 161, 219, 487, 567, 595, 643, 707, 709, 737, 747, 783, 990, 1034, 1128, 1169, 1288, 1737, 1936, 1938, 2115, 2198, 2205, 2410, 2814, 3031, 3431, 3432, 3434, 3503, 3552, 3572, 3582, 3705, 3801, 3818, 3838, 3864, 4033, 4389, 4660, 4942, 4991, 5140, 5144, 12, 77, 262, 518, 664, 724, 971, 1098, 1256, 1723, 2381, 2495, 2597, 3175, 3203, 3563, 3581, 3603, 3991, 4126, 4168, 4531, 4596, 5105, 18, 164, 404, 562, 1079, 1315, 2085, 2093, 2239, 2260, 3394, 3439, 3, 77, 169, 182, 237, 328, 470, 491, 570, 579, 588, 605, 639, 747, 761, 858, 877, 924, 926, 944, 977, 1064, 1192, 1224, 1455, 1523, 1694, 1822, 2018, 2023, 2097, 2362, 2464, 2770, 2790, 2878, 2948, 3004, 3048, 3074, 3082, 3167, 3258, 3457, 3555, 3603, 3634, 3637, 3883, 3932, 4199, 4245, 4365, 4396, 4446, 4554, 4568, 4598, 4779, 4856, 5029, 5105, 5163, 77, 173, 561, 636, 746, 885, 1482, 1687, 1795, 1906, 1930, 1931, 2590, 2722, 3084, 3372, 3395, 3446, 3779, 4351, 4551, 143, 278, 470, 531, 748, 753, 791, 1229, 1368, 1389, 1395, 1558, 1585, 1952, 2163, 2192, 2370, 2562, 2694, 2710, 2772, 3167, 3384, 3431, 3480, 3601, 3972, 4187, 4308, 4475, 4660, 4699, 5150, 5111, 1266, 1639, 2974, 4289, 1358, 1648, 1683, 1797, 2338, 2451, 2633, 2669, 2978, 3376, 3418, 3610, 3991, 4294, 4665, 5040, 5169, 174, 178, 389, 471, 517, 775, 882, 988, 1032, 1134, 1225, 1339, 1574, 1600, 1610, 1692, 2130, 2257, 2362, 2370, 2376, 2592, 3003, 3117, 3314, 3738, 3782, 3843, 4115, 4652, 4700, 4832, 4997, 5018, 335, 481, 595, 601, 778, 885, 917, 1117, 1144, 1251, 1427, 1811, 1827, 1846, 2604, 2646, 2667, 2753, 2779, 2815, 3356, 3528, 4095, 4248, 4928, 4960, 5043, 77, 322, 497, 636, 885, 1327, 1737, 1858, 1877, 1906, 1931, 2008, 2015, 2590, 2748, 3067, 3779, 3908, 4727, 112, 125, 367, 420, 511, 1138, 1239, 1455, 1497, 1522, 1542, 1563, 1814, 2097, 2626, 2746, 3005, 3140, 3406, 3480, 3495, 3844, 3972, 4155, 4230, 4852, 4906, 4913, 4923, 4968, 206, 223, 446, 1174, 1258, 1567, 1573, 1604, 1685, 1695, 2257, 2301, 2449, 2636, 2664, 2883, 2885, 3017, 3214, 3961, 4096, 4139, 4304, 4355, 4443, 4828, 4949, 5061, 370, 485, 797, 981, 1328, 2122, 2640, 2642, 2883, 3131, 3481, 3552, 3564, 3844, 4853, 4861, 5101, 10, 18, 40, 55, 91, 160, 164, 181, 196, 211, 227, 332, 334, 407, 414, 482, 533, 595, 675, 734, 739, 799, 803, 807, 815, 910, 971, 983, 994, 1089, 1128, 1134, 1170, 1202, 1256, 1292, 1320, 1330, 1340, 1452, 1462, 1526, 1558, 1610, 1627, 1660, 1787, 1818, 1861, 1932, 1936, 1963, 1972, 1986, 1987, 2048, 2049, 2054, 2056, 2130, 2137, 2160, 2201, 2294, 2308, 2338, 2396, 2410, 2458, 2467, 2485, 2532, 2574, 2589, 2753, 2754, 2774, 2917, 3006, 3120, 3134, 3234, 3238, 3239, 3288, 3355, 3361, 3365, 3368, 3394, 3406, 3418, 3439, 3452, 3558, 3569, 3597, 3628, 3631, 3644, 3698, 3767, 3902, 3907, 3937, 3996, 4097, 4110, 4139, 4147, 4174, 4219, 4262, 4281, 4311, 4333, 4408, 4445, 4507, 4568, 4624, 4625, 4665, 4677, 4678, 4717, 4833, 4859, 4867, 4911, 4947, 4981, 5079, 5135, 147, 1027, 2216, 3063, 4440, 4724, 4782, 11, 57, 63, 75, 77, 82, 83, 173, 192, 193, 209, 213, 270, 272, 297, 316, 319, 328, 332, 391, 418, 436, 474, 510, 562, 572, 584, 593, 628, 641, 653, 656, 690, 704, 725, 740, 743, 781, 807, 839, 847, 854, 869, 871, 888, 910, 945, 951, 989, 1027, 1049, 1084, 1134, 1136, 1144, 1157, 1170, 1179, 1225, 1258, 1309, 1314, 1321, 1361, 1369, 1449, 1465, 1501, 1519, 1545, 1563, 1573, 1577, 1616, 1677, 1726, 1758, 1772, 1786, 1792, 1796, 1818, 1827, 1854, 1864, 1869, 1904, 1909, 1952, 2006, 2018, 2045, 2066, 2110, 2134, 2137, 2148, 2175, 2180, 2283, 2291, 2310, 2350, 2352, 2368, 2407, 2472, 2482, 2507, 2511, 2517, 2523, 2535, 2552, 2565, 2585, 2646, 2661, 2667, 2688, 2699, 2705, 2706, 2758, 2779, 2806, 2813, 2817, 2866, 2869, 2874, 2933, 2945, 2947, 2978, 2983, 3002, 3004, 3017, 3031, 3039, 3048, 3057, 3085, 3093, 3134, 3141, 3143, 3148, 3170, 3177, 3186, 3245, 3266, 3328, 3352, 3356, 3357, 3361, 3386, 3406, 3434, 3457, 3491, 3502, 3529, 3553, 3564, 3640, 3643, 3648, 3653, 3664, 3709, 3739, 3745, 3801, 3803, 3808, 3837, 3855, 3865, 3890, 3896, 3904, 3908, 3910, 3917, 3953, 4002, 4068, 4171, 4181, 4195, 4247, 4274, 4304, 4306, 4314, 4316, 4331, 4440, 4450, 4463, 4478, 4571, 4606, 4613, 4649, 4665, 4739, 4777, 4778, 4784, 4799, 4823, 4841, 4849, 4876, 4906, 4928, 4947, 4964, 4981, 5022, 5046, 5077, 5133, 5143, 77, 446, 482, 497, 504, 561, 636, 734, 1082, 1261, 1280, 1376, 1687, 1876, 1930, 1931, 2065, 2125, 2198, 3047, 3063, 3395, 3441, 3446, 3472, 3678, 3908, 4351, 4664, 4809, 4841, 5035, 114, 475, 1198, 2705, 3112, 3154, 3247, 3494, 4190, 4374, 4574, 4707, 5054, 262, 482, 834, 1382, 1429, 2442, 2555, 3196, 3423, 3446, 4663</t>
+    <t>33.790000000000006</t>
+  </si>
+  <si>
+    <t>1748</t>
+  </si>
+  <si>
+    <t>172, 238, 264, 272, 314, 457, 579, 657, 746, 847, 1121, 1319, 1432, 1650, 1972, 2237, 2337, 2340, 2590, 2599, 2987, 3251, 3530, 3703, 3818, 4033, 4097, 4136, 4234, 4394, 4396, 4484, 4651, 4655, 4724, 4755, 12, 22, 50, 51, 57, 106, 112, 125, 149, 178, 188, 200, 206, 223, 226, 247, 275, 290, 300, 305, 316, 320, 370, 432, 436, 442, 461, 472, 489, 498, 520, 534, 544, 562, 599, 611, 656, 664, 678, 698, 731, 740, 747, 783, 803, 869, 876, 877, 879, 888, 935, 945, 954, 964, 969, 987, 1003, 1029, 1034, 1035, 1038, 1057, 1068, 1080, 1089, 1094, 1116, 1125, 1128, 1136, 1165, 1190, 1191, 1207, 1249, 1254, 1341, 1363, 1367, 1373, 1432, 1443, 1450, 1460, 1474, 1488, 1518, 1538, 1543, 1562, 1563, 1574, 1585, 1589, 1592, 1598, 1600, 1677, 1679, 1682, 1695, 1705, 1719, 1725, 1743, 1793, 1818, 1819, 1822, 1833, 1869, 1877, 1903, 1931, 1937, 1939, 2016, 2085, 2137, 2195, 2244, 2271, 2306, 2311, 2335, 2346, 2350, 2361, 2368, 2395, 2446, 2449, 2453, 2458, 2485, 2491, 2523, 2558, 2599, 2609, 2626, 2629, 2660, 2665, 2694, 2715, 2744, 2772, 2776, 2779, 2787, 2806, 2827, 2833, 2842, 2845, 2862, 2899, 2978, 3026, 3063, 3091, 3102, 3117, 3133, 3155, 3226, 3299, 3306, 3310, 3324, 3328, 3333, 3334, 3359, 3390, 3394, 3395, 3403, 3432, 3439, 3467, 3508, 3530, 3539, 3542, 3543, 3555, 3561, 3578, 3588, 3615, 3620, 3627, 3628, 3641, 3659, 3667, 3698, 3703, 3705, 3721, 3738, 3883, 3901, 3925, 3953, 3979, 3980, 4004, 4021, 4087, 4104, 4105, 4175, 4179, 4207, 4216, 4266, 4272, 4297, 4313, 4350, 4384, 4389, 4396, 4438, 4486, 4507, 4511, 4519, 4534, 4551, 4565, 4649, 4675, 4681, 4717, 4718, 4732, 4747, 4778, 4842, 4861, 4872, 4937, 4947, 4987, 4997, 5022, 5029, 5054, 5058, 5061, 5103, 5150, 5157, 717, 3440, 3486, 3653, 57, 70, 200, 581, 1272, 1338, 1526, 1761, 1772, 1903, 2175, 2291, 2410, 2842, 3155, 3286, 3361, 3670, 3677, 3691, 3890, 4111, 4318, 4443, 4542, 4624, 4833, 5093, 357, 471, 675, 690, 828, 1288, 1295, 1327, 1350, 1673, 1930, 2205, 2244, 2282, 2442, 2617, 2960, 3106, 3361, 3606, 3812, 3844, 4080, 4174, 4529, 4606, 4664, 4718, 5043, 230, 446, 690, 747, 942, 1135, 1185, 2124, 2309, 2310, 2447, 2895, 3439, 4304, 4389, 4526, 4718, 130, 234, 397, 514, 1066, 1106, 1168, 1361, 1402, 1577, 1590, 1938, 1992, 2011, 2244, 2282, 2777, 2960, 2995, 3480, 3503, 3746, 4017, 4029, 4174, 4216, 4306, 4526, 4554, 4945, 5162, 219, 489, 597, 709, 1256, 1407, 1557, 1694, 2632, 2710, 2899, 3501, 4087, 4314, 4784, 4902, 150, 1518, 1536, 1952, 2470, 3689, 3851, 3869, 4247, 417, 446, 893, 915, 1066, 1402, 1614, 1687, 1930, 1938, 2011, 2125, 2198, 2442, 2662, 2680, 3181, 3338, 3818, 4029, 4306, 4308, 4439, 4551, 4554, 4596, 5111, 513, 717, 747, 923, 1011, 1098, 1145, 1265, 1288, 1465, 1518, 2065, 2710, 2987, 2992, 3063, 3323, 3414, 3503, 3583, 3845, 4171, 4316, 4389, 4562, 4570, 204, 332, 661, 700, 911, 953, 1224, 1459, 1527, 1889, 2035, 2099, 2260, 2298, 2405, 2553, 3153, 3316, 3539, 3581, 3788, 4080, 4207, 5150, 23, 353, 579, 711, 775, 935, 981, 985, 1140, 1257, 1510, 1536, 1592, 1610, 1683, 1931, 1965, 2035, 2164, 2244, 2378, 2405, 2667, 2883, 3324, 3395, 3401, 3415, 3464, 3469, 3567, 3621, 3629, 3647, 3653, 3693, 3716, 3922, 4146, 4351, 4423, 4603, 4712, 4717, 4727, 5066, 5078, 5112, 78, 411, 446, 528, 854, 1066, 1225, 2011, 2034, 2656, 2977, 3177, 3181, 3206, 4423, 4852, 125, 403, 500, 557, 597, 605, 667, 720, 864, 893, 993, 1014, 1165, 1178, 1340, 1370, 1614, 1664, 1929, 1948, 2009, 2238, 2255, 2257, 2311, 2407, 2576, 2645, 2735, 2772, 2875, 2943, 3046, 3063, 3090, 3134, 3224, 3252, 3431, 3502, 3517, 3654, 3661, 3791, 4130, 4374, 4454, 4487, 4495, 4598, 4675, 4960, 4994, 5028, 5056, 5123, 5169, 78, 209, 294, 392, 603, 686, 746, 1033, 1161, 1174, 1195, 1282, 1291, 1338, 1444, 1460, 1654, 1963, 1992, 2029, 2084, 2436, 2600, 2628, 2763, 2963, 3071, 3266, 3352, 3503, 3564, 3703, 3716, 3917, 4004, 4132, 4147, 4155, 4350, 4434, 4598, 4770, 4782, 4828, 4853, 4893, 4960, 4963, 307, 746, 758, 853, 965, 1482, 1510, 1577, 1722, 1901, 1965, 2006, 2442, 2703, 2947, 3049, 3314, 3338, 3363, 3464, 3567, 3779, 4068, 4445, 4463, 4591, 4795, 4861, 56, 294, 706, 969, 1538, 1639, 2346, 2442, 2583, 3063, 3177, 3286, 3693, 3885, 5111, 5151, 534, 1113, 1282, 1647, 2338, 2346, 2517, 2987, 3082, 3310, 3342, 3722, 3885, 3890, 4234, 51, 77, 314, 606, 926, 1817, 1822, 1827, 1960, 2198, 2865, 3156, 3517, 3634, 4029, 4306, 4918, 4967, 506, 880, 913, 950, 1159, 1502, 2161, 2512, 3147, 3406, 3644, 4097, 4494, 4839, 4923, 5013, 5042, 23, 3146, 3296, 3693, 3883, 4779, 4923, 5099, 19, 32, 56, 283, 328, 363, 446, 520, 606, 632, 699, 717, 720, 761, 778, 802, 813, 885, 918, 921, 931, 973, 1002, 1049, 1117, 1128, 1192, 1287, 1315, 1338, 1344, 1468, 1478, 1542, 1572, 1573, 1604, 1611, 1614, 1622, 1632, 1682, 1695, 1939, 1972, 2018, 2069, 2183, 2199, 2283, 2449, 2455, 2479, 2558, 2621, 2636, 2664, 2703, 2776, 2793, 2845, 2995, 3028, 3031, 3214, 3243, 3338, 3384, 3415, 3440, 3472, 3526, 3562, 3620, 3662, 3677, 3716, 3770, 3890, 3902, 3903, 3937, 4049, 4139, 4248, 4263, 4314, 4400, 4533, 4555, 4651, 4678, 4757, 4759, 4781, 4811, 4823, 5097, 5162, 307, 807, 1002, 1181, 1364, 1482, 1667, 1802, 2442, 2458, 2903, 3338, 3779, 3869, 4093, 4591, 4643, 4937, 4981, 77, 108, 267, 667, 743, 753, 812, 893, 945, 1048, 1080, 1431, 1828, 1851, 1884, 1952, 2144, 2201, 2350, 2462, 2555, 2706, 2720, 2767, 3090, 3096, 3159, 3344, 3457, 3631, 3703, 3705, 4024, 4097, 4454, 4578, 4611, 4741, 4853, 429, 2282, 2579, 2671, 2699, 2995, 3336, 3626, 4077, 4287, 4299, 4324, 4598, 4764, 143, 161, 219, 487, 567, 595, 643, 707, 709, 737, 747, 783, 990, 1034, 1128, 1169, 1288, 1737, 1936, 1938, 2115, 2198, 2205, 2410, 2814, 3031, 3431, 3432, 3434, 3503, 3552, 3572, 3582, 3705, 3801, 3818, 3838, 3864, 4033, 4389, 4660, 4942, 4991, 5140, 5144, 12, 77, 262, 518, 664, 724, 971, 1098, 1256, 1723, 2381, 2495, 2597, 3175, 3203, 3563, 3581, 3603, 3991, 4126, 4168, 4531, 4596, 5105, 18, 164, 404, 562, 1079, 1315, 2085, 2093, 2239, 2260, 3394, 3439, 3, 77, 169, 182, 237, 328, 470, 491, 570, 579, 588, 605, 639, 747, 761, 858, 877, 924, 926, 944, 977, 1064, 1192, 1224, 1455, 1523, 1694, 1822, 2018, 2023, 2097, 2362, 2464, 2770, 2790, 2878, 2948, 3004, 3048, 3074, 3082, 3167, 3258, 3457, 3555, 3603, 3634, 3637, 3883, 3932, 4199, 4245, 4365, 4396, 4446, 4554, 4568, 4598, 4779, 4856, 5029, 5105, 5163, 77, 173, 561, 636, 746, 885, 1482, 1687, 1795, 1906, 1930, 1931, 2590, 2722, 3084, 3372, 3395, 3446, 3779, 4351, 4551, 143, 278, 470, 531, 748, 753, 791, 1229, 1368, 1389, 1395, 1558, 1585, 1952, 2163, 2192, 2370, 2562, 2694, 2710, 2772, 3167, 3384, 3431, 3480, 3601, 3972, 4187, 4308, 4475, 4660, 4699, 5150, 1266, 1639, 2974, 4289, 5111, 1358, 1648, 1683, 1797, 2338, 2451, 2633, 2669, 2978, 3376, 3418, 3610, 3991, 4294, 4665, 5040, 5169, 174, 178, 389, 471, 517, 775, 882, 988, 1032, 1134, 1225, 1339, 1574, 1600, 1610, 1692, 2130, 2257, 2362, 2370, 2376, 2592, 3003, 3117, 3314, 3738, 3782, 3843, 4115, 4652, 4700, 4832, 4997, 5018, 335, 481, 595, 601, 778, 885, 917, 1117, 1144, 1251, 1427, 1811, 1827, 1846, 2604, 2646, 2667, 2753, 2779, 2815, 3356, 3528, 4095, 4248, 4928, 4960, 5043, 5167, 77, 322, 497, 636, 885, 1327, 1737, 1858, 1877, 1906, 1931, 2008, 2015, 2590, 2748, 3067, 3779, 3908, 4727, 112, 125, 367, 420, 511, 1138, 1239, 1455, 1497, 1522, 1542, 1563, 1814, 2097, 2626, 2746, 3005, 3140, 3406, 3480, 3495, 3844, 3972, 4155, 4230, 4852, 4906, 4913, 4923, 4968, 206, 223, 446, 1174, 1258, 1567, 1573, 1604, 1685, 1695, 2257, 2301, 2449, 2636, 2664, 2883, 2885, 3017, 3214, 3961, 4096, 4139, 4304, 4355, 4443, 4828, 4949, 5061, 370, 485, 797, 981, 1328, 2122, 2640, 2642, 2883, 3131, 3481, 3552, 3564, 3844, 4853, 4861, 5101, 10, 18, 40, 55, 91, 160, 164, 181, 196, 211, 227, 332, 334, 407, 414, 482, 533, 595, 675, 734, 739, 799, 803, 807, 815, 910, 971, 983, 994, 1089, 1128, 1134, 1170, 1202, 1256, 1292, 1320, 1330, 1340, 1452, 1462, 1526, 1558, 1610, 1627, 1660, 1787, 1818, 1861, 1932, 1936, 1963, 1972, 1986, 1987, 2048, 2049, 2054, 2056, 2130, 2137, 2160, 2201, 2294, 2308, 2338, 2396, 2410, 2458, 2467, 2485, 2532, 2574, 2589, 2753, 2754, 2774, 2917, 3006, 3120, 3134, 3234, 3238, 3239, 3288, 3355, 3361, 3365, 3368, 3394, 3406, 3418, 3439, 3452, 3558, 3569, 3597, 3628, 3631, 3644, 3698, 3767, 3902, 3907, 3937, 3996, 4097, 4110, 4139, 4147, 4174, 4219, 4262, 4281, 4311, 4333, 4408, 4445, 4507, 4568, 4624, 4625, 4665, 4677, 4678, 4717, 4833, 4859, 4867, 4911, 4947, 4981, 5079, 5135, 147, 1027, 2216, 3063, 4440, 4724, 4782, 11, 57, 63, 75, 77, 82, 83, 173, 192, 193, 209, 213, 270, 272, 297, 316, 319, 328, 332, 391, 418, 436, 474, 510, 562, 572, 584, 593, 628, 641, 653, 656, 690, 704, 725, 740, 743, 781, 807, 839, 847, 854, 869, 871, 888, 910, 945, 951, 989, 1027, 1049, 1084, 1134, 1136, 1144, 1157, 1170, 1179, 1225, 1258, 1309, 1314, 1321, 1361, 1369, 1449, 1465, 1501, 1519, 1545, 1563, 1573, 1577, 1616, 1677, 1726, 1758, 1772, 1786, 1792, 1796, 1818, 1827, 1854, 1864, 1869, 1904, 1909, 1952, 2006, 2018, 2045, 2066, 2110, 2134, 2137, 2148, 2175, 2180, 2283, 2291, 2310, 2350, 2352, 2368, 2407, 2472, 2482, 2507, 2511, 2517, 2523, 2535, 2552, 2565, 2585, 2646, 2661, 2667, 2688, 2699, 2705, 2706, 2758, 2779, 2806, 2813, 2817, 2866, 2869, 2874, 2933, 2945, 2947, 2978, 2983, 3002, 3004, 3017, 3031, 3039, 3048, 3057, 3085, 3093, 3134, 3141, 3143, 3148, 3170, 3177, 3186, 3245, 3266, 3328, 3352, 3356, 3357, 3361, 3386, 3406, 3434, 3457, 3491, 3502, 3529, 3553, 3564, 3640, 3643, 3648, 3653, 3664, 3709, 3739, 3745, 3801, 3803, 3808, 3837, 3855, 3865, 3890, 3896, 3904, 3908, 3910, 3917, 3953, 4002, 4068, 4171, 4181, 4195, 4247, 4274, 4304, 4306, 4314, 4316, 4331, 4440, 4450, 4463, 4478, 4571, 4606, 4613, 4649, 4665, 4739, 4777, 4778, 4784, 4799, 4823, 4841, 4849, 4876, 4906, 4928, 4947, 4964, 4981, 5022, 5046, 5077, 5133, 5143, 77, 446, 482, 497, 504, 561, 636, 734, 1082, 1261, 1280, 1376, 1687, 1876, 1930, 1931, 2065, 2125, 2198, 3047, 3063, 3395, 3441, 3446, 3472, 3678, 3908, 4351, 4664, 4809, 4841, 5035, 114, 475, 1198, 2705, 3112, 3154, 3247, 3494, 4190, 4374, 4574, 4707, 5054, 262, 482, 834, 1382, 1429, 2442, 2555, 3196, 3423, 3446, 4663</t>
   </si>
   <si>
     <t>38.76</t>
@@ -559,13 +559,13 @@
     <t>FR12_2, FR12_3, FR12_4, FR12_7, FR12_14, FR12_15, FR12_17, FR12_19, FR12_20, FR12_21, FR12_23, FR12_24, FR12_26, FR12_28, FR12_31, FR12_32, FR12_33, FR12_34, FR12_36, FR12_43, FR12_46, FR12_49, FR12_51, FR12_58, FR12_59, FR12_61, FR12_63, FR12_69, FR12_71, FR12_72, FR12_78, FR12_80, FR12_81, FR12_88, FR12_89, FR12_91, FR12_93, FR12_96, FR12_97, FR12_98, FR12_100, FR12_101, FR12_104, FR12_105, FR12_106, FR12_107, FR12_113, FR12_115, FR12_119, FR12_120, FR12_121, FR12_123, FR12_124, FR12_126, FR12_128, FR12_129, FR12_131, FR12_133, FR12_136, FR12_137, FR12_143, FR12_157, FR12_162, FR12_163, FR12_164, FR12_166, FR17_2, FR17_3, FR17_4, FR17_7, FR17_14, FR17_15, FR17_17, FR17_19, FR17_20, FR17_21, FR17_23, FR17_24, FR17_26, FR17_28, FR17_31, FR17_32, FR17_33, FR17_34, FR17_36, FR17_43, FR17_46, FR17_49, FR17_51, FR17_58, FR17_59, FR17_61, FR17_63, FR17_69, FR17_71, FR17_72, FR17_78, FR17_80, FR17_81, FR17_88, FR17_89, FR17_91, FR17_93, FR17_96, FR17_97, FR17_98, FR17_100, FR17_101, FR17_104, FR17_105, FR17_106, FR17_107, FR17_113, FR17_115, FR17_119, FR17_120, FR17_121, FR17_123, FR17_124, FR17_126, FR17_128, FR17_129, FR17_131, FR17_133, FR17_136, FR17_137, FR17_143, FR17_157, FR17_162, FR17_163, FR17_164, FR17_166</t>
   </si>
   <si>
-    <t>96.66</t>
-  </si>
-  <si>
-    <t>5000</t>
-  </si>
-  <si>
-    <t>287, 310, 375, 432, 852, 1205, 1564, 1613, 1735, 1834, 1997, 2042, 2425, 2460, 2465, 2708, 2782, 2849, 3270, 3273, 3513, 3531, 4262, 5024, 5032, 5106, 5112, 93, 1302, 3968, 4000, 4002, 4354, 4563, 20, 567, 635, 827, 1336, 1524, 1932, 2451, 2585, 2764, 2993, 3066, 3659, 4187, 4423, 4657, 5136, 199, 297, 883, 1057, 1177, 1362, 1484, 1496, 1716, 1846, 1879, 1954, 2046, 2100, 2346, 2404, 2419, 2449, 2590, 2616, 2646, 2653, 2659, 2788, 2833, 2952, 3059, 3126, 3156, 3205, 3249, 3464, 3501, 3624, 3767, 4153, 4366, 4466, 4569, 4733, 5009, 5113, 517, 549, 567, 640, 4053, 4079, 79, 142, 177, 467, 517, 677, 721, 737, 751, 832, 979, 1060, 1077, 1171, 1236, 1348, 1479, 1503, 1509, 1531, 1570, 1610, 1669, 1719, 1820, 1831, 1874, 1878, 1905, 1940, 2012, 2027, 2250, 2316, 2356, 2413, 2427, 2470, 2511, 2672, 2806, 2809, 2864, 3020, 3033, 3184, 3225, 3280, 3308, 3313, 3468, 3474, 3513, 3681, 3708, 3845, 3851, 3862, 3866, 3895, 3931, 4037, 4123, 4206, 4250, 4320, 4359, 4366, 4402, 4478, 4586, 4596, 4661, 4686, 4714, 4752, 4789, 4793, 4912, 4931, 5040, 5089, 5138, 3, 6, 108, 116, 187, 199, 257, 286, 331, 332, 336, 357, 365, 411, 455, 507, 510, 546, 574, 606, 607, 608, 618, 629, 672, 712, 730, 751, 805, 852, 870, 880, 897, 917, 937, 944, 945, 1024, 1060, 1096, 1102, 1150, 1155, 1239, 1245, 1251, 1298, 1306, 1337, 1373, 1396, 1401, 1455, 1473, 1491, 1494, 1499, 1511, 1515, 1533, 1537, 1549, 1564, 1592, 1609, 1637, 1688, 1691, 1712, 1844, 1878, 1890, 1911, 1929, 1944, 1967, 2053, 2074, 2090, 2125, 2128, 2131, 2143, 2149, 2230, 2256, 2262, 2344, 2345, 2346, 2354, 2449, 2461, 2479, 2504, 2578, 2615, 2619, 2627, 2630, 2650, 2671, 2741, 2757, 2763, 2801, 2825, 2861, 2872, 2876, 2893, 2922, 2928, 2944, 2950, 2964, 2977, 2998, 3022, 3036, 3087, 3099, 3135, 3198, 3323, 3326, 3339, 3340, 3348, 3350, 3367, 3375, 3380, 3487, 3512, 3536, 3604, 3605, 3612, 3635, 3692, 3741, 3762, 3771, 3776, 3821, 3836, 3895, 3908, 3917, 3962, 4039, 4052, 4053, 4065, 4089, 4111, 4133, 4141, 4154, 4213, 4254, 4269, 4271, 4318, 4382, 4395, 4408, 4413, 4435, 4478, 4525, 4550, 4561, 4565, 4568, 4573, 4603, 4637, 4640, 4669, 4693, 4736, 4768, 4775, 4817, 4910, 4940, 4969, 4978, 5007, 5018, 5043, 5101, 5122, 287, 308, 320, 331, 446, 467, 519, 545, 604, 729, 1025, 1031, 1535, 1777, 1788, 1806, 1898, 1933, 1947, 1984, 2021, 2137, 2185, 2211, 2272, 2280, 2306, 2434, 2484, 2559, 2591, 2616, 2636, 2802, 2837, 2849, 2854, 2893, 2928, 2977, 3073, 3154, 3163, 3177, 3339, 3366, 3406, 3443, 3490, 3520, 3527, 3559, 3581, 3698, 3755, 3769, 3860, 3862, 3875, 4006, 4025, 4188, 4193, 4318, 4350, 4397, 4610, 4620, 4630, 4774, 4799, 4847, 4857, 4860, 4863, 4882, 4914, 4940, 5001, 5100, 5112, 5121, 5129, 14, 48, 89, 106, 119, 120, 230, 267, 271, 273, 287, 297, 344, 360, 398, 455, 484, 536, 581, 587, 640, 777, 778, 796, 827, 923, 933, 938, 947, 979, 987, 1037, 1046, 1056, 1064, 1084, 1091, 1102, 1111, 1115, 1137, 1172, 1187, 1195, 1216, 1233, 1248, 1275, 1298, 1304, 1308, 1321, 1367, 1372, 1406, 1465, 1531, 1564, 1570, 1612, 1623, 1741, 1831, 1861, 1867, 1886, 1894, 1911, 1917, 1922, 1925, 1931, 1967, 2031, 2044, 2063, 2068, 2083, 2087, 2108, 2126, 2221, 2222, 2239, 2264, 2283, 2295, 2302, 2340, 2358, 2384, 2540, 2553, 2576, 2595, 2627, 2651, 2746, 2780, 2781, 2800, 2818, 2824, 2919, 2929, 2967, 3018, 3050, 3061, 3069, 3085, 3125, 3225, 3245, 3248, 3267, 3279, 3315, 3320, 3334, 3369, 3372, 3439, 3479, 3501, 3577, 3590, 3627, 3658, 3705, 3707, 3724, 3766, 3813, 3860, 3868, 3886, 3892, 3915, 3950, 4006, 4052, 4087, 4096, 4097, 4111, 4251, 4259, 4294, 4323, 4395, 4408, 4467, 4480, 4568, 4591, 4625, 4653, 4733, 4754, 4799, 4827, 4843, 4859, 4882, 4985, 5025, 5043, 5094, 5108, 5121, 5124, 5164, 37, 106, 160, 169, 179, 209, 228, 230, 262, 348, 350, 392, 404, 460, 541, 550, 557, 584, 600, 610, 629, 668, 671, 684, 695, 715, 771, 810, 835, 869, 934, 1011, 1081, 1095, 1105, 1139, 1205, 1401, 1445, 1463, 1475, 1492, 1515, 1533, 1565, 1625, 1635, 1669, 1814, 1940, 1955, 1959, 1970, 2054, 2080, 2084, 2098, 2118, 2131, 2171, 2194, 2230, 2234, 2241, 2246, 2283, 2371, 2374, 2473, 2500, 2560, 2622, 2660, 2727, 2736, 2746, 2928, 2934, 3173, 3245, 3317, 3384, 3405, 3410, 3421, 3507, 3512, 3542, 3552, 3594, 3634, 3645, 3656, 3707, 3740, 3768, 3779, 3844, 3874, 3893, 3894, 3943, 4002, 4074, 4078, 4091, 4231, 4235, 4250, 4261, 4348, 4410, 4419, 4550, 4570, 4584, 4601, 4668, 4669, 4672, 4704, 4710, 4744, 4750, 4793, 4857, 4920, 5103, 5143, 57, 109, 240, 885, 905, 2056, 2241, 2377, 2722, 2977, 5014, 5147, 81, 345, 405, 1105, 1269, 1492, 1954, 2160, 2241, 2491, 2690, 2928, 3071, 3190, 3302, 3655, 3893, 4235, 4857, 5103, 107, 221, 229, 266, 587, 652, 709, 778, 890, 948, 1002, 1053, 1083, 1087, 1096, 1239, 1352, 1407, 1441, 1567, 1663, 1664, 1729, 1774, 1847, 1954, 1967, 2021, 2137, 2285, 2451, 2453, 2472, 2504, 2524, 2526, 2584, 2594, 2600, 2700, 2856, 2913, 2981, 3011, 3015, 3108, 3114, 3117, 3125, 3149, 3266, 3301, 3356, 3420, 3480, 3496, 3688, 3724, 3738, 3803, 3889, 3971, 3996, 4034, 4040, 4076, 4078, 4082, 4087, 4123, 4141, 4163, 4295, 4451, 4479, 4485, 4631, 4654, 4759, 4826, 4883, 5024, 0, 28, 46, 86, 90, 99, 107, 116, 233, 343, 353, 366, 481, 495, 504, 524, 555, 567, 584, 597, 600, 623, 635, 643, 644, 652, 689, 690, 714, 744, 905, 927, 988, 1008, 1024, 1032, 1098, 1120, 1128, 1160, 1187, 1197, 1205, 1211, 1267, 1269, 1323, 1350, 1425, 1477, 1512, 1537, 1648, 1654, 1712, 1720, 1735, 1780, 1816, 1831, 1890, 1904, 1928, 1947, 2047, 2054, 2069, 2125, 2178, 2222, 2226, 2235, 2253, 2260, 2265, 2289, 2408, 2418, 2453, 2469, 2475, 2494, 2570, 2580, 2682, 2734, 2765, 2809, 2824, 2841, 2868, 2892, 2903, 2916, 2934, 2985, 2989, 3020, 3036, 3147, 3296, 3308, 3337, 3388, 3399, 3401, 3406, 3439, 3479, 3498, 3547, 3549, 3599, 3604, 3609, 3619, 3624, 3627, 3663, 3674, 3701, 3771, 3795, 3849, 3911, 3963, 3975, 4012, 4074, 4092, 4134, 4149, 4154, 4193, 4247, 4260, 4265, 4269, 4303, 4346, 4402, 4419, 4546, 4568, 4619, 4623, 4625, 4654, 4726, 4748, 4750, 4827, 4847, 4960, 4999, 5032, 5096, 5097, 5110, 5126, 5136, 5138, 5147, 308, 1032, 2210, 2250, 2714, 3276, 3552, 3908, 4317, 33, 47, 57, 90, 95, 109, 283, 309, 320, 325, 363, 369, 412, 508, 572, 590, 640, 645, 727, 737, 768, 792, 913, 930, 933, 967, 974, 982, 999, 1051, 1058, 1121, 1367, 1511, 1633, 1692, 1712, 1735, 1741, 1766, 1767, 1820, 1849, 1874, 1880, 1898, 1922, 1978, 1988, 2029, 2054, 2057, 2084, 2168, 2244, 2268, 2288, 2295, 2316, 2324, 2344, 2360, 2397, 2403, 2475, 2523, 2540, 2622, 2649, 2652, 2704, 2755, 2779, 2892, 2897, 2952, 2963, 2967, 3011, 3033, 3036, 3061, 3143, 3144, 3227, 3235, 3244, 3266, 3290, 3293, 3331, 3356, 3383, 3396, 3456, 3457, 3464, 3522, 3529, 3557, 3574, 3652, 3663, 3669, 3751, 3793, 3971, 4017, 4033, 4067, 4103, 4126, 4163, 4188, 4222, 4240, 4250, 4272, 4348, 4350, 4366, 4406, 4423, 4510, 4531, 4619, 4631, 4673, 4690, 4726, 4748, 4786, 4814, 4873, 4899, 4922, 5025, 5032, 5080, 5158, 0, 14, 47, 63, 90, 93, 102, 131, 137, 142, 152, 175, 177, 199, 219, 221, 290, 299, 392, 418, 489, 497, 517, 632, 672, 701, 760, 838, 872, 915, 919, 927, 1038, 1057, 1058, 1194, 1204, 1211, 1259, 1298, 1321, 1351, 1451, 1496, 1518, 1559, 1603, 1629, 1645, 1678, 1723, 1735, 1769, 1782, 1811, 1829, 1853, 1880, 1894, 1905, 1927, 1941, 1978, 2018, 2128, 2158, 2166, 2210, 2213, 2217, 2223, 2226, 2289, 2321, 2345, 2351, 2355, 2395, 2435, 2451, 2490, 2553, 2581, 2597, 2612, 2622, 2629, 2654, 2718, 2723, 2731, 2788, 2807, 2825, 2843, 2861, 2890, 2915, 2926, 2935, 2950, 2981, 2983, 2988, 3007, 3127, 3157, 3225, 3248, 3277, 3280, 3296, 3302, 3348, 3366, 3388, 3443, 3445, 3461, 3477, 3547, 3550, 3602, 3610, 3644, 3699, 3718, 3746, 3768, 3815, 3833, 3854, 3979, 4029, 4047, 4094, 4095, 4105, 4133, 4152, 4193, 4294, 4353, 4365, 4381, 4396, 4410, 4423, 4506, 4510, 4531, 4563, 4574, 4597, 4653, 4670, 4688, 4699, 4738, 4775, 4787, 4831, 4852, 4857, 4865, 4870, 4913, 4964, 4969, 4978, 5016, 5027, 5033, 5043, 5046, 5096, 5101, 5112, 5123, 5165, 19, 37, 74, 211, 225, 273, 336, 348, 410, 522, 538, 577, 650, 652, 952, 958, 1137, 1138, 1166, 1187, 1538, 1544, 1555, 1559, 1570, 1646, 1693, 1697, 1712, 1719, 1820, 1880, 1922, 1991, 2168, 2223, 2239, 2244, 2292, 2397, 2540, 2606, 2637, 2726, 2816, 2827, 2981, 3207, 3235, 3244, 3292, 3383, 3388, 3391, 3423, 3545, 3663, 3707, 3861, 3945, 3976, 4039, 4133, 4142, 4217, 4287, 4303, 4523, 4603, 4713, 4733, 4775, 4805, 4874, 4900, 4910, 4920, 4928, 4967, 4970, 4986, 5022, 5089, 24, 75, 118, 186, 233, 238, 258, 318, 360, 398, 796, 952, 1059, 1095, 1188, 1280, 1360, 1465, 1522, 1777, 2042, 2056, 2118, 2143, 2158, 2321, 2395, 2460, 2557, 2581, 2681, 2736, 2986, 3112, 3122, 3137, 3155, 3214, 3241, 3302, 3334, 3356, 3429, 3445, 3501, 3570, 3594, 3644, 4030, 4223, 4354, 4396, 4507, 4544, 4563, 4574, 4646, 4738, 4744, 4895, 4968, 5034, 36, 111, 229, 234, 273, 422, 423, 462, 525, 536, 564, 610, 627, 748, 795, 801, 826, 854, 866, 880, 905, 999, 1002, 1052, 1083, 1092, 1124, 1155, 1212, 1268, 1285, 1409, 1545, 1634, 1667, 1671, 1722, 1770, 1782, 1793, 1796, 1837, 1845, 1874, 1922, 2012, 2018, 2050, 2082, 2106, 2145, 2162, 2226, 2275, 2300, 2311, 2423, 2453, 2461, 2519, 2523, 2559, 2590, 2606, 2648, 2652, 2718, 2742, 2856, 2876, 2915, 2944, 2985, 3011, 3042, 3052, 3087, 3115, 3207, 3209, 3283, 3302, 3367, 3605, 3645, 3827, 3912, 3968, 4064, 4076, 4206, 4221, 4226, 4320, 4327, 4334, 4431, 4541, 4592, 4620, 4630, 4702, 4703, 4735, 4775, 4779, 4928, 4944, 5009, 31, 131, 585, 734, 831, 1042, 1058, 1451, 1489, 1799, 1948, 1996, 2018, 2173, 2508, 2537, 2541, 2597, 2716, 2718, 2722, 2975, 3068, 3449, 3816, 4060, 4439, 4526, 4563, 4572, 4883, 5025, 5046, 5094, 5117, 1581, 1782, 4119, 4171, 4669, 4708, 4729, 4810, 4813, 0, 93, 123, 218, 229, 256, 263, 291, 329, 435, 446, 481, 511, 522, 524, 549, 555, 577, 603, 607, 645, 660, 682, 948, 1060, 1076, 1086, 1215, 1244, 1394, 1549, 1660, 1689, 1711, 1828, 1881, 1905, 1919, 1987, 1995, 2069, 2116, 2210, 2247, 2362, 2404, 2413, 2415, 2501, 2534, 2561, 2629, 2837, 2849, 2933, 2967, 3008, 3054, 3126, 3212, 3318, 3337, 3397, 3513, 3594, 3624, 3666, 3719, 3755, 3908, 4051, 4079, 4087, 4119, 4147, 4171, 4199, 4316, 4353, 4385, 4389, 4498, 4506, 4513, 4710, 4821, 4994, 5057, 5112, 549, 938, 1248, 1801, 2085, 2247, 2415, 3008, 3464, 3624, 4754, 5112, 69, 145, 158, 263, 273, 283, 320, 332, 375, 482, 682, 709, 1090, 1136, 1201, 1236, 1248, 1469, 1648, 1759, 1763, 1776, 1786, 1797, 1821, 1826, 2054, 2055, 2080, 2116, 2117, 2268, 2289, 2302, 2399, 2408, 2426, 2449, 2479, 2536, 2600, 2615, 2653, 2696, 2716, 2755, 2761, 2978, 2981, 2985, 2988, 3000, 3120, 3125, 3165, 3179, 3362, 3363, 3423, 3645, 3795, 3808, 3832, 3836, 3923, 4039, 4040, 4181, 4218, 4231, 4250, 4259, 4316, 4336, 4467, 4520, 4539, 4586, 4650, 4690, 4700, 4711, 4767, 4864, 4900, 4946, 5034, 5042, 5050, 5085, 5109, 5112, 5138, 46, 85, 90, 95, 96, 167, 478, 589, 630, 699, 778, 830, 831, 866, 896, 933, 976, 1029, 1042, 1051, 1065, 1096, 1171, 1210, 1318, 1333, 1459, 1477, 1503, 1507, 1524, 1592, 1780, 1858, 1898, 2002, 2051, 2173, 2230, 2248, 2352, 2373, 2391, 2522, 2545, 2559, 2561, 2624, 2638, 2874, 3217, 3319, 3346, 3360, 3400, 3437, 3448, 3478, 3487, 3526, 3534, 3594, 3687, 3962, 4028, 4065, 4171, 4233, 4291, 4294, 4323, 4526, 4563, 4739, 4863, 4876, 4971, 4977, 5027, 5104, 89, 271, 338, 360, 777, 1205, 1321, 1463, 1623, 1984, 2320, 2786, 3230, 3245, 3248, 3705, 3861, 4653, 4750, 4783, 4843, 4857, 4931, 35, 199, 209, 227, 263, 290, 329, 353, 357, 400, 424, 481, 545, 608, 672, 696, 700, 705, 787, 792, 814, 851, 923, 987, 998, 1016, 1032, 1086, 1189, 1211, 1331, 1333, 1342, 1498, 1524, 1539, 1603, 1659, 1664, 1776, 1793, 1898, 1931, 1996, 2043, 2072, 2080, 2117, 2150, 2183, 2198, 2221, 2239, 2267, 2423, 2528, 2553, 2758, 2766, 2820, 2923, 2954, 3045, 3084, 3093, 3098, 3144, 3156, 3214, 3229, 3270, 3334, 3400, 3445, 3498, 3532, 3557, 3645, 3655, 3699, 3719, 3817, 3870, 3889, 3928, 3932, 3966, 4011, 4058, 4105, 4193, 4226, 4334, 4431, 4435, 4451, 4482, 4528, 4597, 4648, 4740, 4784, 4793, 4909, 4988, 5023, 5032, 5051, 5073, 5124, 5138, 28, 73, 75, 90, 112, 122, 137, 142, 225, 320, 410, 423, 545, 565, 604, 642, 682, 701, 725, 756, 809, 863, 1016, 1051, 1180, 1189, 1210, 1378, 1525, 1535, 1545, 1569, 1570, 1720, 1723, 1769, 1782, 1799, 1807, 1905, 2018, 2040, 2042, 2063, 2130, 2211, 2266, 2326, 2331, 2362, 2483, 2561, 2564, 2582, 2650, 2660, 2714, 2814, 2970, 2978, 3122, 3125, 3249, 3391, 3484, 3513, 3588, 3597, 3660, 3717, 3748, 3769, 3851, 3875, 4042, 4057, 4065, 4163, 4172, 4193, 4262, 4412, 4448, 4453, 4467, 4550, 4593, 4693, 4784, 4814, 4905, 4944, 4969, 4983, 5059, 5112, 5143, 5168, 411, 446, 577, 607, 715, 933, 982, 1042, 1351, 1515, 1689, 1806, 2494, 2849, 3284, 3484, 3569, 3997, 4418, 4669, 4743, 4887, 5046, 28, 107, 299, 660, 838, 1037, 1076, 1168, 1234, 1463, 1552, 1728, 1986, 2030, 2042, 2226, 2395, 2398, 2856, 3725, 3825, 3833, 4002, 4051, 4141, 4213, 4216, 4340, 4385, 4408, 4523, 4733, 4828, 4909, 5025, 5106, 32, 73, 74, 99, 121, 168, 287, 338, 366, 389, 392, 418, 443, 460, 462, 642, 727, 769, 813, 828, 860, 872, 933, 934, 959, 1158, 1177, 1212, 1260, 1290, 1502, 1567, 1641, 1690, 1759, 1796, 1807, 1839, 1847, 1855, 1894, 1912, 2038, 2061, 2128, 2144, 2183, 2353, 2490, 2493, 2514, 2555, 2582, 2680, 2706, 2801, 2824, 2837, 2949, 2981, 2995, 3008, 3026, 3060, 3070, 3118, 3161, 3184, 3276, 3326, 3391, 3397, 3461, 3474, 3576, 3658, 3831, 3836, 3872, 3880, 3916, 4155, 4259, 4354, 4359, 4385, 4563, 4618, 4669, 4690, 4717, 4844, 5021, 5108, 5113, 5169, 89, 151, 210, 555, 776, 880, 913, 979, 1011, 1103, 1115, 1372, 1484, 1712, 2030, 2221, 2408, 2761, 2837, 2963, 2966, 2984, 3043, 3059, 3110, 3265, 3365, 3486, 3762, 3997, 4064, 4097, 4254, 4269, 4274, 4526, 4582, 4736, 4743, 4837, 4838, 4841, 4844, 4865, 35, 162, 258, 343, 417, 477, 709, 860, 1186, 1259, 1297, 1308, 1645, 1675, 1927, 1995, 2084, 2167, 2194, 2217, 2260, 2320, 2346, 2484, 2581, 2585, 2659, 2786, 2817, 2842, 2868, 2938, 2989, 3103, 3136, 3201, 3301, 3427, 3486, 3513, 3738, 3790, 3802, 3886, 4091, 4092, 4213, 4284, 4440, 4515, 4633, 4774, 4831, 4882, 4894, 4960, 4968, 4982, 5021, 5100, 29, 83, 99, 151, 212, 251, 291, 296, 310, 313, 318, 481, 625, 635, 846, 1008, 1029, 1054, 1064, 1220, 1323, 1331, 1396, 1432, 1445, 1503, 1525, 1549, 1575, 1622, 1664, 1707, 1755, 1986, 2020, 2030, 2058, 2131, 2170, 2211, 2220, 2222, 2247, 2264, 2266, 2295, 2306, 2355, 2362, 2410, 2427, 2494, 2554, 2615, 2630, 2636, 2650, 2690, 2704, 2718, 2727, 2766, 2779, 2846, 2876, 2890, 3015, 3099, 3102, 3103, 3108, 3111, 3179, 3190, 3247, 3273, 3290, 3305, 3339, 3345, 3367, 3477, 3570, 3652, 3847, 3891, 3903, 3908, 3923, 3972, 4029, 4048, 4074, 4095, 4183, 4199, 4206, 4213, 4296, 4299, 4359, 4376, 4448, 4490, 4527, 4572, 4575, 4597, 4699, 4709, 4711, 4844, 4876, 4892, 4978, 4985, 5032, 5039, 5055, 5096, 5134, 5168, 64, 81, 144, 332, 396, 504, 652, 680, 771, 866, 987, 1171, 1303, 1441, 1496, 1502, 1544, 2084, 2121, 2170, 2266, 2293, 2339, 2526, 2528, 2583, 2590, 2662, 2696, 2868, 3016, 3033, 3051, 3292, 3340, 3365, 3563, 3574, 3918, 4022, 4042, 4075, 4079, 4135, 4201, 4303, 4456, 4501, 4553, 4667, 4821, 4879, 4883, 4948, 5103, 5104, 93, 111, 122, 169, 209, 210, 211, 218, 226, 238, 309, 323, 376, 385, 405, 427, 481, 488, 517, 555, 577, 584, 595, 608, 621, 642, 646, 658, 687, 712, 727, 773, 785, 829, 846, 848, 870, 933, 941, 966, 971, 985, 1024, 1037, 1073, 1105, 1147, 1217, 1233, 1259, 1275, 1323, 1364, 1374, 1409, 1443, 1453, 1479, 1480, 1514, 1559, 1567, 1596, 1649, 1654, 1675, 1691, 1720, 1780, 1804, 1810, 1834, 1868, 1874, 1885, 1905, 1944, 1945, 1948, 2049, 2061, 2063, 2070, 2088, 2093, 2126, 2223, 2239, 2268, 2271, 2327, 2489, 2560, 2590, 2624, 2685, 2700, 2724, 2756, 2766, 2843, 2848, 2857, 2879, 2919, 2933, 2935, 2954, 2964, 2997, 3029, 3043, 3070, 3084, 3099, 3108, 3111, 3116, 3146, 3157, 3237, 3264, 3356, 3391, 3397, 3457, 3472, 3478, 3504, 3541, 3570, 3582, 3660, 3701, 3740, 3746, 3795, 3821, 3827, 3875, 3884, 3912, 3929, 3934, 3970, 4028, 4074, 4091, 4103, 4162, 4170, 4200, 4201, 4206, 4214, 4256, 4260, 4286, 4306, 4382, 4388, 4413, 4429, 4439, 4533, 4541, 4550, 4633, 4661, 4668, 4705, 4713, 4726, 4769, 4784, 4870, 4886, 4928, 4948, 4994, 5027, 5043, 5057, 5097, 5113, 5123, 5124, 5138, 5156, 5163, 5168, 5170, 5172, 137, 142, 270, 363, 427, 460, 467, 590, 642, 681, 725, 744, 769, 808, 927, 998, 1016, 1024, 1041, 1045, 1051, 1098, 1108, 1172, 1233, 1290, 1325, 1342, 1374, 1378, 1441, 1463, 1538, 1546, 1565, 1570, 1645, 1678, 1799, 1810, 1814, 2036, 2129, 2147, 2149, 2426, 2431, 2541, 2572, 2697, 2717, 2736, 2820, 2870, 2890, 3244, 3249, 3339, 3367, 3375, 3396, 3437, 3472, 3481, 3498, 3663, 3708, 3727, 3769, 3811, 3875, 4028, 4076, 4091, 4103, 4122, 4222, 4226, 4312, 4449, 4550, 4624, 4733, 4787, 4811, 4814, 4816, 4857, 4967, 5094, 416, 499, 529, 549, 728, 1494, 2029, 2264, 2498, 2855, 3015, 3190, 3201, 3276, 3407, 3416, 3458, 3614, 3696, 3751, 4204, 4299, 838, 1064, 1108, 1575, 1621, 4482, 4493, 4601, 4827, 5157, 280, 291, 552, 1520, 1818, 1847, 1971, 2722, 2768, 3863, 2127, 2377, 2939, 3007, 4646, 5157, 35, 96, 256, 336, 348, 415, 443, 460, 554, 564, 685, 795, 796, 848, 875, 963, 982, 1013, 1052, 1067, 1100, 1176, 1305, 1469, 1613, 1616, 1764, 1816, 1834, 1890, 2083, 2108, 2206, 2210, 2225, 2349, 2394, 2473, 2864, 2907, 2915, 2993, 3026, 3076, 3087, 3143, 3158, 3284, 3318, 3457, 3503, 3582, 3627, 3688, 3765, 3913, 3928, 4032, 4042, 4087, 4103, 4111, 4113, 4135, 4200, 4201, 4240, 4271, 4425, 4528, 4549, 4561, 4565, 4615, 4752, 4850, 4940, 5094, 5156, 5159, 5169, 289, 1246, 2259, 3122, 4140, 814, 1604, 1668, 3020, 3880, 10, 47, 137, 266, 273, 464, 557, 566, 810, 1040, 1353, 1457, 1860, 1931, 2084, 2418, 2456, 2613, 2649, 2791, 3051, 3301, 3397, 3531, 3652, 3687, 3706, 3822, 3996, 4039, 4052, 4188, 4204, 4256, 4748, 5100, 168, 1570, 2149, 2167, 2555, 3974, 4899, 113, 273, 432, 481, 524, 554, 644, 682, 763, 971, 1040, 1087, 1348, 1409, 1489, 1514, 1532, 1567, 1579, 1609, 1612, 1721, 1851, 2042, 2068, 2085, 2097, 2271, 2583, 2672, 2717, 2738, 3149, 3334, 3619, 3836, 3851, 4207, 4278, 4481, 4506, 4542, 4750, 4976, 5134, 5149, 3917, 3968, 4055, 138, 191, 424, 1245, 1351, 1507, 1629, 1704, 1928, 2090, 2149, 2416, 2563, 2580, 2697, 3059, 3284, 3547, 3577, 3800, 4141, 4144, 4235, 4256, 4348, 4417, 4430, 4506, 4615, 4640, 4682, 4845, 4914, 4942, 4976, 4986, 48, 83, 137, 175, 202, 318, 329, 347, 350, 378, 524, 534, 570, 589, 592, 616, 680, 797, 800, 826, 1040, 1048, 1058, 1073, 1101, 1216, 1289, 1306, 1321, 1405, 1426, 1517, 1518, 1636, 1654, 1834, 1889, 1938, 2020, 2053, 2087, 2088, 2112, 2168, 2352, 2367, 2451, 2469, 2476, 2554, 2610, 2624, 2629, 2738, 2776, 2928, 2949, 2977, 2997, 3029, 3063, 3087, 3099, 3102, 3114, 3135, 3249, 3282, 3306, 3356, 3422, 3427, 3478, 3502, 3559, 3590, 3706, 3708, 3733, 3738, 3822, 3938, 3971, 3979, 4089, 4193, 4226, 4270, 4459, 4498, 4503, 4515, 4546, 4584, 4676, 4723, 4763, 4768, 4839, 4881, 4960, 5001, 0, 10, 48, 89, 99, 107, 119, 121, 137, 151, 174, 224, 271, 291, 317, 343, 379, 392, 458, 499, 523, 539, 554, 589, 593, 617, 621, 627, 643, 769, 803, 830, 851, 875, 891, 1001, 1006, 1081, 1087, 1137, 1138, 1183, 1220, 1245, 1304, 1323, 1325, 1331, 1340, 1358, 1381, 1402, 1457, 1496, 1567, 1615, 1626, 1634, 1648, 1674, 1712, 1729, 1769, 1774, 1801, 1843, 1898, 1906, 1948, 2020, 2031, 2040, 2070, 2084, 2133, 2153, 2193, 2194, 2239, 2264, 2296, 2326, 2345, 2354, 2391, 2465, 2476, 2591, 2597, 2617, 2623, 2627, 2649, 2759, 2760, 2818, 2841, 2842, 2877, 2884, 2903, 2917, 2919, 2933, 2997, 3029, 3043, 3074, 3080, 3085, 3124, 3125, 3179, 3187, 3198, 3230, 3240, 3248, 3265, 3320, 3322, 3339, 3428, 3478, 3479, 3529, 3617, 3663, 3682, 3708, 3767, 3769, 3821, 3870, 3884, 3893, 3915, 3950, 3955, 3968, 4025, 4067, 4074, 4079, 4094, 4097, 4103, 4250, 4260, 4346, 4404, 4409, 4479, 4482, 4500, 4612, 4664, 4682, 4696, 4709, 4714, 4816, 4931, 4944, 5001, 5014, 5055, 5087, 5165, 26, 74, 112, 163, 251, 314, 422, 523, 538, 642, 678, 828, 830, 906, 926, 941, 999, 1030, 1037, 1048, 1131, 1220, 1253, 1273, 1394, 1494, 1499, 1512, 1557, 1570, 1575, 1596, 1602, 1633, 1771, 1854, 1904, 1913, 1928, 1951, 1995, 2100, 2150, 2248, 2254, 2280, 2435, 2494, 2501, 2597, 2598, 2742, 2776, 2810, 2824, 2842, 2843, 2849, 2907, 2929, 2934, 3040, 3043, 3306, 3369, 3386, 3390, 3410, 3534, 3751, 3755, 3858, 3862, 3872, 3929, 4000, 4118, 4154, 4206, 4257, 4283, 4286, 4350, 4480, 4535, 4574, 4582, 4961, 4966, 4979, 5009, 5089, 5106, 10, 142, 395, 452, 546, 610, 658, 695, 800, 1095, 1119, 1143, 1187, 1298, 1381, 1535, 1615, 1646, 1727, 1776, 1803, 1922, 2038, 2040, 2082, 2121, 2145, 2198, 2226, 2430, 2524, 2587, 2786, 2827, 2856, 2864, 3043, 3400, 3445, 3473, 3513, 3553, 3560, 3577, 3667, 3724, 3878, 3914, 4105, 4111, 4408, 4418, 4430, 4439, 4459, 4542, 4748, 4750, 4779, 4845, 4968, 4999, 5007, 5025, 5055, 5146, 10, 33, 123, 131, 134, 169, 225, 235, 309, 386, 563, 630, 635, 681, 720, 797, 800, 947, 1025, 1060, 1306, 1404, 1539, 1559, 1607, 1622, 1635, 1758, 1780, 1845, 2096, 2175, 2225, 2227, 2239, 2267, 2471, 2481, 2493, 2555, 2638, 2720, 2745, 2772, 2877, 2916, 2939, 2993, 3008, 3011, 3190, 3260, 3345, 3422, 3534, 3593, 3696, 3920, 4012, 4029, 4057, 4065, 4234, 4318, 4334, 4385, 4396, 4434, 4515, 4535, 4554, 4567, 4612, 4625, 4715, 4726, 4769, 4786, 4801, 4849, 4909, 5014, 5039, 5079, 37, 85, 224, 225, 229, 238, 280, 285, 305, 395, 458, 689, 703, 752, 763, 768, 777, 801, 822, 969, 971, 1060, 1073, 1149, 1186, 1189, 1244, 1260, 1456, 1463, 1565, 1640, 1681, 1855, 1867, 1911, 1946, 1997, 2051, 2056, 2173, 2225, 2259, 2386, 2389, 2582, 2606, 2633, 2698, 2717, 2764, 2794, 2806, 2814, 2846, 2851, 2917, 2935, 3011, 3028, 3093, 3116, 3244, 3323, 3347, 3356, 3358, 3423, 3512, 3514, 3596, 3681, 3690, 3702, 3790, 3875, 3886, 3957, 4006, 4213, 4306, 4406, 4459, 4471, 4481, 4545, 4623, 4659, 4669, 4705, 4761, 4797, 4798, 4824, 4843, 4857, 4874, 4910, 4966, 4984, 5007, 5039, 79, 195, 221, 283, 289, 446, 499, 509, 590, 616, 747, 758, 832, 846, 1067, 1115, 1174, 1176, 1218, 1236, 1241, 1253, 1321, 1373, 1427, 1514, 1537, 1590, 1612, 1816, 1833, 1834, 1874, 1954, 2111, 2300, 2331, 2349, 2524, 2616, 2617, 2717, 2765, 2970, 3118, 3177, 3286, 3292, 3306, 3318, 3350, 3436, 3473, 3594, 3663, 3825, 3847, 3954, 3988, 4096, 4163, 4311, 4367, 4565, 4676, 4831, 4879, 4971, 4985, 5002, 5040, 373, 490, 534, 546, 705, 747, 751, 776, 830, 990, 1054, 1155, 1196, 1204, 1244, 1350, 1429, 1497, 1692, 1796, 1847, 1938, 1967, 2106, 2265, 2344, 2418, 2495, 2672, 2718, 2759, 2827, 2872, 2916, 3041, 3136, 3265, 3522, 3684, 3912, 4006, 4025, 4053, 4260, 4384, 4525, 4527, 4554, 4895, 4905, 4988, 5144, 5163, 104, 160, 166, 209, 229, 297, 318, 375, 378, 404, 460, 557, 629, 646, 672, 681, 813, 1016, 1025, 1029, 1032, 1052, 1105, 1124, 1128, 1171, 1195, 1205, 1218, 1220, 1350, 1466, 1499, 1522, 1525, 1538, 1604, 1664, 1668, 1678, 1704, 1771, 1786, 1793, 1928, 1944, 2042, 2080, 2206, 2210, 2223, 2311, 2320, 2371, 2394, 2490, 2493, 2561, 2564, 2704, 2780, 2828, 2888, 2897, 2954, 3000, 3016, 3079, 3227, 3273, 3277, 3396, 3397, 3429, 3461, 3493, 3512, 3513, 3520, 3555, 3582, 3666, 3672, 3682, 3697, 3698, 3746, 3793, 3807, 3808, 3816, 3825, 3851, 3908, 3957, 4065, 4095, 4134, 4284, 4294, 4349, 4412, 4529, 4541, 4571, 4605, 4633, 4640, 4657, 4660, 4676, 4709, 4742, 4767, 4793, 4867, 4883, 4988, 5013, 5018, 5024, 5034, 5045, 5103, 191, 233, 248, 592, 616, 645, 744, 758, 829, 916, 934, 979, 1383, 1404, 1427, 1514, 1588, 1615, 1683, 1867, 1885, 2057, 2061, 2323, 2327, 2371, 2597, 2609, 2674, 2809, 2891, 2892, 3080, 3120, 3235, 3294, 3326, 3363, 3513, 3582, 3604, 3699, 3724, 3971, 4012, 4148, 4188, 4240, 4300, 4345, 4361, 4593, 4601, 4633, 4657, 4690, 4697, 4814, 5043, 19, 92, 144, 170, 177, 224, 226, 232, 248, 360, 365, 385, 395, 536, 555, 556, 600, 618, 642, 696, 725, 727, 783, 808, 829, 846, 902, 926, 948, 966, 974, 1030, 1047, 1058, 1121, 1150, 1183, 1207, 1218, 1220, 1236, 1253, 1321, 1337, 1351, 1352, 1427, 1546, 1567, 1569, 1574, 1688, 1721, 1722, 1793, 1814, 1870, 1919, 1939, 2064, 2082, 2090, 2130, 2154, 2185, 2224, 2321, 2325, 2340, 2355, 2391, 2394, 2408, 2444, 2471, 2514, 2523, 2545, 2555, 2563, 2577, 2609, 2613, 2617, 2653, 2698, 2714, 2721, 2758, 2763, 2820, 2843, 2916, 2922, 2963, 2977, 3034, 3054, 3063, 3066, 3085, 3099, 3100, 3118, 3137, 3190, 3210, 3234, 3282, 3323, 3326, 3348, 3369, 3372, 3389, 3435, 3437, 3439, 3450, 3454, 3458, 3484, 3494, 3520, 3598, 3605, 3613, 3641, 3652, 3696, 3768, 3808, 3813, 3815, 3821, 3861, 3880, 3912, 3918, 4019, 4040, 4087, 4092, 4095, 4171, 4208, 4317, 4350, 4361, 4394, 4406, 4408, 4502, 4511, 4544, 4549, 4569, 4584, 4669, 4672, 4697, 4702, 4731, 4738, 4816, 4827, 4851, 4873, 4946, 4985, 5007, 5013, 5022, 5065, 5170, 323, 524, 891, 941, 1818, 2537, 2569, 2841, 2890, 3532, 3635, 4048, 4117, 4122, 4187, 4961, 5059, 5099, 175, 4359, 7, 37, 75, 95, 107, 108, 112, 160, 283, 318, 369, 376, 392, 412, 423, 457, 458, 479, 526, 549, 557, 598, 604, 635, 680, 701, 728, 747, 756, 875, 883, 885, 890, 910, 944, 963, 971, 985, 1041, 1070, 1083, 1098, 1131, 1233, 1260, 1273, 1340, 1353, 1433, 1448, 1463, 1473, 1490, 1531, 1545, 1546, 1551, 1610, 1623, 1645, 1665, 1711, 1722, 1729, 1735, 1777, 1811, 1819, 1834, 1847, 1854, 1873, 1912, 1922, 1945, 1947, 2003, 2044, 2049, 2072, 2108, 2173, 2184, 2225, 2335, 2350, 2408, 2465, 2471, 2552, 2577, 2616, 2682, 2700, 2727, 2832, 2855, 2857, 2861, 2885, 2898, 2905, 2922, 3072, 3150, 3173, 3177, 3198, 3207, 3273, 3286, 3292, 3305, 3306, 3356, 3386, 3400, 3523, 3527, 3528, 3594, 3681, 3732, 3814, 3843, 3880, 3886, 3974, 4011, 4047, 4049, 4058, 4074, 4081, 4095, 4189, 4207, 4226, 4228, 4238, 4251, 4254, 4257, 4300, 4317, 4323, 4327, 4418, 4440, 4449, 4485, 4493, 4508, 4524, 4545, 4574, 4597, 4628, 4647, 4650, 4660, 4688, 4691, 4700, 4707, 4715, 4738, 4740, 4754, 4767, 4768, 4787, 4865, 4876, 4879, 4893, 4955, 5013, 5023, 5075, 5087, 5099, 5121, 5126, 5144, 32, 35, 37, 162, 271, 290, 320, 428, 592, 671, 710, 796, 870, 923, 971, 974, 988, 998, 1013, 1060, 1066, 1111, 1135, 1241, 1244, 1271, 1323, 1337, 1367, 1401, 1406, 1455, 1530, 1565, 1625, 1660, 1664, 1683, 1704, 1723, 1847, 1855, 1872, 1907, 1932, 1991, 2024, 2031, 2036, 2288, 2298, 2346, 2419, 2526, 2565, 2606, 2609, 2617, 2671, 2674, 2694, 2833, 2846, 2851, 2864, 2919, 2954, 2985, 3040, 3041, 3050, 3116, 3315, 3323, 3490, 3557, 3566, 3579, 3606, 3667, 3690, 3699, 3702, 3751, 3781, 3793, 3795, 3868, 3895, 4094, 4250, 4323, 4336, 4382, 4384, 4412, 4549, 4586, 4629, 4653, 4764, 4771, 4789, 4831, 4864, 4870, 4874, 4938, 4989, 5045, 5079, 60, 95, 145, 209, 224, 257, 258, 511, 538, 550, 553, 585, 600, 752, 971, 1044, 1176, 1202, 1313, 1407, 1443, 1466, 1477, 1514, 1646, 1664, 1729, 1954, 2476, 2569, 2660, 2734, 2854, 3526, 3534, 3962, 4058, 4126, 4134, 4213, 4257, 4350, 4356, 4431, 4789, 4805, 4817, 4843, 4970, 4971, 5057, 2423, 2829, 3063, 4098, 2083, 2259, 4533, 138, 177, 266, 288, 313, 345, 396, 500, 645, 651, 677, 723, 747, 773, 796, 814, 827, 844, 848, 919, 969, 974, 982, 1029, 1091, 1096, 1122, 1149, 1206, 1325, 1381, 1394, 1426, 1455, 1529, 1532, 1712, 1797, 1810, 1847, 1892, 1997, 2004, 2085, 2234, 2267, 2337, 2351, 2382, 2384, 2425, 2494, 2542, 2555, 2617, 2659, 2662, 2686, 2745, 2749, 2893, 2905, 3060, 3146, 3363, 3522, 3527, 3581, 3609, 3656, 3690, 3701, 3775, 3777, 3903, 4017, 4030, 4052, 4060, 4117, 4291, 4311, 4331, 4373, 4384, 4459, 4488, 4531, 4742, 4759, 4817, 4894, 4900, 4912, 5025, 5050, 5080, 5144, 5161, 106, 217, 244, 379, 517, 536, 550, 595, 646, 715, 743, 833, 1189, 1278, 1546, 1570, 1575, 1640, 1642, 1820, 1863, 1868, 1995, 2051, 2054, 2074, 2172, 2188, 2194, 2213, 2316, 2391, 2395, 2470, 2609, 2700, 2824, 2846, 2849, 2919, 3071, 3112, 3116, 3158, 3225, 3272, 3345, 3362, 3364, 3372, 3392, 3406, 3439, 3472, 3682, 3748, 3795, 3845, 3893, 3932, 3953, 4122, 4233, 4303, 4384, 4466, 4557, 4586, 4603, 4699, 4738, 4752, 4798, 4828, 4838, 4936, 5040, 5099, 5110, 5115, 5164, 5170, 81, 235, 1273, 1539, 2768, 3364, 4576, 28, 1336, 3154, 3725, 4535, 2905, 20, 79, 151, 171, 226, 248, 266, 480, 525, 612, 690, 701, 810, 827, 848, 851, 990, 1025, 1028, 1035, 1056, 1064, 1066, 1135, 1146, 1219, 1233, 1290, 1302, 1329, 1331, 1451, 1497, 1569, 1588, 1637, 1641, 1732, 1759, 1814, 1831, 1835, 1836, 1985, 2025, 2027, 2096, 2293, 2325, 2347, 2373, 2726, 2819, 2913, 2981, 3020, 3126, 3280, 3307, 3438, 3478, 3610, 3659, 3696, 3740, 3814, 3832, 3861, 3962, 3971, 3976, 4006, 4034, 4082, 4251, 4300, 4406, 4413, 4488, 4498, 4545, 4637, 4640, 4708, 4729, 4805, 4893, 4920, 4925, 4936, 4968, 5062, 137, 240, 389, 416, 424, 443, 549, 617, 875, 1081, 1137, 1325, 1326, 1331, 1519, 1644, 1680, 1818, 1906, 2211, 2234, 2306, 2374, 2431, 2469, 2524, 2569, 2627, 2698, 2818, 2842, 2870, 2924, 2988, 2992, 3015, 3052, 3074, 3149, 3276, 3585, 3614, 3682, 3719, 3746, 4055, 4200, 4204, 4222, 4305, 4493, 4507, 4597, 4615, 4729, 4764, 4797, 5157, 5169, 93, 120, 446, 1210, 1367, 1467, 1490, 1598, 1649, 1704, 1732, 1826, 2737, 3073, 3116, 3255, 3549, 3714, 3822, 4144, 4164, 4337, 4449, 4690</t>
+    <t>96.81</t>
+  </si>
+  <si>
+    <t>5008</t>
+  </si>
+  <si>
+    <t>93, 287, 310, 375, 432, 852, 1205, 1302, 1564, 1613, 1735, 1834, 1997, 2042, 2425, 2460, 2465, 2708, 2782, 2849, 3270, 3273, 3513, 3531, 3968, 4000, 4002, 4262, 4354, 4563, 5024, 5032, 5106, 5112, 20, 567, 635, 827, 1336, 1524, 1932, 2451, 2585, 2764, 2993, 3066, 3659, 4187, 4423, 4657, 5136, 199, 297, 517, 549, 567, 640, 883, 1057, 1177, 1362, 1484, 1496, 1716, 1846, 1879, 1954, 2046, 2100, 2346, 2404, 2419, 2449, 2590, 2616, 2646, 2653, 2659, 2788, 2833, 2952, 3059, 3126, 3156, 3205, 3249, 3464, 3501, 3624, 3767, 4053, 4079, 4153, 4366, 4466, 4569, 4733, 5009, 5113, 79, 142, 177, 467, 517, 677, 721, 737, 751, 832, 979, 1060, 1077, 1171, 1236, 1348, 1479, 1503, 1509, 1531, 1570, 1610, 1669, 1719, 1820, 1831, 1874, 1878, 1905, 1940, 2012, 2027, 2250, 2316, 2356, 2413, 2427, 2470, 2511, 2672, 2806, 2809, 2864, 3020, 3033, 3184, 3225, 3280, 3308, 3313, 3468, 3474, 3513, 3681, 3708, 3845, 3851, 3862, 3866, 3895, 3931, 4037, 4123, 4206, 4250, 4320, 4359, 4366, 4402, 4478, 4586, 4596, 4661, 4686, 4714, 4752, 4789, 4793, 4912, 4931, 5040, 5089, 5138, 3, 6, 108, 116, 187, 199, 257, 286, 331, 332, 336, 357, 365, 411, 455, 507, 510, 546, 574, 606, 607, 608, 618, 629, 672, 712, 730, 751, 805, 852, 870, 880, 897, 917, 937, 944, 945, 1024, 1060, 1096, 1102, 1150, 1155, 1239, 1245, 1251, 1298, 1306, 1337, 1373, 1396, 1401, 1455, 1473, 1491, 1494, 1499, 1511, 1515, 1533, 1537, 1549, 1564, 1592, 1609, 1637, 1688, 1691, 1712, 1844, 1878, 1890, 1911, 1929, 1944, 1967, 2053, 2074, 2090, 2125, 2128, 2131, 2143, 2149, 2230, 2256, 2262, 2344, 2345, 2346, 2354, 2449, 2461, 2479, 2504, 2578, 2615, 2619, 2627, 2630, 2650, 2671, 2741, 2757, 2763, 2801, 2825, 2861, 2872, 2876, 2893, 2922, 2928, 2944, 2950, 2964, 2977, 2998, 3022, 3036, 3087, 3099, 3135, 3198, 3323, 3326, 3339, 3340, 3348, 3350, 3367, 3375, 3380, 3487, 3512, 3536, 3604, 3605, 3612, 3635, 3692, 3741, 3762, 3771, 3776, 3821, 3836, 3895, 3908, 3917, 3962, 4039, 4052, 4053, 4065, 4089, 4111, 4133, 4141, 4154, 4213, 4254, 4269, 4271, 4318, 4382, 4395, 4408, 4413, 4435, 4478, 4525, 4550, 4561, 4565, 4568, 4573, 4603, 4637, 4640, 4669, 4693, 4736, 4768, 4775, 4817, 4910, 4940, 4969, 4978, 5007, 5018, 5043, 5101, 5122, 287, 308, 320, 331, 446, 467, 519, 545, 604, 729, 1025, 1031, 1535, 1777, 1788, 1806, 1898, 1933, 1947, 1984, 2021, 2137, 2185, 2211, 2272, 2280, 2306, 2434, 2484, 2559, 2591, 2616, 2636, 2802, 2837, 2849, 2854, 2893, 2928, 2977, 3073, 3154, 3163, 3177, 3339, 3366, 3406, 3443, 3490, 3520, 3527, 3559, 3581, 3698, 3755, 3769, 3860, 3862, 3875, 4006, 4025, 4188, 4193, 4318, 4350, 4397, 4610, 4620, 4630, 4774, 4799, 4847, 4857, 4860, 4863, 4882, 4914, 4940, 5001, 5100, 5112, 5121, 5129, 14, 48, 89, 106, 119, 120, 230, 267, 271, 273, 287, 297, 344, 360, 398, 455, 484, 536, 581, 587, 640, 777, 778, 796, 827, 923, 933, 938, 947, 979, 987, 1037, 1046, 1056, 1064, 1084, 1091, 1102, 1111, 1115, 1137, 1172, 1187, 1195, 1216, 1233, 1248, 1275, 1298, 1304, 1308, 1321, 1367, 1372, 1406, 1465, 1531, 1564, 1570, 1612, 1623, 1741, 1831, 1861, 1867, 1886, 1894, 1911, 1917, 1922, 1925, 1931, 1967, 2031, 2044, 2063, 2068, 2083, 2087, 2108, 2126, 2221, 2222, 2239, 2264, 2283, 2295, 2302, 2340, 2358, 2384, 2540, 2553, 2576, 2595, 2627, 2651, 2746, 2780, 2781, 2800, 2818, 2824, 2919, 2929, 2967, 3018, 3050, 3061, 3069, 3085, 3125, 3225, 3245, 3248, 3267, 3279, 3315, 3320, 3334, 3369, 3372, 3439, 3479, 3501, 3577, 3590, 3627, 3658, 3705, 3707, 3724, 3766, 3813, 3860, 3868, 3886, 3892, 3915, 3950, 4006, 4052, 4087, 4096, 4097, 4111, 4251, 4259, 4294, 4323, 4395, 4408, 4467, 4480, 4568, 4591, 4625, 4653, 4733, 4754, 4799, 4827, 4843, 4859, 4882, 4985, 5025, 5043, 5094, 5108, 5121, 5124, 5164, 37, 106, 160, 169, 179, 209, 228, 230, 262, 348, 350, 392, 404, 460, 541, 550, 557, 584, 600, 610, 629, 668, 671, 684, 695, 715, 771, 810, 835, 869, 934, 1011, 1081, 1095, 1105, 1139, 1205, 1401, 1445, 1463, 1475, 1492, 1515, 1533, 1565, 1625, 1635, 1669, 1814, 1940, 1955, 1959, 1970, 2054, 2080, 2084, 2098, 2118, 2131, 2171, 2194, 2230, 2234, 2241, 2246, 2283, 2371, 2374, 2473, 2500, 2560, 2622, 2660, 2727, 2736, 2746, 2928, 2934, 3173, 3245, 3317, 3384, 3405, 3410, 3421, 3507, 3512, 3542, 3552, 3594, 3634, 3645, 3656, 3707, 3740, 3768, 3779, 3844, 3874, 3893, 3894, 3943, 4002, 4074, 4078, 4091, 4231, 4235, 4250, 4261, 4348, 4410, 4419, 4550, 4570, 4584, 4601, 4668, 4669, 4672, 4704, 4710, 4744, 4750, 4793, 4857, 4920, 5103, 5143, 57, 109, 240, 885, 905, 2056, 2241, 2377, 2722, 2977, 5014, 5147, 81, 345, 405, 1105, 1269, 1492, 1954, 2160, 2241, 2491, 2690, 2928, 3071, 3190, 3302, 3655, 3893, 4235, 4857, 5103, 107, 221, 229, 266, 587, 652, 709, 778, 890, 948, 1002, 1053, 1083, 1087, 1096, 1239, 1352, 1407, 1441, 1567, 1663, 1664, 1729, 1774, 1847, 1954, 1967, 2021, 2137, 2285, 2451, 2453, 2472, 2504, 2524, 2526, 2584, 2594, 2600, 2700, 2856, 2913, 2981, 3011, 3015, 3108, 3114, 3117, 3125, 3149, 3266, 3301, 3356, 3420, 3480, 3496, 3688, 3724, 3738, 3803, 3889, 3971, 3996, 4034, 4040, 4076, 4078, 4082, 4087, 4123, 4141, 4163, 4295, 4451, 4479, 4485, 4631, 4654, 4759, 4826, 4883, 5024, 0, 28, 46, 86, 90, 99, 107, 116, 233, 343, 353, 366, 481, 495, 504, 524, 555, 567, 584, 597, 600, 623, 635, 643, 644, 652, 689, 690, 714, 744, 905, 927, 988, 1008, 1024, 1032, 1098, 1120, 1128, 1160, 1187, 1197, 1205, 1211, 1267, 1269, 1323, 1350, 1425, 1477, 1512, 1537, 1648, 1654, 1712, 1720, 1735, 1780, 1816, 1831, 1890, 1904, 1928, 1947, 2047, 2054, 2069, 2125, 2178, 2222, 2226, 2235, 2253, 2260, 2265, 2289, 2408, 2418, 2453, 2469, 2475, 2494, 2570, 2580, 2682, 2734, 2765, 2809, 2824, 2841, 2868, 2892, 2903, 2916, 2934, 2985, 2989, 3020, 3036, 3147, 3296, 3308, 3337, 3388, 3399, 3401, 3406, 3439, 3479, 3498, 3547, 3549, 3599, 3604, 3609, 3619, 3624, 3627, 3663, 3674, 3701, 3771, 3795, 3849, 3911, 3963, 3975, 4012, 4074, 4092, 4134, 4149, 4154, 4193, 4247, 4260, 4265, 4269, 4303, 4346, 4402, 4419, 4546, 4568, 4619, 4623, 4625, 4654, 4726, 4748, 4750, 4827, 4847, 4960, 4999, 5032, 5096, 5097, 5110, 5126, 5136, 5138, 5147, 308, 1032, 2210, 2250, 2714, 3276, 3552, 3908, 4317, 33, 47, 57, 90, 95, 109, 283, 309, 320, 325, 363, 369, 412, 508, 572, 590, 640, 645, 727, 737, 768, 792, 913, 930, 933, 967, 974, 982, 999, 1051, 1058, 1121, 1367, 1511, 1633, 1692, 1712, 1735, 1741, 1766, 1767, 1820, 1849, 1874, 1880, 1898, 1922, 1978, 1988, 2029, 2054, 2057, 2084, 2168, 2244, 2268, 2288, 2295, 2316, 2324, 2344, 2360, 2397, 2403, 2475, 2523, 2540, 2622, 2649, 2652, 2704, 2755, 2779, 2892, 2897, 2952, 2963, 2967, 3011, 3033, 3036, 3061, 3143, 3144, 3227, 3235, 3244, 3266, 3290, 3293, 3331, 3356, 3383, 3396, 3456, 3457, 3464, 3522, 3529, 3557, 3574, 3652, 3663, 3669, 3751, 3793, 3971, 4017, 4033, 4067, 4103, 4126, 4163, 4188, 4222, 4240, 4250, 4272, 4348, 4350, 4366, 4406, 4423, 4510, 4531, 4619, 4631, 4673, 4690, 4726, 4748, 4786, 4814, 4873, 4899, 4922, 5025, 5032, 5080, 5158, 0, 14, 47, 63, 90, 93, 102, 131, 137, 142, 152, 175, 177, 199, 219, 221, 290, 299, 392, 418, 489, 497, 517, 632, 672, 701, 760, 838, 872, 915, 919, 927, 1038, 1057, 1058, 1194, 1204, 1211, 1259, 1298, 1321, 1351, 1451, 1496, 1518, 1559, 1603, 1629, 1645, 1678, 1723, 1735, 1769, 1782, 1811, 1829, 1853, 1880, 1894, 1905, 1927, 1941, 1978, 2018, 2128, 2158, 2166, 2210, 2213, 2217, 2223, 2226, 2289, 2321, 2345, 2351, 2355, 2395, 2435, 2451, 2490, 2553, 2581, 2597, 2612, 2622, 2629, 2654, 2718, 2723, 2731, 2788, 2807, 2825, 2843, 2861, 2890, 2915, 2926, 2935, 2950, 2981, 2983, 2988, 3007, 3127, 3157, 3225, 3248, 3277, 3280, 3296, 3302, 3348, 3366, 3388, 3443, 3445, 3461, 3477, 3547, 3550, 3602, 3610, 3644, 3699, 3718, 3746, 3768, 3815, 3833, 3854, 3979, 4029, 4047, 4094, 4095, 4105, 4133, 4152, 4193, 4294, 4353, 4365, 4381, 4396, 4410, 4423, 4506, 4510, 4531, 4563, 4574, 4597, 4653, 4670, 4688, 4699, 4738, 4775, 4787, 4831, 4852, 4857, 4865, 4870, 4913, 4964, 4969, 4978, 5016, 5027, 5033, 5043, 5046, 5096, 5101, 5112, 5123, 5165, 19, 37, 74, 211, 225, 273, 336, 348, 410, 522, 538, 577, 650, 652, 952, 958, 1137, 1138, 1166, 1187, 1538, 1544, 1555, 1559, 1570, 1646, 1693, 1697, 1712, 1719, 1820, 1880, 1922, 1991, 2168, 2223, 2239, 2244, 2292, 2397, 2540, 2606, 2637, 2726, 2816, 2827, 2981, 3207, 3235, 3244, 3292, 3383, 3388, 3391, 3423, 3545, 3663, 3707, 3861, 3945, 3976, 4039, 4133, 4142, 4217, 4287, 4303, 4523, 4603, 4713, 4733, 4775, 4805, 4874, 4900, 4910, 4920, 4928, 4967, 4970, 4986, 5022, 5089, 24, 75, 118, 186, 233, 238, 258, 318, 360, 398, 796, 952, 1059, 1095, 1188, 1280, 1360, 1465, 1522, 1777, 2042, 2056, 2118, 2143, 2158, 2321, 2395, 2460, 2557, 2581, 2681, 2736, 2986, 3112, 3122, 3137, 3155, 3214, 3241, 3302, 3334, 3356, 3429, 3445, 3501, 3570, 3594, 3644, 4030, 4223, 4354, 4396, 4507, 4544, 4563, 4574, 4646, 4738, 4744, 4895, 4968, 5034, 36, 111, 229, 234, 273, 422, 423, 462, 525, 536, 564, 610, 627, 748, 795, 801, 826, 854, 866, 880, 905, 999, 1002, 1052, 1083, 1092, 1124, 1155, 1212, 1268, 1285, 1409, 1545, 1634, 1667, 1671, 1722, 1770, 1782, 1793, 1796, 1837, 1845, 1874, 1922, 2012, 2018, 2050, 2082, 2106, 2145, 2162, 2226, 2275, 2300, 2311, 2423, 2453, 2461, 2519, 2523, 2559, 2590, 2606, 2648, 2652, 2718, 2742, 2856, 2876, 2915, 2944, 2985, 3011, 3042, 3052, 3087, 3115, 3207, 3209, 3283, 3302, 3367, 3605, 3645, 3827, 3912, 3968, 4064, 4076, 4206, 4221, 4226, 4320, 4327, 4334, 4431, 4541, 4592, 4620, 4630, 4702, 4703, 4735, 4775, 4779, 4928, 4944, 5009, 5163, 31, 131, 585, 734, 831, 1042, 1058, 1451, 1489, 1581, 1782, 1799, 1948, 1996, 2018, 2173, 2508, 2537, 2541, 2597, 2716, 2718, 2722, 2975, 3068, 3449, 3816, 4060, 4119, 4171, 4439, 4526, 4563, 4572, 4669, 4708, 4729, 4810, 4813, 4883, 5025, 5046, 5094, 5117, 0, 93, 123, 218, 229, 256, 263, 291, 329, 435, 446, 481, 511, 522, 524, 549, 555, 577, 603, 607, 645, 660, 682, 948, 1060, 1076, 1086, 1215, 1244, 1394, 1549, 1660, 1689, 1711, 1828, 1881, 1905, 1919, 1987, 1995, 2069, 2116, 2210, 2247, 2362, 2404, 2413, 2415, 2501, 2534, 2561, 2629, 2837, 2849, 2933, 2967, 3008, 3054, 3126, 3212, 3318, 3337, 3397, 3513, 3594, 3624, 3666, 3719, 3755, 3908, 4051, 4079, 4087, 4119, 4147, 4171, 4199, 4316, 4353, 4385, 4389, 4498, 4506, 4513, 4710, 4821, 4994, 5057, 5112, 549, 938, 1248, 1801, 2085, 2247, 2415, 3008, 3464, 3624, 4754, 5112, 69, 145, 158, 263, 273, 283, 320, 332, 375, 482, 682, 709, 1090, 1136, 1201, 1236, 1248, 1469, 1648, 1759, 1763, 1776, 1786, 1797, 1821, 1826, 2054, 2055, 2080, 2116, 2117, 2268, 2289, 2302, 2399, 2408, 2426, 2449, 2479, 2536, 2600, 2615, 2653, 2696, 2716, 2755, 2761, 2978, 2981, 2985, 2988, 3000, 3120, 3125, 3165, 3179, 3362, 3363, 3423, 3645, 3795, 3808, 3832, 3836, 3923, 4039, 4040, 4181, 4218, 4231, 4250, 4259, 4316, 4336, 4467, 4520, 4539, 4586, 4650, 4690, 4700, 4711, 4767, 4864, 4900, 4946, 5034, 5042, 5050, 5085, 5109, 5112, 5138, 46, 85, 90, 95, 96, 167, 478, 589, 630, 699, 778, 830, 831, 866, 896, 933, 976, 1029, 1042, 1051, 1065, 1096, 1171, 1210, 1318, 1333, 1459, 1477, 1503, 1507, 1524, 1592, 1780, 1858, 1898, 2002, 2051, 2173, 2230, 2248, 2352, 2373, 2391, 2522, 2545, 2559, 2561, 2624, 2638, 2874, 3217, 3319, 3346, 3360, 3400, 3437, 3448, 3478, 3487, 3526, 3534, 3594, 3687, 3962, 4028, 4065, 4171, 4233, 4291, 4294, 4323, 4526, 4563, 4739, 4863, 4876, 4971, 4977, 5027, 5104, 89, 271, 338, 360, 777, 1205, 1321, 1463, 1623, 1984, 2320, 2786, 3230, 3245, 3248, 3705, 3861, 4653, 4750, 4783, 4843, 4857, 4931, 35, 199, 209, 227, 263, 290, 329, 353, 357, 400, 424, 481, 545, 608, 672, 696, 700, 705, 787, 792, 814, 851, 923, 987, 998, 1016, 1032, 1086, 1189, 1211, 1331, 1333, 1342, 1498, 1524, 1539, 1603, 1659, 1664, 1776, 1793, 1898, 1931, 1996, 2043, 2072, 2080, 2117, 2150, 2183, 2198, 2221, 2239, 2267, 2423, 2528, 2553, 2758, 2766, 2820, 2923, 2954, 3045, 3084, 3093, 3098, 3144, 3156, 3214, 3229, 3270, 3334, 3400, 3445, 3498, 3532, 3557, 3645, 3655, 3699, 3719, 3817, 3870, 3889, 3928, 3932, 3966, 4011, 4058, 4105, 4193, 4226, 4334, 4431, 4435, 4451, 4482, 4528, 4597, 4648, 4740, 4784, 4793, 4909, 4988, 5023, 5032, 5051, 5073, 5124, 5138, 28, 73, 75, 90, 112, 122, 137, 142, 225, 320, 410, 423, 545, 565, 604, 642, 682, 701, 725, 756, 809, 863, 1016, 1051, 1180, 1189, 1210, 1378, 1525, 1535, 1545, 1569, 1570, 1720, 1723, 1769, 1782, 1799, 1807, 1905, 2018, 2040, 2042, 2063, 2130, 2211, 2266, 2326, 2331, 2362, 2483, 2561, 2564, 2582, 2650, 2660, 2714, 2814, 2970, 2978, 3122, 3125, 3249, 3391, 3484, 3513, 3588, 3597, 3660, 3717, 3748, 3769, 3851, 3875, 4042, 4057, 4065, 4163, 4172, 4193, 4262, 4412, 4448, 4453, 4467, 4550, 4593, 4693, 4784, 4814, 4905, 4944, 4969, 4983, 5059, 5112, 5143, 5168, 411, 446, 577, 607, 715, 933, 982, 1042, 1351, 1515, 1689, 1806, 2494, 2849, 3284, 3484, 3569, 3997, 4418, 4669, 4743, 4887, 5046, 28, 107, 299, 660, 838, 1037, 1076, 1168, 1234, 1463, 1552, 1728, 1986, 2030, 2042, 2226, 2395, 2398, 2856, 3725, 3825, 3833, 4002, 4051, 4141, 4213, 4216, 4340, 4385, 4408, 4523, 4733, 4828, 4909, 5025, 5106, 32, 73, 74, 99, 121, 168, 287, 338, 366, 389, 392, 418, 443, 460, 462, 642, 727, 769, 813, 828, 860, 872, 933, 934, 959, 1158, 1177, 1212, 1260, 1290, 1502, 1567, 1641, 1690, 1759, 1796, 1807, 1839, 1847, 1855, 1894, 1912, 2038, 2061, 2128, 2144, 2183, 2353, 2490, 2493, 2514, 2555, 2582, 2680, 2706, 2801, 2824, 2837, 2949, 2981, 2995, 3008, 3026, 3060, 3070, 3118, 3161, 3184, 3276, 3326, 3391, 3397, 3461, 3474, 3576, 3658, 3831, 3836, 3872, 3880, 3916, 4155, 4259, 4354, 4359, 4385, 4563, 4618, 4669, 4690, 4717, 4844, 5021, 5108, 5113, 5169, 89, 151, 210, 555, 776, 880, 913, 979, 1011, 1103, 1115, 1372, 1484, 1712, 2030, 2221, 2408, 2761, 2837, 2963, 2966, 2984, 3043, 3059, 3110, 3265, 3365, 3486, 3762, 3997, 4064, 4097, 4254, 4269, 4274, 4526, 4582, 4736, 4743, 4837, 4838, 4841, 4844, 4865, 35, 162, 258, 343, 417, 477, 709, 860, 1186, 1259, 1297, 1308, 1645, 1675, 1927, 1995, 2084, 2167, 2194, 2217, 2260, 2320, 2346, 2484, 2581, 2585, 2659, 2786, 2817, 2842, 2868, 2938, 2989, 3103, 3136, 3201, 3301, 3427, 3486, 3513, 3738, 3790, 3802, 3886, 4091, 4092, 4213, 4284, 4440, 4515, 4633, 4774, 4831, 4882, 4894, 4960, 4968, 4982, 5021, 5100, 29, 83, 99, 151, 212, 251, 291, 296, 310, 313, 318, 481, 625, 635, 846, 1008, 1029, 1054, 1064, 1220, 1323, 1331, 1396, 1432, 1445, 1503, 1525, 1549, 1575, 1622, 1664, 1707, 1755, 1986, 2020, 2030, 2058, 2131, 2170, 2211, 2220, 2222, 2247, 2264, 2266, 2295, 2306, 2355, 2362, 2410, 2427, 2494, 2554, 2615, 2630, 2636, 2650, 2690, 2704, 2718, 2727, 2766, 2779, 2846, 2876, 2890, 3015, 3099, 3102, 3103, 3108, 3111, 3179, 3190, 3247, 3273, 3290, 3305, 3339, 3345, 3367, 3477, 3570, 3652, 3847, 3891, 3903, 3908, 3923, 3972, 4029, 4048, 4074, 4095, 4183, 4199, 4206, 4213, 4296, 4299, 4359, 4376, 4448, 4490, 4527, 4572, 4575, 4597, 4699, 4709, 4711, 4844, 4876, 4892, 4978, 4985, 5032, 5039, 5055, 5096, 5134, 5168, 64, 81, 144, 332, 396, 504, 652, 680, 771, 866, 987, 1171, 1303, 1441, 1496, 1502, 1544, 1797, 1996, 2031, 2042, 2084, 2121, 2170, 2266, 2293, 2339, 2526, 2528, 2583, 2590, 2662, 2696, 2868, 3016, 3033, 3051, 3292, 3340, 3365, 3563, 3574, 3918, 4022, 4042, 4075, 4079, 4135, 4201, 4303, 4456, 4501, 4553, 4667, 4821, 4879, 4883, 4948, 5103, 5104, 5121, 93, 111, 122, 169, 209, 210, 211, 218, 226, 238, 309, 323, 376, 385, 405, 427, 481, 488, 517, 555, 577, 584, 595, 608, 621, 642, 646, 658, 687, 712, 727, 773, 785, 829, 846, 848, 870, 933, 941, 966, 971, 985, 1024, 1037, 1073, 1105, 1147, 1217, 1233, 1259, 1275, 1323, 1364, 1374, 1409, 1443, 1453, 1479, 1480, 1514, 1559, 1567, 1596, 1649, 1654, 1675, 1691, 1720, 1780, 1804, 1810, 1834, 1868, 1874, 1885, 1905, 1944, 1945, 1948, 2049, 2061, 2063, 2070, 2088, 2093, 2126, 2223, 2239, 2268, 2271, 2327, 2489, 2560, 2590, 2624, 2685, 2700, 2724, 2756, 2766, 2843, 2848, 2857, 2879, 2919, 2933, 2935, 2954, 2964, 2997, 3029, 3043, 3070, 3084, 3099, 3108, 3111, 3116, 3146, 3157, 3237, 3264, 3356, 3391, 3397, 3457, 3472, 3478, 3504, 3541, 3570, 3582, 3660, 3701, 3740, 3746, 3795, 3821, 3827, 3875, 3884, 3912, 3929, 3934, 3970, 4028, 4074, 4091, 4103, 4162, 4170, 4200, 4201, 4206, 4214, 4256, 4260, 4286, 4306, 4382, 4388, 4413, 4429, 4439, 4533, 4541, 4550, 4633, 4661, 4668, 4705, 4713, 4726, 4769, 4784, 4870, 4886, 4928, 4948, 4994, 5027, 5043, 5057, 5097, 5113, 5123, 5124, 5138, 5156, 5163, 5168, 5170, 5172, 137, 142, 270, 363, 427, 460, 467, 590, 642, 681, 725, 744, 769, 808, 927, 998, 1016, 1024, 1041, 1045, 1051, 1098, 1108, 1172, 1233, 1290, 1325, 1342, 1374, 1378, 1441, 1463, 1538, 1546, 1565, 1570, 1645, 1678, 1799, 1810, 1814, 2036, 2129, 2147, 2149, 2426, 2431, 2541, 2572, 2697, 2717, 2736, 2820, 2870, 2890, 3244, 3249, 3339, 3367, 3375, 3396, 3437, 3472, 3481, 3498, 3663, 3708, 3727, 3769, 3811, 3875, 4028, 4076, 4091, 4103, 4122, 4222, 4226, 4312, 4449, 4550, 4624, 4733, 4787, 4811, 4814, 4816, 4857, 4967, 5094, 416, 499, 529, 549, 728, 838, 1064, 1108, 1494, 1575, 1621, 2029, 2264, 2498, 2855, 3015, 3190, 3201, 3276, 3407, 3416, 3458, 3614, 3696, 3751, 4204, 4299, 4482, 4493, 4601, 4827, 5157, 280, 291, 552, 1520, 1818, 1847, 1971, 2127, 2377, 2722, 2768, 2939, 3007, 3863, 4646, 5157, 35, 96, 256, 336, 348, 415, 443, 460, 554, 564, 685, 795, 796, 848, 875, 963, 982, 1013, 1052, 1067, 1100, 1176, 1305, 1469, 1613, 1616, 1764, 1816, 1834, 1890, 2083, 2108, 2206, 2210, 2225, 2349, 2394, 2473, 2864, 2907, 2915, 2993, 3026, 3076, 3087, 3143, 3158, 3284, 3318, 3457, 3503, 3582, 3627, 3688, 3765, 3913, 3928, 4032, 4042, 4087, 4103, 4111, 4113, 4135, 4200, 4201, 4240, 4271, 4425, 4528, 4549, 4561, 4565, 4615, 4752, 4850, 4940, 5094, 5156, 5159, 5169, 289, 814, 1246, 1604, 1668, 2259, 3020, 3122, 3880, 4140, 10, 47, 137, 266, 273, 464, 557, 566, 810, 1040, 1353, 1457, 1860, 1931, 2084, 2418, 2456, 2613, 2649, 2791, 3051, 3301, 3397, 3531, 3652, 3687, 3706, 3822, 3996, 4039, 4052, 4188, 4204, 4256, 4748, 5100, 168, 1570, 2149, 2167, 2555, 3974, 4899, 113, 273, 432, 481, 524, 554, 644, 682, 763, 971, 1040, 1087, 1348, 1409, 1489, 1514, 1532, 1567, 1579, 1609, 1612, 1721, 1851, 2042, 2068, 2085, 2097, 2271, 2583, 2672, 2717, 2738, 3149, 3334, 3619, 3836, 3851, 4207, 4278, 4481, 4506, 4542, 4750, 4976, 5134, 5149, 138, 191, 424, 1245, 1351, 1507, 1629, 1704, 1928, 2090, 2149, 2416, 2563, 2580, 2697, 3059, 3284, 3547, 3577, 3800, 3917, 3968, 4055, 4141, 4144, 4235, 4256, 4348, 4417, 4430, 4506, 4615, 4640, 4682, 4845, 4914, 4942, 4976, 4986, 48, 83, 137, 175, 202, 318, 329, 347, 350, 378, 524, 534, 570, 589, 592, 616, 680, 797, 800, 826, 1040, 1048, 1058, 1073, 1101, 1216, 1289, 1306, 1321, 1405, 1426, 1517, 1518, 1636, 1654, 1834, 1889, 1938, 2020, 2053, 2087, 2088, 2112, 2168, 2352, 2367, 2451, 2469, 2476, 2554, 2610, 2624, 2629, 2738, 2776, 2928, 2949, 2977, 2997, 3029, 3063, 3087, 3099, 3102, 3114, 3135, 3249, 3282, 3306, 3356, 3422, 3427, 3478, 3502, 3559, 3590, 3706, 3708, 3733, 3738, 3822, 3938, 3971, 3979, 4089, 4193, 4226, 4270, 4459, 4498, 4503, 4515, 4546, 4584, 4676, 4723, 4763, 4768, 4839, 4881, 4960, 5001, 0, 10, 48, 89, 99, 107, 119, 121, 137, 151, 174, 224, 271, 291, 317, 343, 379, 392, 458, 499, 523, 539, 554, 589, 593, 617, 621, 627, 643, 769, 803, 830, 851, 875, 891, 1001, 1006, 1081, 1087, 1137, 1138, 1183, 1220, 1245, 1304, 1323, 1325, 1331, 1340, 1358, 1381, 1402, 1457, 1496, 1567, 1615, 1626, 1634, 1648, 1674, 1712, 1729, 1769, 1774, 1801, 1843, 1898, 1906, 1948, 2020, 2031, 2040, 2070, 2084, 2133, 2153, 2193, 2194, 2239, 2264, 2296, 2326, 2345, 2354, 2391, 2465, 2476, 2591, 2597, 2617, 2623, 2627, 2649, 2759, 2760, 2818, 2841, 2842, 2877, 2884, 2903, 2917, 2919, 2933, 2997, 3029, 3043, 3074, 3080, 3085, 3124, 3125, 3179, 3187, 3198, 3230, 3240, 3248, 3265, 3320, 3322, 3339, 3428, 3478, 3479, 3529, 3617, 3663, 3682, 3708, 3767, 3769, 3821, 3870, 3884, 3893, 3915, 3950, 3955, 3968, 4025, 4067, 4074, 4079, 4094, 4097, 4103, 4250, 4260, 4346, 4404, 4409, 4479, 4482, 4500, 4612, 4664, 4682, 4696, 4709, 4714, 4816, 4931, 4944, 5001, 5014, 5055, 5087, 5165, 26, 74, 112, 163, 251, 314, 422, 523, 538, 642, 678, 828, 830, 906, 926, 941, 999, 1030, 1037, 1048, 1131, 1220, 1253, 1273, 1394, 1494, 1499, 1512, 1557, 1570, 1575, 1596, 1602, 1633, 1771, 1854, 1904, 1913, 1928, 1951, 1995, 2100, 2150, 2248, 2254, 2280, 2435, 2494, 2501, 2597, 2598, 2742, 2776, 2810, 2824, 2842, 2843, 2849, 2907, 2929, 2934, 3040, 3043, 3306, 3369, 3386, 3390, 3410, 3534, 3751, 3755, 3858, 3862, 3872, 3929, 4000, 4118, 4154, 4206, 4257, 4283, 4286, 4350, 4480, 4535, 4574, 4582, 4961, 4966, 4979, 5009, 5089, 5106, 10, 142, 395, 452, 546, 610, 658, 695, 800, 1095, 1119, 1143, 1187, 1298, 1381, 1535, 1615, 1646, 1727, 1776, 1803, 1922, 2038, 2040, 2082, 2121, 2145, 2198, 2226, 2430, 2524, 2587, 2786, 2827, 2856, 2864, 3043, 3400, 3445, 3473, 3513, 3553, 3560, 3577, 3667, 3724, 3878, 3914, 4105, 4111, 4408, 4418, 4430, 4439, 4459, 4542, 4748, 4750, 4779, 4845, 4968, 4999, 5007, 5025, 5055, 5146, 10, 33, 123, 131, 134, 169, 225, 235, 309, 386, 563, 630, 635, 681, 720, 797, 800, 947, 1025, 1060, 1306, 1404, 1539, 1559, 1607, 1622, 1635, 1758, 1780, 1845, 2096, 2175, 2225, 2227, 2239, 2267, 2471, 2481, 2493, 2555, 2638, 2720, 2745, 2772, 2877, 2916, 2939, 2993, 3008, 3011, 3190, 3260, 3345, 3422, 3534, 3593, 3696, 3920, 4012, 4029, 4057, 4065, 4234, 4318, 4334, 4385, 4396, 4434, 4515, 4535, 4554, 4567, 4612, 4625, 4715, 4726, 4769, 4786, 4801, 4849, 4909, 5014, 5039, 5079, 37, 85, 224, 225, 229, 238, 280, 285, 305, 395, 458, 689, 703, 752, 763, 768, 777, 801, 822, 969, 971, 1060, 1073, 1149, 1186, 1189, 1244, 1260, 1456, 1463, 1565, 1640, 1681, 1855, 1867, 1911, 1946, 1997, 2051, 2056, 2173, 2225, 2259, 2386, 2389, 2582, 2606, 2633, 2698, 2717, 2764, 2794, 2806, 2814, 2846, 2851, 2917, 2935, 3011, 3028, 3093, 3116, 3244, 3323, 3347, 3356, 3358, 3423, 3512, 3514, 3596, 3681, 3690, 3702, 3790, 3875, 3886, 3957, 4006, 4213, 4306, 4406, 4459, 4471, 4481, 4545, 4623, 4659, 4669, 4705, 4761, 4797, 4798, 4824, 4843, 4857, 4874, 4910, 4966, 4984, 5007, 5039, 79, 195, 221, 283, 289, 446, 499, 509, 590, 616, 747, 758, 832, 846, 1067, 1115, 1174, 1176, 1218, 1236, 1241, 1253, 1321, 1373, 1427, 1514, 1537, 1590, 1612, 1816, 1833, 1834, 1874, 1954, 2111, 2300, 2331, 2349, 2524, 2616, 2617, 2717, 2765, 2970, 3118, 3177, 3286, 3292, 3306, 3318, 3350, 3436, 3473, 3594, 3663, 3825, 3847, 3954, 3988, 4096, 4163, 4311, 4367, 4565, 4676, 4831, 4879, 4971, 4985, 5002, 5040, 5126, 373, 490, 534, 546, 705, 747, 751, 776, 830, 990, 1054, 1155, 1196, 1204, 1244, 1350, 1429, 1497, 1692, 1796, 1847, 1938, 1967, 2106, 2265, 2344, 2418, 2495, 2672, 2718, 2759, 2827, 2872, 2916, 3041, 3136, 3265, 3522, 3684, 3912, 4006, 4025, 4053, 4260, 4384, 4525, 4527, 4554, 4895, 4905, 4988, 5144, 5163, 104, 160, 166, 209, 229, 297, 318, 375, 378, 404, 460, 557, 629, 646, 672, 681, 813, 1016, 1025, 1029, 1032, 1052, 1105, 1124, 1128, 1171, 1195, 1205, 1218, 1220, 1350, 1466, 1499, 1522, 1525, 1538, 1604, 1664, 1668, 1678, 1704, 1771, 1786, 1793, 1928, 1944, 2042, 2080, 2206, 2210, 2223, 2311, 2320, 2371, 2394, 2490, 2493, 2561, 2564, 2704, 2780, 2828, 2888, 2897, 2954, 3000, 3016, 3079, 3227, 3273, 3277, 3396, 3397, 3429, 3461, 3493, 3512, 3513, 3520, 3555, 3582, 3666, 3672, 3682, 3697, 3698, 3746, 3793, 3807, 3808, 3816, 3825, 3851, 3908, 3957, 4065, 4095, 4134, 4284, 4294, 4349, 4412, 4529, 4541, 4571, 4605, 4633, 4640, 4657, 4660, 4676, 4709, 4742, 4767, 4793, 4867, 4883, 4988, 5013, 5018, 5024, 5034, 5045, 5103, 5124, 191, 233, 248, 592, 616, 645, 744, 758, 829, 916, 934, 979, 1383, 1404, 1427, 1514, 1588, 1615, 1683, 1867, 1885, 2057, 2061, 2323, 2327, 2371, 2597, 2609, 2674, 2809, 2891, 2892, 3080, 3120, 3235, 3294, 3326, 3363, 3513, 3582, 3604, 3699, 3724, 3971, 4012, 4148, 4188, 4240, 4300, 4345, 4361, 4593, 4601, 4633, 4657, 4690, 4697, 4814, 5043, 19, 92, 144, 170, 177, 224, 226, 232, 248, 360, 365, 385, 395, 536, 555, 556, 600, 618, 642, 696, 725, 727, 783, 808, 829, 846, 902, 926, 948, 966, 974, 1030, 1047, 1058, 1121, 1150, 1183, 1207, 1218, 1220, 1236, 1253, 1321, 1337, 1351, 1352, 1427, 1546, 1567, 1569, 1574, 1688, 1721, 1722, 1793, 1814, 1870, 1919, 1939, 2064, 2082, 2090, 2130, 2154, 2185, 2224, 2321, 2325, 2340, 2355, 2391, 2394, 2408, 2444, 2471, 2514, 2523, 2545, 2555, 2563, 2577, 2609, 2613, 2617, 2653, 2698, 2714, 2721, 2758, 2763, 2820, 2843, 2916, 2922, 2963, 2977, 3034, 3054, 3063, 3066, 3085, 3099, 3100, 3118, 3137, 3190, 3210, 3234, 3282, 3323, 3326, 3348, 3369, 3372, 3389, 3435, 3437, 3439, 3450, 3454, 3458, 3484, 3494, 3520, 3598, 3605, 3613, 3641, 3652, 3696, 3768, 3808, 3813, 3815, 3821, 3861, 3880, 3912, 3918, 4019, 4040, 4087, 4092, 4095, 4171, 4208, 4317, 4350, 4361, 4394, 4406, 4408, 4502, 4511, 4544, 4549, 4569, 4584, 4669, 4672, 4697, 4702, 4731, 4738, 4816, 4827, 4851, 4873, 4946, 4985, 5007, 5013, 5022, 5065, 5170, 175, 323, 524, 891, 941, 1818, 2537, 2569, 2841, 2890, 3532, 3635, 4048, 4117, 4122, 4187, 4359, 4961, 5059, 5099, 7, 37, 75, 95, 107, 108, 112, 160, 283, 318, 369, 376, 392, 412, 423, 457, 458, 479, 526, 549, 557, 598, 604, 635, 680, 701, 728, 747, 756, 875, 883, 885, 890, 910, 944, 963, 971, 985, 1041, 1070, 1083, 1098, 1131, 1233, 1260, 1273, 1340, 1353, 1433, 1448, 1463, 1473, 1490, 1531, 1545, 1546, 1551, 1610, 1623, 1645, 1665, 1711, 1722, 1729, 1735, 1777, 1811, 1819, 1834, 1847, 1854, 1873, 1912, 1922, 1945, 1947, 2003, 2044, 2049, 2072, 2108, 2173, 2184, 2225, 2335, 2350, 2408, 2465, 2471, 2552, 2577, 2616, 2682, 2700, 2727, 2832, 2855, 2857, 2861, 2885, 2898, 2905, 2922, 3072, 3150, 3173, 3177, 3198, 3207, 3273, 3286, 3292, 3305, 3306, 3356, 3386, 3400, 3523, 3527, 3528, 3594, 3681, 3732, 3814, 3843, 3880, 3886, 3974, 4011, 4047, 4049, 4058, 4074, 4081, 4095, 4189, 4207, 4226, 4228, 4238, 4251, 4254, 4257, 4300, 4317, 4323, 4327, 4418, 4440, 4449, 4485, 4493, 4508, 4524, 4545, 4574, 4597, 4628, 4647, 4650, 4660, 4688, 4691, 4700, 4707, 4715, 4738, 4740, 4754, 4767, 4768, 4787, 4865, 4876, 4879, 4893, 4955, 5013, 5023, 5075, 5087, 5099, 5121, 5126, 5144, 32, 35, 37, 162, 271, 290, 320, 428, 592, 671, 710, 796, 870, 923, 971, 974, 988, 998, 1013, 1060, 1066, 1111, 1135, 1241, 1244, 1271, 1323, 1337, 1367, 1401, 1406, 1455, 1530, 1565, 1625, 1660, 1664, 1683, 1704, 1723, 1847, 1855, 1872, 1907, 1932, 1991, 2024, 2031, 2036, 2288, 2298, 2346, 2419, 2526, 2565, 2606, 2609, 2617, 2671, 2674, 2694, 2833, 2846, 2851, 2864, 2919, 2954, 2985, 3040, 3041, 3050, 3116, 3315, 3323, 3490, 3557, 3566, 3579, 3606, 3667, 3690, 3699, 3702, 3751, 3781, 3793, 3795, 3868, 3895, 4094, 4250, 4323, 4336, 4382, 4384, 4412, 4549, 4586, 4629, 4653, 4764, 4771, 4789, 4831, 4864, 4870, 4874, 4938, 4989, 5045, 5079, 60, 95, 145, 209, 224, 257, 258, 511, 538, 550, 553, 585, 600, 752, 971, 1044, 1176, 1202, 1313, 1407, 1443, 1466, 1477, 1514, 1646, 1664, 1729, 1954, 2476, 2569, 2660, 2734, 2854, 3526, 3534, 3962, 4058, 4126, 4134, 4213, 4257, 4350, 4356, 4431, 4789, 4805, 4817, 4843, 4970, 4971, 5057, 2083, 2259, 2423, 2829, 3063, 4098, 4533, 138, 177, 266, 288, 313, 345, 396, 500, 645, 651, 677, 723, 747, 773, 796, 814, 827, 844, 848, 919, 969, 974, 982, 1029, 1091, 1096, 1122, 1149, 1206, 1325, 1381, 1394, 1426, 1455, 1529, 1532, 1712, 1797, 1810, 1847, 1892, 1997, 2004, 2085, 2234, 2267, 2337, 2351, 2382, 2384, 2425, 2494, 2542, 2555, 2617, 2659, 2662, 2686, 2745, 2749, 2893, 2905, 3060, 3146, 3363, 3522, 3527, 3581, 3609, 3656, 3690, 3701, 3775, 3777, 3903, 4017, 4030, 4052, 4060, 4117, 4291, 4311, 4331, 4373, 4384, 4459, 4488, 4531, 4742, 4759, 4817, 4894, 4900, 4912, 5025, 5050, 5080, 5144, 5161, 106, 217, 244, 379, 517, 536, 550, 595, 646, 715, 743, 833, 1189, 1278, 1546, 1570, 1575, 1640, 1642, 1820, 1863, 1868, 1995, 2051, 2054, 2074, 2172, 2188, 2194, 2213, 2316, 2391, 2395, 2470, 2609, 2700, 2824, 2846, 2849, 2919, 3071, 3112, 3116, 3158, 3225, 3272, 3345, 3362, 3364, 3372, 3392, 3406, 3439, 3472, 3682, 3748, 3795, 3845, 3893, 3932, 3953, 4122, 4233, 4303, 4384, 4466, 4557, 4586, 4603, 4699, 4738, 4752, 4798, 4828, 4838, 4936, 5040, 5099, 5110, 5115, 5164, 5170, 81, 235, 1273, 1539, 2768, 3364, 4576, 28, 1336, 2905, 3154, 3725, 4535, 20, 79, 151, 171, 226, 248, 266, 480, 525, 612, 690, 701, 810, 827, 848, 851, 990, 1025, 1028, 1035, 1056, 1064, 1066, 1135, 1146, 1219, 1233, 1290, 1302, 1329, 1331, 1451, 1497, 1569, 1588, 1637, 1641, 1732, 1759, 1814, 1831, 1835, 1836, 1985, 2025, 2027, 2096, 2293, 2325, 2347, 2373, 2726, 2819, 2913, 2981, 3020, 3126, 3280, 3307, 3438, 3478, 3610, 3659, 3696, 3740, 3814, 3832, 3861, 3962, 3971, 3976, 4006, 4034, 4082, 4251, 4300, 4406, 4413, 4488, 4498, 4545, 4637, 4640, 4708, 4729, 4805, 4893, 4920, 4925, 4936, 4968, 5062, 137, 240, 389, 416, 424, 443, 549, 617, 875, 1081, 1137, 1325, 1326, 1331, 1519, 1644, 1680, 1818, 1906, 2211, 2234, 2306, 2374, 2431, 2469, 2524, 2569, 2627, 2698, 2818, 2842, 2870, 2924, 2988, 2992, 3015, 3052, 3074, 3149, 3276, 3585, 3614, 3682, 3719, 3746, 4055, 4200, 4204, 4222, 4305, 4493, 4507, 4597, 4615, 4729, 4764, 4797, 5157, 5169, 93, 120, 446, 1210, 1367, 1467, 1490, 1598, 1649, 1704, 1732, 1826, 2737, 3073, 3116, 3255, 3549, 3714, 3822, 4144, 4164, 4337, 4449, 4690</t>
   </si>
   <si>
     <t>98.86</t>
@@ -821,6 +821,21 @@
   </si>
   <si>
     <t>0, 2, 3, 7, 11, 12, 13, 17, 22, 26, 30, 34, 38, 39, 48, 58, 60, 65, 66, 68, 74, 78, 85, 87, 91, 93, 94, 98, 99, 100, 105, 108, 111, 112, 119, 130, 132, 135, 136, 145, 151, 157, 158, 161, 167, 168, 169, 170, 182, 186, 189, 194, 195, 196, 198, 199, 204, 206, 207, 208, 216, 217, 218, 220, 223, 225, 229, 233, 238, 239, 240, 245, 250, 255, 257, 259, 260, 266, 267, 269, 271, 275, 277, 282, 283, 288, 292, 293, 294, 298, 301, 310, 314, 315, 316, 317, 320, 329, 333, 338, 341, 346, 347, 352, 355, 358, 360, 365, 366, 367, 368, 372, 381, 382, 387, 389, 401, 407, 414, 415, 422, 423, 430, 434, 435, 436, 437, 440, 443, 445, 447, 449, 454, 456, 461, 463, 467, 469, 471, 475, 477, 479, 487, 488, 491, 493, 494, 496, 497, 500, 501, 518, 521, 528, 538, 547, 549, 550, 551, 556, 557, 563, 566, 574, 575, 576, 577, 578, 579, 582, 583, 591, 592, 604, 609, 610, 611, 612, 614, 616, 618, 620, 621, 622, 623, 626, 627, 628, 633, 638, 639, 644, 647, 651, 655, 657, 658, 662, 666, 668, 672, 680, 684, 685, 688, 694, 697, 702, 703, 707, 709, 711, 713, 716, 717, 720, 721, 732, 738, 739, 741, 742, 755, 758, 759, 766, 767, 769, 771, 772, 778, 780, 784, 787, 788, 790, 793, 797, 804, 805, 806, 809, 812, 827, 829, 833, 836, 837, 838, 840, 843, 844, 849, 856, 858, 859, 861, 862, 865, 869, 872, 874, 878, 883, 888, 889, 891, 892, 895, 902, 904, 907, 912, 914, 919, 922, 923, 924, 926, 930, 936, 937, 941, 955, 958, 962, 965, 968, 969, 971, 973, 977, 980, 994, 996, 997, 1000, 1011, 1013, 1016, 1017, 1018, 1022, 1026, 1027, 1030, 1031, 1032, 1033, 1036, 1039, 1041, 1045, 1049, 1050, 1053, 1058, 1060, 1063, 1069, 1073, 1075, 1080, 1082, 1091, 1093, 1095, 1096, 1099, 1100, 1104, 1105, 1112, 1119, 1122, 1125, 1126, 1131, 1144, 1145, 1150, 1151, 1152, 1153, 1158, 1162, 1163, 1165, 1166, 1169, 1170, 1180, 1182, 1185, 1191, 1192, 1194, 1198, 1199, 1200, 1201, 1204, 1207, 1208, 1211, 1213, 1217, 1219, 1220, 1222, 1227, 1229, 1232, 1235, 1237, 1238, 1243, 1245, 1247, 1250, 1256, 1257, 1262, 1266, 1276, 1278, 1281, 1282, 1283, 1284, 1287, 1290, 1292, 1294, 1297, 1307, 1312, 1318, 1320, 1322, 1324, 1325, 1326, 1327, 1328, 1330, 1331, 1334, 1335, 1336, 1337, 1341, 1344, 1346, 1348, 1351, 1353, 1354, 1355, 1357, 1358, 1359, 1362, 1365, 1367, 1370, 1376, 1377, 1379, 1383, 1386, 1390, 1392, 1394, 1396, 1398, 1399, 1400, 1401, 1410, 1411, 1416, 1418, 1423, 1428, 1429, 1437, 1440, 1442, 1444, 1446, 1451, 1454, 1455, 1456, 1461, 1465, 1466, 1468, 1470, 1474, 1475, 1481, 1490, 1493, 1494, 1495, 1498, 1499, 1500, 1505, 1509, 1513, 1517, 1523, 1527, 1528, 1529, 1530, 1533, 1535, 1536, 1539, 1543, 1548, 1549, 1550, 1551, 1560, 1562, 1565, 1568, 1569, 1571, 1573, 1580, 1581, 1583, 1587, 1590, 1592, 1601, 1605, 1609, 1622, 1623, 1624, 1627, 1628, 1629, 1630, 1632, 1633, 1634, 1637, 1639, 1640, 1643, 1649, 1651, 1654, 1655, 1656, 1661, 1662, 1666, 1667, 1669, 1670, 1679, 1688, 1698, 1702, 1706, 1708, 1711, 1712, 1714, 1721, 1722, 1725, 1729, 1731, 1734, 1738, 1739, 1743, 1744, 1745, 1746, 1747, 1748, 1750, 1751, 1752, 1760, 1764, 1765, 1774, 1775, 1783, 1788, 1790, 1792, 1794, 1795, 1797, 1798, 1799, 1800, 1801, 1807, 1808, 1810, 1811, 1821, 1822, 1825, 1829, 1830, 1831, 1834, 1835, 1838, 1840, 1843, 1845, 1853, 1855, 1859, 1861, 1863, 1867, 1868, 1869, 1870, 1872, 1874, 1875, 1876, 1882, 1885, 1886, 1888, 1890, 1892, 1895, 1896, 1897, 1901, 1902, 1903, 1904, 1909, 1910, 1911, 1915, 1918, 1919, 1921, 1922, 1930, 1931, 1934, 1937, 1938, 1941, 1949, 1950, 1952, 1953, 1955, 1957, 1961, 1965, 1969, 1970, 1972, 1973, 1977, 1979, 1982, 1988, 1990, 1993, 1996, 2002, 2004, 2006, 2010, 2013, 2015, 2016, 2019, 2021, 2025, 2026, 2029, 2032, 2034, 2045, 2046, 2050, 2055, 2056, 2059, 2061, 2062, 2066, 2068, 2070, 2073, 2074, 2076, 2079, 2080, 2086, 2087, 2089, 2097, 2098, 2099, 2110, 2111, 2114, 2116, 2118, 2121, 2122, 2125, 2133, 2134, 2136, 2141, 2154, 2157, 2158, 2161, 2163, 2164, 2176, 2178, 2180, 2186, 2190, 2191, 2196, 2199, 2201, 2203, 2207, 2208, 2212, 2219, 2221, 2229, 2231, 2232, 2239, 2240, 2241, 2242, 2243, 2252, 2258, 2265, 2271, 2275, 2276, 2279, 2284, 2286, 2288, 2291, 2292, 2294, 2296, 2310, 2313, 2314, 2317, 2327, 2328, 2330, 2331, 2334, 2336, 2337, 2341, 2343, 2347, 2350, 2354, 2355, 2356, 2358, 2359, 2362, 2365, 2366, 2370, 2372, 2374, 2380, 2388, 2393, 2397, 2405, 2409, 2412, 2414, 2419, 2424, 2425, 2429, 2431, 2434, 2437, 2442, 2444, 2445, 2446, 2447, 2450, 2458, 2459, 2465, 2466, 2468, 2473, 2475, 2476, 2477, 2478, 2481, 2482, 2483, 2484, 2490, 2493, 2496, 2497, 2500, 2501, 2507, 2509, 2515, 2518, 2521, 2527, 2543, 2546, 2550, 2551, 2555, 2559, 2568, 2572, 2576, 2579, 2587, 2589, 2592, 2595, 2597, 2600, 2601, 2604, 2606, 2607, 2609, 2612, 2613, 2615, 2618, 2622, 2630, 2632, 2638, 2639, 2643, 2648, 2649, 2650, 2655, 2656, 2657, 2662, 2665, 2666, 2669, 2670, 2674, 2675, 2677, 2679, 2685, 2691, 2695, 2696, 2697, 2700, 2701, 2702, 2703, 2704, 2706, 2707, 2714, 2715, 2727, 2728, 2731, 2738, 2740, 2741, 2743, 2747, 2748, 2752, 2757, 2766, 2768, 2769, 2775, 2785, 2787, 2788, 2789, 2792, 2796, 2798, 2799, 2802, 2807, 2808, 2811, 2813, 2818, 2819, 2823, 2826, 2827, 2828, 2829, 2831, 2835, 2838, 2845, 2855, 2861, 2863, 2864, 2868, 2869, 2872, 2873, 2886, 2887, 2895, 2896, 2897, 2898, 2903, 2908, 2910, 2911, 2914, 2916, 2918, 2919, 2920, 2925, 2928, 2929, 2931, 2932, 2941, 2945, 2946, 2952, 2956, 2959, 2960, 2962, 2964, 2966, 2967, 2970, 2975, 2976, 2980, 2988, 2990, 2993, 2997, 3003, 3004, 3005, 3006, 3008, 3009, 3010, 3013, 3018, 3028, 3033, 3034, 3035, 3038, 3040, 3047, 3049, 3051, 3058, 3064, 3069, 3072, 3078, 3079, 3080, 3087, 3090, 3094, 3104, 3105, 3110, 3114, 3115, 3120, 3124, 3130, 3131, 3134, 3135, 3136, 3140, 3143, 3145, 3149, 3152, 3153, 3162, 3166, 3169, 3171, 3174, 3178, 3179, 3181, 3183, 3185, 3187, 3188, 3198, 3200, 3206, 3207, 3209, 3212, 3215, 3218, 3222, 3230, 3232, 3235, 3241, 3243, 3245, 3246, 3247, 3250, 3251, 3256, 3258, 3259, 3261, 3262, 3263, 3270, 3275, 3277, 3279, 3281, 3297, 3300, 3303, 3304, 3305, 3310, 3312, 3314, 3315, 3322, 3327, 3329, 3330, 3339, 3344, 3345, 3346, 3347, 3361, 3365, 3371, 3373, 3377, 3378, 3379, 3382, 3383, 3394, 3395, 3397, 3399, 3408, 3412, 3413, 3419, 3420, 3421, 3425, 3431, 3433, 3435, 3436, 3437, 3440, 3441, 3443, 3444, 3445, 3447, 3452, 3458, 3459, 3460, 3465, 3466, 3467, 3470, 3480, 3482, 3484, 3489, 3491, 3493, 3499, 3500, 3502, 3506, 3509, 3510, 3512, 3514, 3516, 3517, 3521, 3525, 3533, 3536, 3538, 3539, 3547, 3548, 3557, 3565, 3567, 3571, 3587, 3590, 3593, 3594, 3604, 3605, 3608, 3609, 3611, 3612, 3613, 3615, 3618, 3619, 3620, 3628, 3630, 3631, 3633, 3635, 3639, 3643, 3646, 3649, 3650, 3657, 3661, 3662, 3664, 3665, 3671, 3672, 3673, 3674, 3675, 3676, 3678, 3683, 3685, 3687, 3689, 3692, 3697, 3701, 3705, 3706, 3709, 3710, 3711, 3718, 3723, 3725, 3726, 3729, 3730, 3737, 3740, 3741, 3755, 3760, 3766, 3768, 3770, 3771, 3774, 3775, 3778, 3781, 3782, 3791, 3800, 3801, 3803, 3804, 3806, 3813, 3822, 3825, 3832, 3833, 3839, 3846, 3852, 3854, 3861, 3864, 3866, 3872, 3876, 3879, 3880, 3881, 3883, 3886, 3887, 3888, 3895, 3897, 3898, 3900, 3902, 3907, 3911, 3913, 3914, 3920, 3921, 3922, 3925, 3928, 3930, 3932, 3936, 3937, 3940, 3941, 3943, 3944, 3947, 3956, 3957, 3963, 3969, 3970, 3971, 3974, 3982, 3983, 3987, 3989, 3991, 3992, 3994, 3995, 3998, 3999, 4000, 4007, 4008, 4009, 4010, 4012, 4014, 4016, 4018, 4020, 4021, 4024, 4025, 4027, 4031, 4032, 4037, 4052, 4055, 4057, 4062, 4077, 4080, 4086, 4089, 4095, 4098, 4099, 4100, 4101, 4105, 4106, 4107, 4108, 4114, 4117, 4120, 4125, 4127, 4128, 4130, 4134, 4135, 4138, 4139, 4146, 4151, 4158, 4160, 4161, 4162, 4168, 4170, 4173, 4174, 4177, 4186, 4191, 4205, 4206, 4208, 4212, 4215, 4216, 4221, 4226, 4227, 4230, 4232, 4233, 4235, 4237, 4240, 4241, 4242, 4245, 4247, 4251, 4257, 4260, 4261, 4264, 4266, 4267, 4269, 4271, 4283, 4284, 4285, 4287, 4288, 4289, 4292, 4295, 4296, 4297, 4298, 4304, 4307, 4308, 4312, 4313, 4316, 4319, 4321, 4323, 4332, 4337, 4339, 4340, 4342, 4344, 4349, 4350, 4353, 4354, 4356, 4361, 4362, 4363, 4371, 4372, 4375, 4378, 4383, 4387, 4389, 4391, 4397, 4402, 4403, 4406, 4407, 4408, 4412, 4414, 4422, 4423, 4425, 4426, 4427, 4432, 4436, 4437, 4439, 4441, 4443, 4445, 4446, 4456, 4460, 4462, 4465, 4466, 4468, 4469, 4470, 4473, 4479, 4480, 4483, 4485, 4486, 4487, 4491, 4493, 4495, 4499, 4502, 4504, 4512, 4513, 4514, 4519, 4524, 4527, 4528, 4532, 4533, 4534, 4537, 4545, 4548, 4552, 4556, 4559, 4560, 4565, 4569, 4577, 4578, 4582, 4596, 4597, 4599, 4600, 4601, 4602, 4604, 4606, 4618, 4622, 4628, 4633, 4634, 4635, 4639, 4640, 4641, 4642, 4652, 4653, 4655, 4656, 4662, 4667, 4669, 4675, 4679, 4680, 4683, 4685, 4690, 4691, 4693, 4703, 4704, 4711, 4721, 4725, 4727, 4729, 4739, 4742, 4743, 4746, 4749, 4751, 4754, 4755, 4758, 4760, 4775, 4777, 4778, 4785, 4786, 4790, 4791, 4794, 4796, 4801, 4810, 4813, 4815, 4822, 4827, 4831, 4837, 4845, 4854, 4855, 4859, 4866, 4868, 4875, 4877, 4878, 4886, 4889, 4890, 4894, 4896, 4897, 4898, 4906, 4907, 4910, 4919, 4920, 4921, 4924, 4926, 4927, 4934, 4937, 4940, 4947, 4948, 4949, 4951, 4956, 4957, 4960, 4961, 4962, 4967, 4972, 4973, 4981, 4989, 4993, 4994, 4998, 5001, 5002, 5004, 5011, 5014, 5016, 5018, 5021, 5023, 5026, 5028, 5030, 5033, 5036, 5037, 5038, 5041, 5044, 5050, 5052, 5053, 5054, 5056, 5057, 5058, 5059, 5061, 5065, 5067, 5075, 5078, 5079, 5080, 5084, 5094, 5098, 5099, 5101, 5104, 5105, 5106, 5108, 5116, 5117, 5118, 5122, 5125, 5129, 5130, 5139, 5142, 5146, 5147, 5148, 5152, 5154, 5156, 5163</t>
+  </si>
+  <si>
+    <t>ASK G6 IF (G5 &lt;&gt; “(98) None of these”)</t>
+  </si>
+  <si>
+    <t>G6.1, G6.2, G6.3, G6.4, G6.5, G6.6, G6.7, G6.8, G6.10, G6.11, G5_12</t>
+  </si>
+  <si>
+    <t>6.459999999999994</t>
+  </si>
+  <si>
+    <t>334</t>
+  </si>
+  <si>
+    <t>19, 21, 39, 47, 66, 75, 76, 96, 97, 117, 123, 135, 138, 152, 187, 194, 198, 216, 227, 248, 255, 281, 288, 297, 312, 338, 356, 413, 417, 421, 424, 434, 464, 478, 479, 486, 502, 528, 546, 561, 573, 593, 599, 639, 652, 655, 668, 671, 705, 709, 712, 714, 717, 729, 757, 774, 781, 789, 806, 807, 811, 816, 829, 864, 892, 903, 946, 948, 966, 1002, 1029, 1035, 1047, 1055, 1060, 1062, 1124, 1131, 1141, 1157, 1173, 1182, 1194, 1199, 1204, 1209, 1216, 1227, 1245, 1263, 1268, 1270, 1287, 1291, 1292, 1311, 1322, 1332, 1341, 1345, 1351, 1355, 1378, 1392, 1399, 1401, 1411, 1421, 1448, 1449, 1452, 1524, 1545, 1559, 1588, 1591, 1626, 1650, 1656, 1673, 1679, 1720, 1788, 1796, 1820, 1827, 1830, 1876, 1882, 1936, 1966, 1967, 1995, 1998, 2012, 2065, 2089, 2115, 2125, 2140, 2141, 2159, 2161, 2165, 2171, 2195, 2229, 2244, 2253, 2256, 2301, 2303, 2308, 2359, 2367, 2378, 2386, 2390, 2392, 2408, 2415, 2416, 2417, 2418, 2422, 2425, 2437, 2440, 2441, 2443, 2447, 2456, 2465, 2481, 2484, 2506, 2520, 2575, 2586, 2627, 2630, 2636, 2659, 2661, 2673, 2681, 2682, 2764, 2795, 2814, 2827, 2883, 2914, 2930, 2934, 2955, 2957, 2965, 3026, 3030, 3045, 3063, 3069, 3091, 3131, 3152, 3153, 3155, 3160, 3170, 3198, 3203, 3206, 3213, 3216, 3225, 3261, 3265, 3285, 3346, 3378, 3383, 3387, 3407, 3411, 3422, 3427, 3429, 3435, 3466, 3470, 3500, 3503, 3505, 3506, 3512, 3515, 3517, 3540, 3556, 3565, 3605, 3619, 3624, 3626, 3656, 3717, 3723, 3731, 3744, 3773, 3794, 3803, 3819, 3826, 3854, 3867, 3870, 3890, 3891, 3947, 3951, 3952, 3954, 3957, 3974, 3994, 4036, 4043, 4061, 4078, 4089, 4103, 4123, 4131, 4155, 4160, 4184, 4189, 4192, 4197, 4218, 4236, 4254, 4255, 4270, 4276, 4310, 4331, 4334, 4337, 4370, 4383, 4392, 4399, 4400, 4413, 4433, 4458, 4470, 4513, 4528, 4571, 4583, 4674, 4680, 4691, 4697, 4708, 4754, 4762, 4777, 4798, 4802, 4806, 4852, 4853, 4885, 4900, 4918, 4935, 4952, 4954, 4963, 4990, 4998, 5013, 5015, 5034, 5078, 5082, 5139, 5143, 5161</t>
   </si>
   <si>
     <t>SK1, SK7</t>
@@ -1243,7 +1258,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="6" width="30.7109375" customWidth="1"/>
@@ -2796,47 +2811,47 @@
         <v>16</v>
       </c>
     </row>
-    <row r="74" spans="2:8" ht="30" customHeight="1">
+    <row r="74" spans="2:8" ht="45" customHeight="1">
       <c r="B74" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>24</v>
+        <v>269</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G74" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H74" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="75" spans="2:8" ht="20" customHeight="1">
+    <row r="75" spans="2:8" ht="30" customHeight="1">
       <c r="B75" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E75" s="4" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="G75" s="4" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="H75" s="4" t="s">
         <v>16</v>
@@ -2847,32 +2862,55 @@
         <v>10</v>
       </c>
       <c r="C76" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="E76" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="F76" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="G76" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="H76" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="77" spans="2:8" ht="20" customHeight="1">
+      <c r="B77" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C77" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D76" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="E76" s="4" t="s">
-        <v>270</v>
-      </c>
-      <c r="F76" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="G76" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="H76" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="78" spans="2:8">
-      <c r="F78" s="5" t="s">
+      <c r="D77" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="E77" s="4" t="s">
         <v>275</v>
+      </c>
+      <c r="F77" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="G77" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="H77" s="4" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="79" spans="2:8">
       <c r="F79" s="5" t="s">
-        <v>276</v>
+        <v>280</v>
+      </c>
+    </row>
+    <row r="80" spans="2:8">
+      <c r="F80" s="5" t="s">
+        <v>281</v>
       </c>
     </row>
   </sheetData>

</xml_diff>